<commit_message>
ANW-2050 PR2 Add header guard, lang/user_defined/collection_management subrecords (#4205)
* ANW-2050 PR2 Add header guard, lang/user_defined/collection_management subrecords

* ANW-2050 Address PR2 bulk import review feedback

* to be squashed: add a spec showing that an error raised outside of the db transaction can fail the job but write records

* to be squashed: fix for terminal errors rolling back the db transaction

* ANW-2050 Internationalize User Defined numeric errors

* ANW-2050 PR2 Fix Rubocop errors on extra spec commit

---------

Co-authored-by: Thimios <thimios.dimopulos@lyrasis.org>
</commit_message>
<xml_diff>
--- a/frontend/public/bulk_import_templates/bulk_import_DO_template.xlsx
+++ b/frontend/public/bulk_import_templates/bulk_import_DO_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lyrasis-my.sharepoint.com/personal/zmorgan_lyrasis_org/Documents/Desktop/ANW-2050/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zeffmorgan/src/lyrasis/archivesspace/frontend/public/bulk_import_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="11_9E13F37379FC7C110D611ECD94F66E7260655893" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC8C42CC-FFD9-E84C-84B4-EF1D86D10C42}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F0FAF1-A5CC-B04E-9E6A-64EFA72571BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34560" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="376">
   <si>
     <t>This is the template for use with the bulk_import ("Load SpreadSheet") for importing digital ob jects to associate with archival objects .  You may replace this line with something of your choosing after you've copied the file for your use.</t>
   </si>
@@ -108,36 +108,6 @@
     <t>Digital Object Restrictions (FALSE/TRUE)</t>
   </si>
   <si>
-    <t>Linked-to URL for representative file version</t>
-  </si>
-  <si>
-    <t>Use Statement for representative file version</t>
-  </si>
-  <si>
-    <t>Xlink actuate attribute for representative file version (previous default 'onRequest')</t>
-  </si>
-  <si>
-    <t>Xlink show attribute for representative file version (previous default 'new')</t>
-  </si>
-  <si>
-    <t>File Format Name for representative file version</t>
-  </si>
-  <si>
-    <t>File Format Version for representative file version</t>
-  </si>
-  <si>
-    <t>File size (bytes) for representative file version</t>
-  </si>
-  <si>
-    <t>Checksum for representative file version</t>
-  </si>
-  <si>
-    <t>Checksum Method for representative file version</t>
-  </si>
-  <si>
-    <t>Caption for representative file version</t>
-  </si>
-  <si>
     <t>Dates label (default: Creation)</t>
   </si>
   <si>
@@ -474,30 +444,6 @@
     <t>corporate_entities_agent_relator_3</t>
   </si>
   <si>
-    <t>subject_1_record_id</t>
-  </si>
-  <si>
-    <t>subject_1_term</t>
-  </si>
-  <si>
-    <t>subject_1_type</t>
-  </si>
-  <si>
-    <t>subject_1_source</t>
-  </si>
-  <si>
-    <t>subject_2_record_id</t>
-  </si>
-  <si>
-    <t>subject_2_term</t>
-  </si>
-  <si>
-    <t>subject_2_type</t>
-  </si>
-  <si>
-    <t>subject_2_source</t>
-  </si>
-  <si>
     <t>note_type</t>
   </si>
   <si>
@@ -744,30 +690,6 @@
     <t>CorporateRelator(3)</t>
   </si>
   <si>
-    <t>Subject (1) Record ID</t>
-  </si>
-  <si>
-    <t>Subject (1) Term</t>
-  </si>
-  <si>
-    <t>Subject (1) Type</t>
-  </si>
-  <si>
-    <t>Subject (1) Source</t>
-  </si>
-  <si>
-    <t>Subject (2) Record ID</t>
-  </si>
-  <si>
-    <t>Subject (2) Term</t>
-  </si>
-  <si>
-    <t>Subject (2) Type</t>
-  </si>
-  <si>
-    <t>Subject (2) Source</t>
-  </si>
-  <si>
     <t>Note Type</t>
   </si>
   <si>
@@ -868,6 +790,391 @@
   </si>
   <si>
     <t>Is Representative(1)</t>
+  </si>
+  <si>
+    <t>subject_record_id_1</t>
+  </si>
+  <si>
+    <t>Subject Record ID(1)</t>
+  </si>
+  <si>
+    <t>subject_term_1</t>
+  </si>
+  <si>
+    <t>Subject Term(1)</t>
+  </si>
+  <si>
+    <t>Subject Source(2)</t>
+  </si>
+  <si>
+    <t>Subject Type(2)</t>
+  </si>
+  <si>
+    <t>Subject Term(2)</t>
+  </si>
+  <si>
+    <t>Subject Record ID(2)</t>
+  </si>
+  <si>
+    <t>Subject Source(1)</t>
+  </si>
+  <si>
+    <t>Subject Type(1)</t>
+  </si>
+  <si>
+    <t>subject_type_1</t>
+  </si>
+  <si>
+    <t>subject_source_1</t>
+  </si>
+  <si>
+    <t>subject_record_id_2</t>
+  </si>
+  <si>
+    <t>subject_term_2</t>
+  </si>
+  <si>
+    <t>subject_type_2</t>
+  </si>
+  <si>
+    <t>subject_source_2</t>
+  </si>
+  <si>
+    <t>Language Materials</t>
+  </si>
+  <si>
+    <t>User Defined</t>
+  </si>
+  <si>
+    <t>Processing</t>
+  </si>
+  <si>
+    <t>Language of the material (ISO 639-2, e.g. eng)</t>
+  </si>
+  <si>
+    <t>Script of the material (ISO 15924, e.g. Latn)</t>
+  </si>
+  <si>
+    <t>Processing priority (controlled value: high/medium/low)</t>
+  </si>
+  <si>
+    <t>Rights determined? (true/false)</t>
+  </si>
+  <si>
+    <t>Free-text processing plan</t>
+  </si>
+  <si>
+    <t>Staff assigned to processing</t>
+  </si>
+  <si>
+    <t>Processing hours per unit estimate</t>
+  </si>
+  <si>
+    <t>Total extent processed; REQUIRES Extent Type</t>
+  </si>
+  <si>
+    <t>Extent type (controlled value); REQUIRED with Total Extent</t>
+  </si>
+  <si>
+    <t>Total processing hours</t>
+  </si>
+  <si>
+    <t>Source of processing funding (free text)</t>
+  </si>
+  <si>
+    <t>Processing status (controlled value: new/in_progress/completed)</t>
+  </si>
+  <si>
+    <t>user_defined_boolean_1</t>
+  </si>
+  <si>
+    <t>user_defined_boolean_2</t>
+  </si>
+  <si>
+    <t>user_defined_boolean_3</t>
+  </si>
+  <si>
+    <t>user_defined_date_1</t>
+  </si>
+  <si>
+    <t>user_defined_date_2</t>
+  </si>
+  <si>
+    <t>user_defined_date_3</t>
+  </si>
+  <si>
+    <t>user_defined_integer_1</t>
+  </si>
+  <si>
+    <t>user_defined_integer_2</t>
+  </si>
+  <si>
+    <t>user_defined_integer_3</t>
+  </si>
+  <si>
+    <t>user_defined_real_1</t>
+  </si>
+  <si>
+    <t>user_defined_real_2</t>
+  </si>
+  <si>
+    <t>user_defined_real_3</t>
+  </si>
+  <si>
+    <t>user_defined_string_1</t>
+  </si>
+  <si>
+    <t>user_defined_string_2</t>
+  </si>
+  <si>
+    <t>user_defined_string_3</t>
+  </si>
+  <si>
+    <t>user_defined_string_4</t>
+  </si>
+  <si>
+    <t>user_defined_text_1</t>
+  </si>
+  <si>
+    <t>user_defined_text_2</t>
+  </si>
+  <si>
+    <t>user_defined_text_3</t>
+  </si>
+  <si>
+    <t>user_defined_text_4</t>
+  </si>
+  <si>
+    <t>user_defined_text_5</t>
+  </si>
+  <si>
+    <t>user_defined_enum_1</t>
+  </si>
+  <si>
+    <t>user_defined_enum_2</t>
+  </si>
+  <si>
+    <t>user_defined_enum_3</t>
+  </si>
+  <si>
+    <t>user_defined_enum_4</t>
+  </si>
+  <si>
+    <t>User Defined Boolean 1</t>
+  </si>
+  <si>
+    <t>User Defined Boolean 2</t>
+  </si>
+  <si>
+    <t>User Defined Boolean 3</t>
+  </si>
+  <si>
+    <t>User Defined Date 1</t>
+  </si>
+  <si>
+    <t>User Defined Date 2</t>
+  </si>
+  <si>
+    <t>User Defined Date 3</t>
+  </si>
+  <si>
+    <t>User Defined Integer 1</t>
+  </si>
+  <si>
+    <t>User Defined Integer 2</t>
+  </si>
+  <si>
+    <t>User Defined Integer 3</t>
+  </si>
+  <si>
+    <t>User Defined Real 1</t>
+  </si>
+  <si>
+    <t>User Defined Real 2</t>
+  </si>
+  <si>
+    <t>User Defined Real 3</t>
+  </si>
+  <si>
+    <t>User Defined String 1</t>
+  </si>
+  <si>
+    <t>User Defined String 2</t>
+  </si>
+  <si>
+    <t>User Defined String 3</t>
+  </si>
+  <si>
+    <t>User Defined String 4</t>
+  </si>
+  <si>
+    <t>User Defined Text 1</t>
+  </si>
+  <si>
+    <t>User Defined Text 2</t>
+  </si>
+  <si>
+    <t>User Defined Text 3</t>
+  </si>
+  <si>
+    <t>User Defined Text 4</t>
+  </si>
+  <si>
+    <t>User Defined Text 5</t>
+  </si>
+  <si>
+    <t>User Defined Enum 1</t>
+  </si>
+  <si>
+    <t>User Defined Enum 2</t>
+  </si>
+  <si>
+    <t>User Defined Enum 3</t>
+  </si>
+  <si>
+    <t>User Defined Enum 4</t>
+  </si>
+  <si>
+    <t>Processing Priority</t>
+  </si>
+  <si>
+    <t>Rights Determined?</t>
+  </si>
+  <si>
+    <t>Processing Plan</t>
+  </si>
+  <si>
+    <t>Processors</t>
+  </si>
+  <si>
+    <t>Processing hrs/unit Estimate</t>
+  </si>
+  <si>
+    <t>Processing Total Extent</t>
+  </si>
+  <si>
+    <t>Processing Total Extent Type</t>
+  </si>
+  <si>
+    <t>Total Processing Hours</t>
+  </si>
+  <si>
+    <t>Funding Source</t>
+  </si>
+  <si>
+    <t>Processing Status</t>
+  </si>
+  <si>
+    <t>lang_material_language_1</t>
+  </si>
+  <si>
+    <t>lang_material_script_1</t>
+  </si>
+  <si>
+    <t>Language Materials Language(1)</t>
+  </si>
+  <si>
+    <t>Language Materials Script(1)</t>
+  </si>
+  <si>
+    <t>Local-use boolean (true/false)
+Non-repeatable</t>
+  </si>
+  <si>
+    <t>Local-use date (YYYY-MM-DD)
+Non-repeatable</t>
+  </si>
+  <si>
+    <t>Local-use integer (stored as string)
+Non-repeatable</t>
+  </si>
+  <si>
+    <t>Local-use decimal (2 places, max 13 chars)
+Non-repeatable</t>
+  </si>
+  <si>
+    <t>Local-use short text (max 255)
+Non-repeatable</t>
+  </si>
+  <si>
+    <t>Local-use long text (max 65000)
+Non-repeatable</t>
+  </si>
+  <si>
+    <t>Local-use controlled value list 1
+Non-repeatable</t>
+  </si>
+  <si>
+    <t>Local-use controlled value list 2
+Non-repeatable</t>
+  </si>
+  <si>
+    <t>Local-use controlled value list 3
+Non-repeatable</t>
+  </si>
+  <si>
+    <t>Local-use controlled value list 4
+Non-repeatable</t>
+  </si>
+  <si>
+    <t>collection_management_processing_priority</t>
+  </si>
+  <si>
+    <t>collection_management_processing_plan</t>
+  </si>
+  <si>
+    <t>collection_management_processing_total_extent</t>
+  </si>
+  <si>
+    <t>collection_management_processing_total_extent_type</t>
+  </si>
+  <si>
+    <t>collection_management_processing_funding_source</t>
+  </si>
+  <si>
+    <t>collection_management_processing_status</t>
+  </si>
+  <si>
+    <t>collection_management_processors</t>
+  </si>
+  <si>
+    <t>collection_management_processing_hours_per_foot_estimate</t>
+  </si>
+  <si>
+    <t>collection_management_processing_hours_total</t>
+  </si>
+  <si>
+    <t>collection_management_rights_determined</t>
+  </si>
+  <si>
+    <t>Linked-to URL</t>
+  </si>
+  <si>
+    <t>Use Statement</t>
+  </si>
+  <si>
+    <t>Xlink actuate attribute (previous default 'onRequest')</t>
+  </si>
+  <si>
+    <t>Xlink show attribute (previous default 'new')</t>
+  </si>
+  <si>
+    <t>File Format Name</t>
+  </si>
+  <si>
+    <t>File Format Version</t>
+  </si>
+  <si>
+    <t>File size (bytes)</t>
+  </si>
+  <si>
+    <t>Checksum</t>
+  </si>
+  <si>
+    <t>Checksum Method</t>
+  </si>
+  <si>
+    <t>Caption</t>
   </si>
 </sst>
 </file>
@@ -941,7 +1248,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -994,6 +1301,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFACCCF3"/>
         <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+        <bgColor rgb="FFE6E0EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8DDF2"/>
+        <bgColor rgb="FFE6E0EC"/>
       </patternFill>
     </fill>
   </fills>
@@ -1079,7 +1398,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1195,6 +1514,20 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1269,6 +1602,9 @@
       <rgbColor rgb="00333333"/>
     </indexedColors>
     <mruColors>
+      <color rgb="FFE8DDF2"/>
+      <color rgb="FFD9EAF7"/>
+      <color rgb="FFC5FFFF"/>
       <color rgb="FFACCCF3"/>
     </mruColors>
   </colors>
@@ -1610,7 +1946,7 @@
     <col min="5" max="6" width="10.6640625" style="2" customWidth="1"/>
     <col min="7" max="7" width="29.33203125" style="2" customWidth="1"/>
     <col min="8" max="8" width="25.1640625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="20.6640625" customWidth="1"/>
+    <col min="9" max="9" width="22.6640625" customWidth="1"/>
     <col min="10" max="11" width="17.33203125" customWidth="1"/>
     <col min="12" max="12" width="20.6640625" customWidth="1"/>
     <col min="13" max="14" width="17.33203125" style="2" customWidth="1"/>
@@ -1664,25 +2000,34 @@
     <col min="84" max="86" width="13.5" style="2" customWidth="1"/>
     <col min="87" max="88" width="10.83203125" style="2" customWidth="1"/>
     <col min="89" max="89" width="15.5" style="2" customWidth="1"/>
-    <col min="90" max="90" width="9.33203125" style="2"/>
+    <col min="90" max="90" width="16.83203125" style="2" customWidth="1"/>
     <col min="91" max="91" width="17.6640625" style="2" customWidth="1"/>
     <col min="92" max="92" width="17.6640625" customWidth="1"/>
     <col min="93" max="93" width="17" style="2" customWidth="1"/>
     <col min="94" max="94" width="17.6640625" style="2" customWidth="1"/>
     <col min="95" max="95" width="17.6640625" customWidth="1"/>
     <col min="96" max="104" width="17.6640625" style="2" customWidth="1"/>
-    <col min="105" max="994" width="9.33203125" style="2"/>
+    <col min="105" max="106" width="16.83203125" style="2" customWidth="1"/>
+    <col min="107" max="107" width="23.33203125" style="2" customWidth="1"/>
+    <col min="108" max="131" width="12.83203125" style="2" customWidth="1"/>
+    <col min="132" max="132" width="15.33203125" style="2" customWidth="1"/>
+    <col min="133" max="133" width="16.6640625" style="2" customWidth="1"/>
+    <col min="134" max="135" width="13.5" style="2" customWidth="1"/>
+    <col min="136" max="136" width="17.33203125" style="2" customWidth="1"/>
+    <col min="137" max="140" width="16" style="2" customWidth="1"/>
+    <col min="141" max="141" width="13.5" style="2" customWidth="1"/>
+    <col min="142" max="994" width="9.33203125" style="2"/>
     <col min="995" max="1015" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:104" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:141" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="CN1" s="2"/>
       <c r="CQ1" s="2"/>
     </row>
-    <row r="2" spans="1:104" s="2" customFormat="1" ht="41.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:141" s="2" customFormat="1" ht="41.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1995,8 +2340,119 @@
       <c r="CZ2" s="12" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:104" ht="132" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="DA2" s="39" t="s">
+        <v>267</v>
+      </c>
+      <c r="DB2" s="39" t="s">
+        <v>267</v>
+      </c>
+      <c r="DC2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DD2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DE2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DF2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DG2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DH2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DI2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DJ2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DK2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DL2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DM2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DN2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DO2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DP2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DQ2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DR2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DS2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DT2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DU2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DV2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DW2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DX2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DY2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="DZ2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="EA2" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="EB2" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="EC2" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="ED2" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="EE2" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="EF2" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="EG2" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="EH2" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="EI2" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="EJ2" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="EK2" s="12" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="3" spans="1:141" ht="132" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>13</v>
       </c>
@@ -2034,911 +2490,1244 @@
         <v>24</v>
       </c>
       <c r="M3" s="38" t="s">
+        <v>366</v>
+      </c>
+      <c r="N3" s="38" t="s">
+        <v>227</v>
+      </c>
+      <c r="O3" s="38" t="s">
+        <v>367</v>
+      </c>
+      <c r="P3" s="38" t="s">
+        <v>368</v>
+      </c>
+      <c r="Q3" s="38" t="s">
+        <v>369</v>
+      </c>
+      <c r="R3" s="38" t="s">
+        <v>370</v>
+      </c>
+      <c r="S3" s="38" t="s">
+        <v>371</v>
+      </c>
+      <c r="T3" s="38" t="s">
+        <v>372</v>
+      </c>
+      <c r="U3" s="38" t="s">
+        <v>373</v>
+      </c>
+      <c r="V3" s="38" t="s">
+        <v>374</v>
+      </c>
+      <c r="W3" s="38" t="s">
+        <v>249</v>
+      </c>
+      <c r="X3" s="38" t="s">
+        <v>375</v>
+      </c>
+      <c r="Y3" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="N3" s="38" t="s">
+      <c r="Z3" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA3" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB3" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="AC3" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD3" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="AE3" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="AF3" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="AG3" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="AH3" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="AI3" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="AJ3" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="AK3" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="AL3" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="AM3" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="AN3" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="AO3" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="AP3" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="AQ3" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="AR3" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="AS3" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="AT3" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="AU3" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="AV3" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="AW3" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="AX3" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AY3" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="AZ3" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="BA3" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="BB3" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="BC3" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="BD3" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="BE3" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="BF3" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="BG3" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="BH3" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="BI3" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="BJ3" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="BK3" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="BL3" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="BM3" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="BN3" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="BO3" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="BP3" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="BQ3" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="BR3" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="BS3" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="BT3" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="BU3" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="BV3" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="BW3" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="BX3" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="BY3" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="BZ3" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="CA3" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="CB3" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="CC3" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="CD3" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="CE3" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="CF3" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="CG3" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="CH3" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="CI3" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="CJ3" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="CK3" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="CL3" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="CM3" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="CN3" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="CO3" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="CP3" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="CQ3" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="CR3" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="CS3" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="CT3" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="CU3" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="CV3" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="CW3" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="CX3" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="CY3" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="CZ3" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="DA3" s="40" t="s">
+        <v>270</v>
+      </c>
+      <c r="DB3" s="40" t="s">
+        <v>271</v>
+      </c>
+      <c r="DC3" s="42" t="s">
+        <v>346</v>
+      </c>
+      <c r="DD3" s="42" t="s">
+        <v>346</v>
+      </c>
+      <c r="DE3" s="42" t="s">
+        <v>346</v>
+      </c>
+      <c r="DF3" s="42" t="s">
+        <v>347</v>
+      </c>
+      <c r="DG3" s="42" t="s">
+        <v>347</v>
+      </c>
+      <c r="DH3" s="42" t="s">
+        <v>347</v>
+      </c>
+      <c r="DI3" s="42" t="s">
+        <v>348</v>
+      </c>
+      <c r="DJ3" s="42" t="s">
+        <v>348</v>
+      </c>
+      <c r="DK3" s="42" t="s">
+        <v>348</v>
+      </c>
+      <c r="DL3" s="42" t="s">
+        <v>349</v>
+      </c>
+      <c r="DM3" s="42" t="s">
+        <v>349</v>
+      </c>
+      <c r="DN3" s="42" t="s">
+        <v>349</v>
+      </c>
+      <c r="DO3" s="42" t="s">
+        <v>350</v>
+      </c>
+      <c r="DP3" s="42" t="s">
+        <v>350</v>
+      </c>
+      <c r="DQ3" s="42" t="s">
+        <v>350</v>
+      </c>
+      <c r="DR3" s="42" t="s">
+        <v>350</v>
+      </c>
+      <c r="DS3" s="42" t="s">
+        <v>351</v>
+      </c>
+      <c r="DT3" s="42" t="s">
+        <v>351</v>
+      </c>
+      <c r="DU3" s="42" t="s">
+        <v>351</v>
+      </c>
+      <c r="DV3" s="42" t="s">
+        <v>351</v>
+      </c>
+      <c r="DW3" s="42" t="s">
+        <v>351</v>
+      </c>
+      <c r="DX3" s="42" t="s">
+        <v>352</v>
+      </c>
+      <c r="DY3" s="42" t="s">
+        <v>353</v>
+      </c>
+      <c r="DZ3" s="42" t="s">
+        <v>354</v>
+      </c>
+      <c r="EA3" s="42" t="s">
+        <v>355</v>
+      </c>
+      <c r="EB3" s="25" t="s">
+        <v>272</v>
+      </c>
+      <c r="EC3" s="25" t="s">
+        <v>273</v>
+      </c>
+      <c r="ED3" s="25" t="s">
+        <v>274</v>
+      </c>
+      <c r="EE3" s="25" t="s">
+        <v>275</v>
+      </c>
+      <c r="EF3" s="25" t="s">
+        <v>276</v>
+      </c>
+      <c r="EG3" s="25" t="s">
+        <v>277</v>
+      </c>
+      <c r="EH3" s="25" t="s">
+        <v>278</v>
+      </c>
+      <c r="EI3" s="25" t="s">
+        <v>279</v>
+      </c>
+      <c r="EJ3" s="25" t="s">
+        <v>280</v>
+      </c>
+      <c r="EK3" s="25" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="4" spans="1:141" s="27" customFormat="1" ht="41.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="I4" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="J4" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="K4" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="L4" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="M4" s="27" t="s">
+        <v>225</v>
+      </c>
+      <c r="N4" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="O4" s="27" t="s">
+        <v>230</v>
+      </c>
+      <c r="P4" s="27" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q4" s="27" t="s">
+        <v>234</v>
+      </c>
+      <c r="R4" s="27" t="s">
+        <v>236</v>
+      </c>
+      <c r="S4" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="T4" s="27" t="s">
+        <v>240</v>
+      </c>
+      <c r="U4" s="27" t="s">
+        <v>242</v>
+      </c>
+      <c r="V4" s="27" t="s">
+        <v>244</v>
+      </c>
+      <c r="W4" s="27" t="s">
+        <v>246</v>
+      </c>
+      <c r="X4" s="27" t="s">
+        <v>247</v>
+      </c>
+      <c r="Y4" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z4" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="AA4" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="AB4" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="AC4" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="AD4" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE4" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="AF4" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG4" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="AH4" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="AI4" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="AJ4" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="AK4" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="AL4" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="AM4" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="AN4" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="AO4" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="AP4" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="AQ4" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="AR4" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="AS4" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="AT4" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="AU4" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="AV4" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="AW4" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="AX4" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="AY4" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="AZ4" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="BA4" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="BB4" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="BC4" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="BD4" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="BE4" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="BF4" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="BG4" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="BH4" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="BI4" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="BJ4" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="BK4" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="BL4" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="BM4" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="BN4" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="BO4" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="BP4" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="BQ4" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="BR4" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="BS4" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="BT4" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="BU4" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="BV4" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="BW4" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="BX4" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="BY4" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="BZ4" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="CA4" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="CB4" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="CC4" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="CD4" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CE4" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="CF4" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="CG4" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="CH4" s="27" t="s">
+        <v>132</v>
+      </c>
+      <c r="CI4" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="CJ4" s="27" t="s">
+        <v>134</v>
+      </c>
+      <c r="CK4" s="27" t="s">
+        <v>251</v>
+      </c>
+      <c r="CL4" s="27" t="s">
         <v>253</v>
       </c>
-      <c r="O3" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="P3" s="38" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q3" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="R3" s="38" t="s">
-        <v>29</v>
-      </c>
-      <c r="S3" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="T3" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="U3" s="38" t="s">
+      <c r="CM4" s="27" t="s">
+        <v>261</v>
+      </c>
+      <c r="CN4" s="27" t="s">
+        <v>262</v>
+      </c>
+      <c r="CO4" s="27" t="s">
+        <v>263</v>
+      </c>
+      <c r="CP4" s="27" t="s">
+        <v>264</v>
+      </c>
+      <c r="CQ4" s="27" t="s">
+        <v>265</v>
+      </c>
+      <c r="CR4" s="27" t="s">
+        <v>266</v>
+      </c>
+      <c r="CS4" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="CT4" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="CU4" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="CV4" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="CW4" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="CX4" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="CY4" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="CZ4" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="DA4" s="27" t="s">
+        <v>342</v>
+      </c>
+      <c r="DB4" s="27" t="s">
+        <v>343</v>
+      </c>
+      <c r="DC4" s="27" t="s">
+        <v>282</v>
+      </c>
+      <c r="DD4" s="27" t="s">
+        <v>283</v>
+      </c>
+      <c r="DE4" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="DF4" s="27" t="s">
+        <v>285</v>
+      </c>
+      <c r="DG4" s="27" t="s">
+        <v>286</v>
+      </c>
+      <c r="DH4" s="27" t="s">
+        <v>287</v>
+      </c>
+      <c r="DI4" s="27" t="s">
+        <v>288</v>
+      </c>
+      <c r="DJ4" s="27" t="s">
+        <v>289</v>
+      </c>
+      <c r="DK4" s="27" t="s">
+        <v>290</v>
+      </c>
+      <c r="DL4" s="27" t="s">
+        <v>291</v>
+      </c>
+      <c r="DM4" s="27" t="s">
+        <v>292</v>
+      </c>
+      <c r="DN4" s="27" t="s">
+        <v>293</v>
+      </c>
+      <c r="DO4" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="DP4" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="DQ4" s="27" t="s">
+        <v>296</v>
+      </c>
+      <c r="DR4" s="27" t="s">
+        <v>297</v>
+      </c>
+      <c r="DS4" s="27" t="s">
+        <v>298</v>
+      </c>
+      <c r="DT4" s="27" t="s">
+        <v>299</v>
+      </c>
+      <c r="DU4" s="27" t="s">
+        <v>300</v>
+      </c>
+      <c r="DV4" s="27" t="s">
+        <v>301</v>
+      </c>
+      <c r="DW4" s="27" t="s">
+        <v>302</v>
+      </c>
+      <c r="DX4" s="27" t="s">
+        <v>303</v>
+      </c>
+      <c r="DY4" s="27" t="s">
+        <v>304</v>
+      </c>
+      <c r="DZ4" s="27" t="s">
+        <v>305</v>
+      </c>
+      <c r="EA4" s="27" t="s">
+        <v>306</v>
+      </c>
+      <c r="EB4" s="27" t="s">
+        <v>356</v>
+      </c>
+      <c r="EC4" s="27" t="s">
+        <v>365</v>
+      </c>
+      <c r="ED4" s="27" t="s">
+        <v>357</v>
+      </c>
+      <c r="EE4" s="27" t="s">
+        <v>362</v>
+      </c>
+      <c r="EF4" s="27" t="s">
+        <v>363</v>
+      </c>
+      <c r="EG4" s="27" t="s">
+        <v>358</v>
+      </c>
+      <c r="EH4" s="27" t="s">
+        <v>359</v>
+      </c>
+      <c r="EI4" s="27" t="s">
+        <v>364</v>
+      </c>
+      <c r="EJ4" s="27" t="s">
+        <v>360</v>
+      </c>
+      <c r="EK4" s="27" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="5" spans="1:141" ht="31" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="31" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>144</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>145</v>
+      </c>
+      <c r="D5" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>149</v>
+      </c>
+      <c r="H5" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="I5" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="J5" s="33" t="s">
+        <v>152</v>
+      </c>
+      <c r="K5" s="33" t="s">
+        <v>153</v>
+      </c>
+      <c r="L5" s="33" t="s">
+        <v>154</v>
+      </c>
+      <c r="M5" s="33" t="s">
+        <v>229</v>
+      </c>
+      <c r="N5" s="33" t="s">
+        <v>228</v>
+      </c>
+      <c r="O5" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="P5" s="33" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q5" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="R5" s="33" t="s">
+        <v>237</v>
+      </c>
+      <c r="S5" s="33" t="s">
+        <v>239</v>
+      </c>
+      <c r="T5" s="33" t="s">
+        <v>241</v>
+      </c>
+      <c r="U5" s="33" t="s">
+        <v>243</v>
+      </c>
+      <c r="V5" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="W5" s="33" t="s">
+        <v>250</v>
+      </c>
+      <c r="X5" s="33" t="s">
+        <v>248</v>
+      </c>
+      <c r="Y5" s="33" t="s">
+        <v>155</v>
+      </c>
+      <c r="Z5" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="AA5" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="AB5" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="AC5" s="34" t="s">
+        <v>159</v>
+      </c>
+      <c r="AD5" s="33" t="s">
+        <v>160</v>
+      </c>
+      <c r="AE5" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="AF5" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="AG5" s="34" t="s">
+        <v>163</v>
+      </c>
+      <c r="AH5" s="32" t="s">
+        <v>164</v>
+      </c>
+      <c r="AI5" s="34" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ5" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK5" s="33" t="s">
+        <v>167</v>
+      </c>
+      <c r="AL5" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="V3" s="38" t="s">
-        <v>33</v>
-      </c>
-      <c r="W3" s="38" t="s">
-        <v>275</v>
-      </c>
-      <c r="X3" s="38" t="s">
+      <c r="AM5" s="32" t="s">
+        <v>168</v>
+      </c>
+      <c r="AN5" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="Y3" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z3" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="AA3" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="AB3" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="AC3" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD3" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="AE3" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="AF3" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="AG3" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="AH3" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="AI3" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="AJ3" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="AK3" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="AL3" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="AM3" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN3" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="AO3" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="AP3" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="AQ3" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="AR3" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="AS3" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="AT3" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="AU3" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="AV3" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="AW3" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="AX3" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="AY3" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="AZ3" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="BA3" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="BB3" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="BC3" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="BD3" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="BE3" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="BF3" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="BG3" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="BH3" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="BI3" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="BJ3" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="BK3" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="BL3" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="BM3" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="BN3" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="BO3" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="BP3" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="BQ3" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="BR3" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="BS3" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="BT3" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="BU3" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="BV3" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="BW3" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="BX3" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="BY3" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="BZ3" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="CA3" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="CB3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="CC3" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="CD3" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="CE3" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="CF3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="CG3" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="CH3" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="CI3" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="CJ3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="CK3" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="CL3" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="CM3" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="CN3" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="CO3" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="CP3" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="CQ3" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="CR3" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="CS3" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="CT3" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="CU3" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="CV3" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="CW3" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="CX3" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="CY3" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="CZ3" s="25" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="4" spans="1:104" s="27" customFormat="1" ht="41.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" s="27" t="s">
-        <v>70</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="D4" s="27" t="s">
-        <v>72</v>
-      </c>
-      <c r="E4" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="F4" s="27" t="s">
-        <v>74</v>
-      </c>
-      <c r="G4" s="27" t="s">
-        <v>75</v>
-      </c>
-      <c r="H4" s="27" t="s">
-        <v>76</v>
-      </c>
-      <c r="I4" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="J4" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="K4" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="L4" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="M4" s="27" t="s">
-        <v>251</v>
-      </c>
-      <c r="N4" s="27" t="s">
+      <c r="AO5" s="33" t="s">
+        <v>169</v>
+      </c>
+      <c r="AP5" s="33" t="s">
+        <v>170</v>
+      </c>
+      <c r="AQ5" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="AR5" s="32" t="s">
+        <v>172</v>
+      </c>
+      <c r="AS5" s="32" t="s">
+        <v>173</v>
+      </c>
+      <c r="AT5" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="AU5" s="33" t="s">
+        <v>175</v>
+      </c>
+      <c r="AV5" s="33" t="s">
+        <v>176</v>
+      </c>
+      <c r="AW5" s="33" t="s">
+        <v>177</v>
+      </c>
+      <c r="AX5" s="33" t="s">
+        <v>178</v>
+      </c>
+      <c r="AY5" s="33" t="s">
+        <v>179</v>
+      </c>
+      <c r="AZ5" s="33" t="s">
+        <v>180</v>
+      </c>
+      <c r="BA5" s="33" t="s">
+        <v>181</v>
+      </c>
+      <c r="BB5" s="33" t="s">
+        <v>182</v>
+      </c>
+      <c r="BC5" s="33" t="s">
+        <v>183</v>
+      </c>
+      <c r="BD5" s="33" t="s">
+        <v>184</v>
+      </c>
+      <c r="BE5" s="33" t="s">
+        <v>185</v>
+      </c>
+      <c r="BF5" s="33" t="s">
+        <v>186</v>
+      </c>
+      <c r="BG5" s="33" t="s">
+        <v>187</v>
+      </c>
+      <c r="BH5" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="BI5" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="BJ5" s="33" t="s">
+        <v>190</v>
+      </c>
+      <c r="BK5" s="33" t="s">
+        <v>191</v>
+      </c>
+      <c r="BL5" s="33" t="s">
+        <v>192</v>
+      </c>
+      <c r="BM5" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="BN5" s="33" t="s">
+        <v>194</v>
+      </c>
+      <c r="BO5" s="33" t="s">
+        <v>195</v>
+      </c>
+      <c r="BP5" s="33" t="s">
+        <v>196</v>
+      </c>
+      <c r="BQ5" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="BR5" s="33" t="s">
+        <v>198</v>
+      </c>
+      <c r="BS5" s="33" t="s">
+        <v>199</v>
+      </c>
+      <c r="BT5" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="BU5" s="33" t="s">
+        <v>201</v>
+      </c>
+      <c r="BV5" s="33" t="s">
+        <v>202</v>
+      </c>
+      <c r="BW5" s="33" t="s">
+        <v>203</v>
+      </c>
+      <c r="BX5" s="33" t="s">
+        <v>204</v>
+      </c>
+      <c r="BY5" s="33" t="s">
+        <v>205</v>
+      </c>
+      <c r="BZ5" s="33" t="s">
+        <v>206</v>
+      </c>
+      <c r="CA5" s="33" t="s">
+        <v>207</v>
+      </c>
+      <c r="CB5" s="33" t="s">
+        <v>208</v>
+      </c>
+      <c r="CC5" s="33" t="s">
+        <v>209</v>
+      </c>
+      <c r="CD5" s="33" t="s">
+        <v>210</v>
+      </c>
+      <c r="CE5" s="33" t="s">
+        <v>211</v>
+      </c>
+      <c r="CF5" s="33" t="s">
+        <v>212</v>
+      </c>
+      <c r="CG5" s="33" t="s">
+        <v>213</v>
+      </c>
+      <c r="CH5" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="CI5" s="33" t="s">
+        <v>215</v>
+      </c>
+      <c r="CJ5" s="33" t="s">
+        <v>216</v>
+      </c>
+      <c r="CK5" s="33" t="s">
         <v>252</v>
       </c>
-      <c r="O4" s="27" t="s">
+      <c r="CL5" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="CM5" s="33" t="s">
+        <v>260</v>
+      </c>
+      <c r="CN5" s="33" t="s">
+        <v>259</v>
+      </c>
+      <c r="CO5" s="33" t="s">
+        <v>258</v>
+      </c>
+      <c r="CP5" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="CQ5" s="33" t="s">
         <v>256</v>
       </c>
-      <c r="P4" s="27" t="s">
-        <v>258</v>
-      </c>
-      <c r="Q4" s="27" t="s">
-        <v>260</v>
-      </c>
-      <c r="R4" s="27" t="s">
-        <v>262</v>
-      </c>
-      <c r="S4" s="27" t="s">
-        <v>264</v>
-      </c>
-      <c r="T4" s="27" t="s">
-        <v>266</v>
-      </c>
-      <c r="U4" s="27" t="s">
-        <v>268</v>
-      </c>
-      <c r="V4" s="27" t="s">
-        <v>270</v>
-      </c>
-      <c r="W4" s="27" t="s">
-        <v>272</v>
-      </c>
-      <c r="X4" s="27" t="s">
-        <v>273</v>
-      </c>
-      <c r="Y4" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="Z4" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA4" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="AB4" s="27" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC4" s="28" t="s">
-        <v>85</v>
-      </c>
-      <c r="AD4" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="AE4" s="27" t="s">
-        <v>87</v>
-      </c>
-      <c r="AF4" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="AG4" s="28" t="s">
-        <v>89</v>
-      </c>
-      <c r="AH4" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="AI4" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="AJ4" s="27" t="s">
-        <v>92</v>
-      </c>
-      <c r="AK4" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="AL4" s="27" t="s">
-        <v>94</v>
-      </c>
-      <c r="AM4" s="27" t="s">
-        <v>95</v>
-      </c>
-      <c r="AN4" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="AO4" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="AP4" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="AQ4" s="27" t="s">
-        <v>99</v>
-      </c>
-      <c r="AR4" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="AS4" s="27" t="s">
-        <v>101</v>
-      </c>
-      <c r="AT4" s="27" t="s">
-        <v>102</v>
-      </c>
-      <c r="AU4" s="27" t="s">
-        <v>103</v>
-      </c>
-      <c r="AV4" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="AW4" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="AX4" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="AY4" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="AZ4" s="27" t="s">
-        <v>108</v>
-      </c>
-      <c r="BA4" s="27" t="s">
-        <v>109</v>
-      </c>
-      <c r="BB4" s="27" t="s">
-        <v>110</v>
-      </c>
-      <c r="BC4" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="BD4" s="27" t="s">
-        <v>112</v>
-      </c>
-      <c r="BE4" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="BF4" s="27" t="s">
-        <v>114</v>
-      </c>
-      <c r="BG4" s="27" t="s">
-        <v>115</v>
-      </c>
-      <c r="BH4" s="27" t="s">
-        <v>116</v>
-      </c>
-      <c r="BI4" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="BJ4" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="BK4" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="BL4" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="BM4" s="27" t="s">
-        <v>121</v>
-      </c>
-      <c r="BN4" s="27" t="s">
-        <v>122</v>
-      </c>
-      <c r="BO4" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="BP4" s="27" t="s">
-        <v>124</v>
-      </c>
-      <c r="BQ4" s="27" t="s">
-        <v>125</v>
-      </c>
-      <c r="BR4" s="27" t="s">
-        <v>126</v>
-      </c>
-      <c r="BS4" s="27" t="s">
-        <v>127</v>
-      </c>
-      <c r="BT4" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="BU4" s="27" t="s">
-        <v>129</v>
-      </c>
-      <c r="BV4" s="27" t="s">
-        <v>130</v>
-      </c>
-      <c r="BW4" s="27" t="s">
-        <v>131</v>
-      </c>
-      <c r="BX4" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="BY4" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="BZ4" s="27" t="s">
-        <v>134</v>
-      </c>
-      <c r="CA4" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="CB4" s="27" t="s">
-        <v>136</v>
-      </c>
-      <c r="CC4" s="27" t="s">
-        <v>137</v>
-      </c>
-      <c r="CD4" s="27" t="s">
-        <v>138</v>
-      </c>
-      <c r="CE4" s="27" t="s">
-        <v>139</v>
-      </c>
-      <c r="CF4" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="CG4" s="27" t="s">
-        <v>141</v>
-      </c>
-      <c r="CH4" s="27" t="s">
-        <v>142</v>
-      </c>
-      <c r="CI4" s="27" t="s">
-        <v>143</v>
-      </c>
-      <c r="CJ4" s="27" t="s">
-        <v>144</v>
-      </c>
-      <c r="CK4" s="27" t="s">
-        <v>145</v>
-      </c>
-      <c r="CL4" s="27" t="s">
-        <v>146</v>
-      </c>
-      <c r="CM4" s="27" t="s">
-        <v>147</v>
-      </c>
-      <c r="CN4" s="27" t="s">
-        <v>148</v>
-      </c>
-      <c r="CO4" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="CP4" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="CQ4" s="27" t="s">
-        <v>151</v>
-      </c>
-      <c r="CR4" s="27" t="s">
-        <v>152</v>
-      </c>
-      <c r="CS4" s="27" t="s">
-        <v>153</v>
-      </c>
-      <c r="CT4" s="27" t="s">
-        <v>154</v>
-      </c>
-      <c r="CU4" s="27" t="s">
-        <v>155</v>
-      </c>
-      <c r="CV4" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="CW4" s="27" t="s">
-        <v>157</v>
-      </c>
-      <c r="CX4" s="27" t="s">
-        <v>158</v>
-      </c>
-      <c r="CY4" s="27" t="s">
-        <v>159</v>
-      </c>
-      <c r="CZ4" s="27" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="5" spans="1:104" ht="31" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
-        <v>161</v>
-      </c>
-      <c r="B5" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="C5" s="33" t="s">
-        <v>163</v>
-      </c>
-      <c r="D5" s="32" t="s">
-        <v>164</v>
-      </c>
-      <c r="E5" s="32" t="s">
-        <v>165</v>
-      </c>
-      <c r="F5" s="32" t="s">
-        <v>166</v>
-      </c>
-      <c r="G5" s="33" t="s">
-        <v>167</v>
-      </c>
-      <c r="H5" s="33" t="s">
-        <v>168</v>
-      </c>
-      <c r="I5" s="33" t="s">
-        <v>169</v>
-      </c>
-      <c r="J5" s="33" t="s">
-        <v>170</v>
-      </c>
-      <c r="K5" s="33" t="s">
-        <v>171</v>
-      </c>
-      <c r="L5" s="33" t="s">
-        <v>172</v>
-      </c>
-      <c r="M5" s="33" t="s">
+      <c r="CR5" s="33" t="s">
         <v>255</v>
       </c>
-      <c r="N5" s="33" t="s">
-        <v>254</v>
-      </c>
-      <c r="O5" s="33" t="s">
-        <v>257</v>
-      </c>
-      <c r="P5" s="33" t="s">
-        <v>259</v>
-      </c>
-      <c r="Q5" s="33" t="s">
-        <v>261</v>
-      </c>
-      <c r="R5" s="33" t="s">
-        <v>263</v>
-      </c>
-      <c r="S5" s="33" t="s">
-        <v>265</v>
-      </c>
-      <c r="T5" s="33" t="s">
-        <v>267</v>
-      </c>
-      <c r="U5" s="33" t="s">
-        <v>269</v>
-      </c>
-      <c r="V5" s="33" t="s">
-        <v>271</v>
-      </c>
-      <c r="W5" s="33" t="s">
-        <v>276</v>
-      </c>
-      <c r="X5" s="33" t="s">
-        <v>274</v>
-      </c>
-      <c r="Y5" s="33" t="s">
-        <v>173</v>
-      </c>
-      <c r="Z5" s="34" t="s">
-        <v>174</v>
-      </c>
-      <c r="AA5" s="34" t="s">
-        <v>175</v>
-      </c>
-      <c r="AB5" s="32" t="s">
-        <v>176</v>
-      </c>
-      <c r="AC5" s="34" t="s">
-        <v>177</v>
-      </c>
-      <c r="AD5" s="33" t="s">
-        <v>178</v>
-      </c>
-      <c r="AE5" s="33" t="s">
-        <v>179</v>
-      </c>
-      <c r="AF5" s="34" t="s">
-        <v>180</v>
-      </c>
-      <c r="AG5" s="34" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH5" s="32" t="s">
-        <v>182</v>
-      </c>
-      <c r="AI5" s="34" t="s">
-        <v>183</v>
-      </c>
-      <c r="AJ5" s="33" t="s">
-        <v>184</v>
-      </c>
-      <c r="AK5" s="33" t="s">
-        <v>185</v>
-      </c>
-      <c r="AL5" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="AM5" s="32" t="s">
-        <v>186</v>
-      </c>
-      <c r="AN5" s="33" t="s">
-        <v>44</v>
-      </c>
-      <c r="AO5" s="33" t="s">
-        <v>187</v>
-      </c>
-      <c r="AP5" s="33" t="s">
-        <v>188</v>
-      </c>
-      <c r="AQ5" s="33" t="s">
-        <v>189</v>
-      </c>
-      <c r="AR5" s="32" t="s">
-        <v>190</v>
-      </c>
-      <c r="AS5" s="32" t="s">
-        <v>191</v>
-      </c>
-      <c r="AT5" s="33" t="s">
-        <v>192</v>
-      </c>
-      <c r="AU5" s="33" t="s">
-        <v>193</v>
-      </c>
-      <c r="AV5" s="33" t="s">
-        <v>194</v>
-      </c>
-      <c r="AW5" s="33" t="s">
-        <v>195</v>
-      </c>
-      <c r="AX5" s="33" t="s">
-        <v>196</v>
-      </c>
-      <c r="AY5" s="33" t="s">
-        <v>197</v>
-      </c>
-      <c r="AZ5" s="33" t="s">
-        <v>198</v>
-      </c>
-      <c r="BA5" s="33" t="s">
-        <v>199</v>
-      </c>
-      <c r="BB5" s="33" t="s">
-        <v>200</v>
-      </c>
-      <c r="BC5" s="33" t="s">
-        <v>201</v>
-      </c>
-      <c r="BD5" s="33" t="s">
-        <v>202</v>
-      </c>
-      <c r="BE5" s="33" t="s">
-        <v>203</v>
-      </c>
-      <c r="BF5" s="33" t="s">
-        <v>204</v>
-      </c>
-      <c r="BG5" s="33" t="s">
-        <v>205</v>
-      </c>
-      <c r="BH5" s="33" t="s">
-        <v>206</v>
-      </c>
-      <c r="BI5" s="33" t="s">
-        <v>207</v>
-      </c>
-      <c r="BJ5" s="33" t="s">
-        <v>208</v>
-      </c>
-      <c r="BK5" s="33" t="s">
-        <v>209</v>
-      </c>
-      <c r="BL5" s="33" t="s">
-        <v>210</v>
-      </c>
-      <c r="BM5" s="33" t="s">
-        <v>211</v>
-      </c>
-      <c r="BN5" s="33" t="s">
-        <v>212</v>
-      </c>
-      <c r="BO5" s="33" t="s">
-        <v>213</v>
-      </c>
-      <c r="BP5" s="33" t="s">
-        <v>214</v>
-      </c>
-      <c r="BQ5" s="33" t="s">
-        <v>215</v>
-      </c>
-      <c r="BR5" s="33" t="s">
-        <v>216</v>
-      </c>
-      <c r="BS5" s="33" t="s">
+      <c r="CS5" s="33" t="s">
         <v>217</v>
       </c>
-      <c r="BT5" s="33" t="s">
+      <c r="CT5" s="33" t="s">
         <v>218</v>
       </c>
-      <c r="BU5" s="33" t="s">
+      <c r="CU5" s="33" t="s">
         <v>219</v>
       </c>
-      <c r="BV5" s="33" t="s">
+      <c r="CV5" s="33" t="s">
         <v>220</v>
       </c>
-      <c r="BW5" s="33" t="s">
+      <c r="CW5" s="33" t="s">
         <v>221</v>
       </c>
-      <c r="BX5" s="33" t="s">
+      <c r="CX5" s="33" t="s">
         <v>222</v>
       </c>
-      <c r="BY5" s="33" t="s">
+      <c r="CY5" s="33" t="s">
         <v>223</v>
       </c>
-      <c r="BZ5" s="33" t="s">
+      <c r="CZ5" s="33" t="s">
         <v>224</v>
       </c>
-      <c r="CA5" s="33" t="s">
-        <v>225</v>
-      </c>
-      <c r="CB5" s="33" t="s">
-        <v>226</v>
-      </c>
-      <c r="CC5" s="33" t="s">
-        <v>227</v>
-      </c>
-      <c r="CD5" s="33" t="s">
-        <v>228</v>
-      </c>
-      <c r="CE5" s="33" t="s">
-        <v>229</v>
-      </c>
-      <c r="CF5" s="33" t="s">
-        <v>230</v>
-      </c>
-      <c r="CG5" s="33" t="s">
-        <v>231</v>
-      </c>
-      <c r="CH5" s="33" t="s">
-        <v>232</v>
-      </c>
-      <c r="CI5" s="33" t="s">
-        <v>233</v>
-      </c>
-      <c r="CJ5" s="33" t="s">
-        <v>234</v>
-      </c>
-      <c r="CK5" s="33" t="s">
-        <v>235</v>
-      </c>
-      <c r="CL5" s="33" t="s">
-        <v>236</v>
-      </c>
-      <c r="CM5" s="33" t="s">
-        <v>237</v>
-      </c>
-      <c r="CN5" s="33" t="s">
-        <v>238</v>
-      </c>
-      <c r="CO5" s="33" t="s">
-        <v>239</v>
-      </c>
-      <c r="CP5" s="33" t="s">
-        <v>240</v>
-      </c>
-      <c r="CQ5" s="33" t="s">
-        <v>241</v>
-      </c>
-      <c r="CR5" s="33" t="s">
-        <v>242</v>
-      </c>
-      <c r="CS5" s="33" t="s">
-        <v>243</v>
-      </c>
-      <c r="CT5" s="33" t="s">
-        <v>244</v>
-      </c>
-      <c r="CU5" s="33" t="s">
-        <v>245</v>
-      </c>
-      <c r="CV5" s="33" t="s">
-        <v>246</v>
-      </c>
-      <c r="CW5" s="33" t="s">
-        <v>247</v>
-      </c>
-      <c r="CX5" s="33" t="s">
-        <v>248</v>
-      </c>
-      <c r="CY5" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="CZ5" s="33" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="6" spans="1:104" ht="19" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="DA5" s="33" t="s">
+        <v>344</v>
+      </c>
+      <c r="DB5" s="33" t="s">
+        <v>345</v>
+      </c>
+      <c r="DC5" s="33" t="s">
+        <v>307</v>
+      </c>
+      <c r="DD5" s="33" t="s">
+        <v>308</v>
+      </c>
+      <c r="DE5" s="33" t="s">
+        <v>309</v>
+      </c>
+      <c r="DF5" s="33" t="s">
+        <v>310</v>
+      </c>
+      <c r="DG5" s="33" t="s">
+        <v>311</v>
+      </c>
+      <c r="DH5" s="33" t="s">
+        <v>312</v>
+      </c>
+      <c r="DI5" s="33" t="s">
+        <v>313</v>
+      </c>
+      <c r="DJ5" s="33" t="s">
+        <v>314</v>
+      </c>
+      <c r="DK5" s="33" t="s">
+        <v>315</v>
+      </c>
+      <c r="DL5" s="33" t="s">
+        <v>316</v>
+      </c>
+      <c r="DM5" s="33" t="s">
+        <v>317</v>
+      </c>
+      <c r="DN5" s="33" t="s">
+        <v>318</v>
+      </c>
+      <c r="DO5" s="33" t="s">
+        <v>319</v>
+      </c>
+      <c r="DP5" s="33" t="s">
+        <v>320</v>
+      </c>
+      <c r="DQ5" s="33" t="s">
+        <v>321</v>
+      </c>
+      <c r="DR5" s="33" t="s">
+        <v>322</v>
+      </c>
+      <c r="DS5" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="DT5" s="33" t="s">
+        <v>324</v>
+      </c>
+      <c r="DU5" s="33" t="s">
+        <v>325</v>
+      </c>
+      <c r="DV5" s="33" t="s">
+        <v>326</v>
+      </c>
+      <c r="DW5" s="33" t="s">
+        <v>327</v>
+      </c>
+      <c r="DX5" s="33" t="s">
+        <v>328</v>
+      </c>
+      <c r="DY5" s="33" t="s">
+        <v>329</v>
+      </c>
+      <c r="DZ5" s="33" t="s">
+        <v>330</v>
+      </c>
+      <c r="EA5" s="33" t="s">
+        <v>331</v>
+      </c>
+      <c r="EB5" s="33" t="s">
+        <v>332</v>
+      </c>
+      <c r="EC5" s="33" t="s">
+        <v>333</v>
+      </c>
+      <c r="ED5" s="33" t="s">
+        <v>334</v>
+      </c>
+      <c r="EE5" s="33" t="s">
+        <v>335</v>
+      </c>
+      <c r="EF5" s="33" t="s">
+        <v>336</v>
+      </c>
+      <c r="EG5" s="33" t="s">
+        <v>337</v>
+      </c>
+      <c r="EH5" s="33" t="s">
+        <v>338</v>
+      </c>
+      <c r="EI5" s="33" t="s">
+        <v>339</v>
+      </c>
+      <c r="EJ5" s="33" t="s">
+        <v>340</v>
+      </c>
+      <c r="EK5" s="33" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="6" spans="1:141" ht="19" thickTop="1" x14ac:dyDescent="0.2">
       <c r="E6" s="35"/>
       <c r="CS6" s="36"/>
       <c r="CT6" s="36"/>
@@ -2949,43 +3738,43 @@
       <c r="CY6" s="36"/>
       <c r="CZ6" s="36"/>
     </row>
-    <row r="7" spans="1:104" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:141" x14ac:dyDescent="0.2">
       <c r="CN7" s="2"/>
       <c r="CQ7" s="2"/>
     </row>
-    <row r="8" spans="1:104" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:141" x14ac:dyDescent="0.2">
       <c r="CN8" s="2"/>
       <c r="CQ8" s="2"/>
     </row>
-    <row r="9" spans="1:104" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:141" x14ac:dyDescent="0.2">
       <c r="CN9" s="2"/>
       <c r="CQ9" s="2"/>
     </row>
-    <row r="10" spans="1:104" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:141" x14ac:dyDescent="0.2">
       <c r="CN10" s="2"/>
       <c r="CQ10" s="2"/>
     </row>
-    <row r="11" spans="1:104" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:141" x14ac:dyDescent="0.2">
       <c r="CN11" s="2"/>
       <c r="CQ11" s="2"/>
     </row>
-    <row r="12" spans="1:104" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:141" x14ac:dyDescent="0.2">
       <c r="CN12" s="2"/>
       <c r="CQ12" s="2"/>
     </row>
-    <row r="13" spans="1:104" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:141" x14ac:dyDescent="0.2">
       <c r="CN13" s="2"/>
       <c r="CQ13" s="2"/>
     </row>
-    <row r="14" spans="1:104" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:141" x14ac:dyDescent="0.2">
       <c r="CN14" s="2"/>
       <c r="CQ14" s="2"/>
     </row>
-    <row r="15" spans="1:104" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:141" x14ac:dyDescent="0.2">
       <c r="CN15" s="2"/>
       <c r="CQ15" s="2"/>
     </row>
-    <row r="16" spans="1:104" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:141" x14ac:dyDescent="0.2">
       <c r="CN16" s="2"/>
       <c r="CQ16" s="2"/>
     </row>

</xml_diff>

<commit_message>
ANW-2999 Add validated BDO Events to bulk import
Planning-assisted-by: Codex [GPT-5.6 Sol]
Code-assisted-by: Codex [GPT-5.6 Sol]
Tests-coauthored-by: Grok [Grok 4.7]
</commit_message>
<xml_diff>
--- a/frontend/public/bulk_import_templates/bulk_import_DO_template.xlsx
+++ b/frontend/public/bulk_import_templates/bulk_import_DO_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zeffmorgan/src/lyrasis/archivesspace/frontend/public/bulk_import_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6626C96-CED2-3646-9CBC-6C76BAC05211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A992613F-4A02-ED4D-A0B6-7BC7EEE406C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34560" yWindow="600" windowWidth="38400" windowHeight="11860" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="338">
   <si>
     <t>This is the template for use with the bulk_import ("Load SpreadSheet") for importing digital ob jects to associate with archival objects .  You may replace this line with something of your choosing after you've copied the file for your use.</t>
   </si>
@@ -983,13 +983,281 @@
   <si>
     <t>Agent Type (agent_person/agent_family/agent_corporate_entity)
 Replaces the</t>
+  </si>
+  <si>
+    <t>Event</t>
+  </si>
+  <si>
+    <t>event_1_type</t>
+  </si>
+  <si>
+    <t>event_1_date</t>
+  </si>
+  <si>
+    <t>event_1_date_label</t>
+  </si>
+  <si>
+    <t>event_1_outcome</t>
+  </si>
+  <si>
+    <t>event_1_outcome_note</t>
+  </si>
+  <si>
+    <t>event_1_agent_1_record_id</t>
+  </si>
+  <si>
+    <t>event_1_agent_1_agent_type</t>
+  </si>
+  <si>
+    <t>event_1_agent_1_role</t>
+  </si>
+  <si>
+    <t>Event(1) Outcome</t>
+  </si>
+  <si>
+    <t>Event(1) Outcome Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event(1) Type </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event(1) Date </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event(1) Date Label </t>
+  </si>
+  <si>
+    <t>Event(1) Agent(1) Record ID</t>
+  </si>
+  <si>
+    <t>Event(1) Agent(1) Type</t>
+  </si>
+  <si>
+    <t>Event(1) Agent(1) Role</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>REQUIRED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> with an explicit Agent Record ID</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>REQUIRED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> for numeric ID
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">LEAVE BLANK </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>for URI</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Numeric ID or canonical URI
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">MUST </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>be an existing agent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+If all Agent fields are blank, uses the ArchivesSpace software Agent with the `executing_program` role.</t>
+    </r>
+  </si>
+  <si>
+    <t>Event outcome (installation-wide controlled value; optional)
+Example: pass</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>REQUIRED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> if specifying Event
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+YYYY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>YYYY-MM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, or </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>YYYY-MM-DD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> e</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>ntered as text.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Excel can convert partial dates into numeric dates, losing the intended precision and causing an import error.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>REQUIRED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> if specifying Event
+Installation-wide controlled value. 
+Example: cataloged</t>
+    </r>
+  </si>
+  <si>
+    <t>Installation-wide controlled value. When a Date is supplied without a Date Label, ArchivesSpace stores 'other'.</t>
+  </si>
+  <si>
+    <t>Additional information about the event outcome (free text; optional; may be supplied without an Outcome)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1055,8 +1323,19 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1120,6 +1399,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE8DDF2"/>
+        <bgColor rgb="FFE6E0EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor rgb="FFDCE6F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF2DF"/>
+        <bgColor rgb="FFFDEADA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF2DF"/>
         <bgColor rgb="FFE6E0EC"/>
       </patternFill>
     </fill>
@@ -1206,7 +1503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1296,9 +1593,6 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1336,6 +1630,30 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1410,6 +1728,9 @@
       <rgbColor rgb="00333399"/>
       <rgbColor rgb="00333333"/>
     </indexedColors>
+    <mruColors>
+      <color rgb="FFEBF2DF"/>
+    </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1739,7 +2060,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DH6"/>
+  <dimension ref="A1:DP6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.33203125" style="1" customWidth="1"/>
@@ -1800,16 +2121,19 @@
     <col min="107" max="107" width="17.33203125" style="2" customWidth="1"/>
     <col min="108" max="111" width="16" style="2" customWidth="1"/>
     <col min="112" max="112" width="13.5" style="2" customWidth="1"/>
+    <col min="113" max="113" width="21.5" style="2" customWidth="1"/>
+    <col min="114" max="114" width="21.5" style="3" customWidth="1"/>
+    <col min="115" max="120" width="21.5" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:112" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:120" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="BG1" s="2"/>
       <c r="BJ1" s="2"/>
     </row>
-    <row r="2" spans="1:112" s="2" customFormat="1" ht="41.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:120" s="2" customFormat="1" ht="41.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1885,40 +2209,40 @@
       <c r="Y2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="Z2" s="35" t="s">
+      <c r="Z2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AA2" s="35" t="s">
+      <c r="AA2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AB2" s="35" t="s">
+      <c r="AB2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AC2" s="35" t="s">
+      <c r="AC2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AD2" s="35" t="s">
+      <c r="AD2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AE2" s="35" t="s">
+      <c r="AE2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AF2" s="35" t="s">
+      <c r="AF2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AG2" s="35" t="s">
+      <c r="AG2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AH2" s="35" t="s">
+      <c r="AH2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AI2" s="35" t="s">
+      <c r="AI2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AJ2" s="35" t="s">
+      <c r="AJ2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AK2" s="35" t="s">
+      <c r="AK2" s="34" t="s">
         <v>5</v>
       </c>
       <c r="AL2" s="12" t="s">
@@ -2035,85 +2359,85 @@
       <c r="BW2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="BX2" s="37" t="s">
+      <c r="BX2" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="BY2" s="37" t="s">
+      <c r="BY2" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="BZ2" s="39" t="s">
+      <c r="BZ2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CA2" s="39" t="s">
+      <c r="CA2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CB2" s="39" t="s">
+      <c r="CB2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CC2" s="39" t="s">
+      <c r="CC2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CD2" s="39" t="s">
+      <c r="CD2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CE2" s="39" t="s">
+      <c r="CE2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CF2" s="39" t="s">
+      <c r="CF2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CG2" s="39" t="s">
+      <c r="CG2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CH2" s="39" t="s">
+      <c r="CH2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CI2" s="39" t="s">
+      <c r="CI2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CJ2" s="39" t="s">
+      <c r="CJ2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CK2" s="39" t="s">
+      <c r="CK2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CL2" s="39" t="s">
+      <c r="CL2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CM2" s="39" t="s">
+      <c r="CM2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CN2" s="39" t="s">
+      <c r="CN2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CO2" s="39" t="s">
+      <c r="CO2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CP2" s="39" t="s">
+      <c r="CP2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CQ2" s="39" t="s">
+      <c r="CQ2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CR2" s="39" t="s">
+      <c r="CR2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CS2" s="39" t="s">
+      <c r="CS2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CT2" s="39" t="s">
+      <c r="CT2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CU2" s="39" t="s">
+      <c r="CU2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CV2" s="39" t="s">
+      <c r="CV2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CW2" s="39" t="s">
+      <c r="CW2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CX2" s="39" t="s">
+      <c r="CX2" s="38" t="s">
         <v>14</v>
       </c>
       <c r="CY2" s="12" t="s">
@@ -2146,8 +2470,32 @@
       <c r="DH2" s="12" t="s">
         <v>15</v>
       </c>
+      <c r="DI2" s="44" t="s">
+        <v>313</v>
+      </c>
+      <c r="DJ2" s="45" t="s">
+        <v>313</v>
+      </c>
+      <c r="DK2" s="44" t="s">
+        <v>313</v>
+      </c>
+      <c r="DL2" s="44" t="s">
+        <v>313</v>
+      </c>
+      <c r="DM2" s="44" t="s">
+        <v>313</v>
+      </c>
+      <c r="DN2" s="44" t="s">
+        <v>313</v>
+      </c>
+      <c r="DO2" s="44" t="s">
+        <v>313</v>
+      </c>
+      <c r="DP2" s="44" t="s">
+        <v>313</v>
+      </c>
     </row>
-    <row r="3" spans="1:112" ht="132" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:120" ht="132" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>16</v>
       </c>
@@ -2223,40 +2571,40 @@
       <c r="Y3" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="Z3" s="36" t="s">
+      <c r="Z3" s="35" t="s">
         <v>311</v>
       </c>
-      <c r="AA3" s="36" t="s">
+      <c r="AA3" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="AB3" s="36" t="s">
+      <c r="AB3" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="AC3" s="36" t="s">
+      <c r="AC3" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="AD3" s="36" t="s">
+      <c r="AD3" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="AE3" s="36" t="s">
+      <c r="AE3" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="AF3" s="36" t="s">
+      <c r="AF3" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="AG3" s="36" t="s">
+      <c r="AG3" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="AH3" s="36" t="s">
+      <c r="AH3" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="AI3" s="36" t="s">
+      <c r="AI3" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="AJ3" s="36" t="s">
+      <c r="AJ3" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="AK3" s="36" t="s">
+      <c r="AK3" s="35" t="s">
         <v>45</v>
       </c>
       <c r="AL3" s="25" t="s">
@@ -2352,7 +2700,7 @@
       <c r="BP3" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="BQ3" s="22" t="s">
+      <c r="BQ3" s="43" t="s">
         <v>64</v>
       </c>
       <c r="BR3" s="20" t="s">
@@ -2373,85 +2721,85 @@
       <c r="BW3" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="BX3" s="38" t="s">
+      <c r="BX3" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="BY3" s="38" t="s">
+      <c r="BY3" s="37" t="s">
         <v>66</v>
       </c>
-      <c r="BZ3" s="40" t="s">
+      <c r="BZ3" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="CA3" s="40" t="s">
+      <c r="CA3" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="CB3" s="40" t="s">
+      <c r="CB3" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="CC3" s="40" t="s">
+      <c r="CC3" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="CD3" s="40" t="s">
+      <c r="CD3" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="CE3" s="40" t="s">
+      <c r="CE3" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="CF3" s="40" t="s">
+      <c r="CF3" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="CG3" s="40" t="s">
+      <c r="CG3" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="CH3" s="40" t="s">
+      <c r="CH3" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="CI3" s="40" t="s">
+      <c r="CI3" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="CJ3" s="40" t="s">
+      <c r="CJ3" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="CK3" s="40" t="s">
+      <c r="CK3" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="CL3" s="40" t="s">
+      <c r="CL3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="CM3" s="40" t="s">
+      <c r="CM3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="CN3" s="40" t="s">
+      <c r="CN3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="CO3" s="40" t="s">
+      <c r="CO3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="CP3" s="40" t="s">
+      <c r="CP3" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="CQ3" s="40" t="s">
+      <c r="CQ3" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="CR3" s="40" t="s">
+      <c r="CR3" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="CS3" s="40" t="s">
+      <c r="CS3" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="CT3" s="40" t="s">
+      <c r="CT3" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="CU3" s="40" t="s">
+      <c r="CU3" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="CV3" s="40" t="s">
+      <c r="CV3" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="CW3" s="40" t="s">
+      <c r="CW3" s="39" t="s">
         <v>75</v>
       </c>
-      <c r="CX3" s="40" t="s">
+      <c r="CX3" s="39" t="s">
         <v>76</v>
       </c>
       <c r="CY3" s="25" t="s">
@@ -2484,12 +2832,36 @@
       <c r="DH3" s="25" t="s">
         <v>86</v>
       </c>
+      <c r="DI3" s="46" t="s">
+        <v>335</v>
+      </c>
+      <c r="DJ3" s="47" t="s">
+        <v>334</v>
+      </c>
+      <c r="DK3" s="48" t="s">
+        <v>336</v>
+      </c>
+      <c r="DL3" s="48" t="s">
+        <v>333</v>
+      </c>
+      <c r="DM3" s="48" t="s">
+        <v>337</v>
+      </c>
+      <c r="DN3" s="48" t="s">
+        <v>332</v>
+      </c>
+      <c r="DO3" s="46" t="s">
+        <v>331</v>
+      </c>
+      <c r="DP3" s="46" t="s">
+        <v>330</v>
+      </c>
     </row>
-    <row r="4" spans="1:112" s="27" customFormat="1" ht="41.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:120" s="27" customFormat="1" ht="41.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="40" t="s">
         <v>88</v>
       </c>
       <c r="C4" s="27" t="s">
@@ -2708,7 +3080,7 @@
       <c r="BV4" s="27" t="s">
         <v>160</v>
       </c>
-      <c r="BW4" s="30" t="s">
+      <c r="BW4" s="42" t="s">
         <v>161</v>
       </c>
       <c r="BX4" s="27" t="s">
@@ -2822,348 +3194,396 @@
       <c r="DH4" s="27" t="s">
         <v>198</v>
       </c>
+      <c r="DI4" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="DJ4" s="28" t="s">
+        <v>315</v>
+      </c>
+      <c r="DK4" s="27" t="s">
+        <v>316</v>
+      </c>
+      <c r="DL4" s="27" t="s">
+        <v>317</v>
+      </c>
+      <c r="DM4" s="27" t="s">
+        <v>318</v>
+      </c>
+      <c r="DN4" s="27" t="s">
+        <v>319</v>
+      </c>
+      <c r="DO4" s="27" t="s">
+        <v>320</v>
+      </c>
+      <c r="DP4" s="27" t="s">
+        <v>321</v>
+      </c>
     </row>
-    <row r="5" spans="1:112" ht="31" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
+    <row r="5" spans="1:120" ht="31" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="30" t="s">
         <v>199</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="41" t="s">
         <v>200</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="31" t="s">
         <v>201</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="32" t="s">
         <v>202</v>
       </c>
-      <c r="E5" s="32" t="s">
+      <c r="E5" s="31" t="s">
         <v>203</v>
       </c>
-      <c r="F5" s="32" t="s">
+      <c r="F5" s="31" t="s">
         <v>204</v>
       </c>
-      <c r="G5" s="32" t="s">
+      <c r="G5" s="31" t="s">
         <v>205</v>
       </c>
-      <c r="H5" s="33" t="s">
+      <c r="H5" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="I5" s="33" t="s">
+      <c r="I5" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="J5" s="33" t="s">
+      <c r="J5" s="32" t="s">
         <v>208</v>
       </c>
-      <c r="K5" s="33" t="s">
+      <c r="K5" s="32" t="s">
         <v>209</v>
       </c>
-      <c r="L5" s="33" t="s">
+      <c r="L5" s="32" t="s">
         <v>210</v>
       </c>
-      <c r="M5" s="33" t="s">
+      <c r="M5" s="32" t="s">
         <v>211</v>
       </c>
-      <c r="N5" s="33" t="s">
+      <c r="N5" s="32" t="s">
         <v>212</v>
       </c>
-      <c r="O5" s="34" t="s">
+      <c r="O5" s="33" t="s">
         <v>213</v>
       </c>
-      <c r="P5" s="34" t="s">
+      <c r="P5" s="33" t="s">
         <v>214</v>
       </c>
-      <c r="Q5" s="32" t="s">
+      <c r="Q5" s="31" t="s">
         <v>215</v>
       </c>
-      <c r="R5" s="34" t="s">
+      <c r="R5" s="33" t="s">
         <v>216</v>
       </c>
-      <c r="S5" s="33" t="s">
+      <c r="S5" s="32" t="s">
         <v>217</v>
       </c>
-      <c r="T5" s="33" t="s">
+      <c r="T5" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="U5" s="34" t="s">
+      <c r="U5" s="33" t="s">
         <v>219</v>
       </c>
-      <c r="V5" s="34" t="s">
+      <c r="V5" s="33" t="s">
         <v>220</v>
       </c>
-      <c r="W5" s="32" t="s">
+      <c r="W5" s="31" t="s">
         <v>221</v>
       </c>
-      <c r="X5" s="34" t="s">
+      <c r="X5" s="33" t="s">
         <v>222</v>
       </c>
-      <c r="Y5" s="33" t="s">
+      <c r="Y5" s="32" t="s">
         <v>223</v>
       </c>
-      <c r="Z5" s="33" t="s">
+      <c r="Z5" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="AA5" s="33" t="s">
+      <c r="AA5" s="32" t="s">
         <v>225</v>
       </c>
-      <c r="AB5" s="33" t="s">
+      <c r="AB5" s="32" t="s">
         <v>226</v>
       </c>
-      <c r="AC5" s="33" t="s">
+      <c r="AC5" s="32" t="s">
         <v>227</v>
       </c>
-      <c r="AD5" s="33" t="s">
+      <c r="AD5" s="32" t="s">
         <v>228</v>
       </c>
-      <c r="AE5" s="33" t="s">
+      <c r="AE5" s="32" t="s">
         <v>229</v>
       </c>
-      <c r="AF5" s="33" t="s">
+      <c r="AF5" s="32" t="s">
         <v>230</v>
       </c>
-      <c r="AG5" s="33" t="s">
+      <c r="AG5" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="AH5" s="33" t="s">
+      <c r="AH5" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="AI5" s="33" t="s">
+      <c r="AI5" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="AJ5" s="33" t="s">
+      <c r="AJ5" s="32" t="s">
         <v>234</v>
       </c>
-      <c r="AK5" s="33" t="s">
+      <c r="AK5" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="AL5" s="33" t="s">
+      <c r="AL5" s="32" t="s">
         <v>236</v>
       </c>
-      <c r="AM5" s="33" t="s">
+      <c r="AM5" s="32" t="s">
         <v>237</v>
       </c>
-      <c r="AN5" s="33" t="s">
+      <c r="AN5" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="AO5" s="33" t="s">
+      <c r="AO5" s="32" t="s">
         <v>239</v>
       </c>
-      <c r="AP5" s="33" t="s">
+      <c r="AP5" s="32" t="s">
         <v>240</v>
       </c>
-      <c r="AQ5" s="33" t="s">
+      <c r="AQ5" s="32" t="s">
         <v>241</v>
       </c>
-      <c r="AR5" s="33" t="s">
+      <c r="AR5" s="32" t="s">
         <v>242</v>
       </c>
-      <c r="AS5" s="33" t="s">
+      <c r="AS5" s="32" t="s">
         <v>243</v>
       </c>
-      <c r="AT5" s="33" t="s">
+      <c r="AT5" s="32" t="s">
         <v>244</v>
       </c>
-      <c r="AU5" s="33" t="s">
+      <c r="AU5" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="AV5" s="33" t="s">
+      <c r="AV5" s="32" t="s">
         <v>246</v>
       </c>
-      <c r="AW5" s="33" t="s">
+      <c r="AW5" s="32" t="s">
         <v>247</v>
       </c>
-      <c r="AX5" s="33" t="s">
+      <c r="AX5" s="32" t="s">
         <v>248</v>
       </c>
-      <c r="AY5" s="33" t="s">
+      <c r="AY5" s="32" t="s">
         <v>249</v>
       </c>
-      <c r="AZ5" s="33" t="s">
+      <c r="AZ5" s="32" t="s">
         <v>250</v>
       </c>
-      <c r="BA5" s="33" t="s">
+      <c r="BA5" s="32" t="s">
         <v>251</v>
       </c>
-      <c r="BB5" s="33" t="s">
+      <c r="BB5" s="32" t="s">
         <v>252</v>
       </c>
-      <c r="BC5" s="33" t="s">
+      <c r="BC5" s="32" t="s">
         <v>253</v>
       </c>
-      <c r="BD5" s="33" t="s">
+      <c r="BD5" s="32" t="s">
         <v>254</v>
       </c>
-      <c r="BE5" s="33" t="s">
+      <c r="BE5" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="BF5" s="33" t="s">
+      <c r="BF5" s="32" t="s">
         <v>256</v>
       </c>
-      <c r="BG5" s="33" t="s">
+      <c r="BG5" s="32" t="s">
         <v>257</v>
       </c>
-      <c r="BH5" s="33" t="s">
+      <c r="BH5" s="32" t="s">
         <v>258</v>
       </c>
-      <c r="BI5" s="33" t="s">
+      <c r="BI5" s="32" t="s">
         <v>259</v>
       </c>
-      <c r="BJ5" s="33" t="s">
+      <c r="BJ5" s="32" t="s">
         <v>260</v>
       </c>
-      <c r="BK5" s="33" t="s">
+      <c r="BK5" s="32" t="s">
         <v>261</v>
       </c>
-      <c r="BL5" s="33" t="s">
+      <c r="BL5" s="32" t="s">
         <v>262</v>
       </c>
-      <c r="BM5" s="32" t="s">
+      <c r="BM5" s="31" t="s">
         <v>263</v>
       </c>
-      <c r="BN5" s="32" t="s">
+      <c r="BN5" s="31" t="s">
         <v>264</v>
       </c>
-      <c r="BO5" s="33" t="s">
+      <c r="BO5" s="32" t="s">
         <v>265</v>
       </c>
-      <c r="BP5" s="33" t="s">
+      <c r="BP5" s="32" t="s">
         <v>266</v>
       </c>
-      <c r="BQ5" s="33" t="s">
+      <c r="BQ5" s="32" t="s">
         <v>267</v>
       </c>
-      <c r="BR5" s="33" t="s">
+      <c r="BR5" s="32" t="s">
         <v>268</v>
       </c>
-      <c r="BS5" s="32" t="s">
+      <c r="BS5" s="31" t="s">
         <v>269</v>
       </c>
-      <c r="BT5" s="32" t="s">
+      <c r="BT5" s="31" t="s">
         <v>270</v>
       </c>
-      <c r="BU5" s="33" t="s">
+      <c r="BU5" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="BV5" s="33" t="s">
+      <c r="BV5" s="32" t="s">
         <v>272</v>
       </c>
-      <c r="BW5" s="33" t="s">
+      <c r="BW5" s="32" t="s">
         <v>273</v>
       </c>
-      <c r="BX5" s="33" t="s">
+      <c r="BX5" s="32" t="s">
         <v>274</v>
       </c>
-      <c r="BY5" s="33" t="s">
+      <c r="BY5" s="32" t="s">
         <v>275</v>
       </c>
-      <c r="BZ5" s="33" t="s">
+      <c r="BZ5" s="32" t="s">
         <v>276</v>
       </c>
-      <c r="CA5" s="33" t="s">
+      <c r="CA5" s="32" t="s">
         <v>277</v>
       </c>
-      <c r="CB5" s="33" t="s">
+      <c r="CB5" s="32" t="s">
         <v>278</v>
       </c>
-      <c r="CC5" s="33" t="s">
+      <c r="CC5" s="32" t="s">
         <v>279</v>
       </c>
-      <c r="CD5" s="33" t="s">
+      <c r="CD5" s="32" t="s">
         <v>280</v>
       </c>
-      <c r="CE5" s="33" t="s">
+      <c r="CE5" s="32" t="s">
         <v>281</v>
       </c>
-      <c r="CF5" s="33" t="s">
+      <c r="CF5" s="32" t="s">
         <v>282</v>
       </c>
-      <c r="CG5" s="33" t="s">
+      <c r="CG5" s="32" t="s">
         <v>283</v>
       </c>
-      <c r="CH5" s="33" t="s">
+      <c r="CH5" s="32" t="s">
         <v>284</v>
       </c>
-      <c r="CI5" s="33" t="s">
+      <c r="CI5" s="32" t="s">
         <v>285</v>
       </c>
-      <c r="CJ5" s="33" t="s">
+      <c r="CJ5" s="32" t="s">
         <v>286</v>
       </c>
-      <c r="CK5" s="33" t="s">
+      <c r="CK5" s="32" t="s">
         <v>287</v>
       </c>
-      <c r="CL5" s="33" t="s">
+      <c r="CL5" s="32" t="s">
         <v>288</v>
       </c>
-      <c r="CM5" s="33" t="s">
+      <c r="CM5" s="32" t="s">
         <v>289</v>
       </c>
-      <c r="CN5" s="33" t="s">
+      <c r="CN5" s="32" t="s">
         <v>290</v>
       </c>
-      <c r="CO5" s="33" t="s">
+      <c r="CO5" s="32" t="s">
         <v>291</v>
       </c>
-      <c r="CP5" s="33" t="s">
+      <c r="CP5" s="32" t="s">
         <v>292</v>
       </c>
-      <c r="CQ5" s="33" t="s">
+      <c r="CQ5" s="32" t="s">
         <v>293</v>
       </c>
-      <c r="CR5" s="33" t="s">
+      <c r="CR5" s="32" t="s">
         <v>294</v>
       </c>
-      <c r="CS5" s="33" t="s">
+      <c r="CS5" s="32" t="s">
         <v>295</v>
       </c>
-      <c r="CT5" s="33" t="s">
+      <c r="CT5" s="32" t="s">
         <v>296</v>
       </c>
-      <c r="CU5" s="33" t="s">
+      <c r="CU5" s="32" t="s">
         <v>297</v>
       </c>
-      <c r="CV5" s="33" t="s">
+      <c r="CV5" s="32" t="s">
         <v>298</v>
       </c>
-      <c r="CW5" s="33" t="s">
+      <c r="CW5" s="32" t="s">
         <v>299</v>
       </c>
-      <c r="CX5" s="33" t="s">
+      <c r="CX5" s="32" t="s">
         <v>300</v>
       </c>
-      <c r="CY5" s="33" t="s">
+      <c r="CY5" s="32" t="s">
         <v>301</v>
       </c>
-      <c r="CZ5" s="33" t="s">
+      <c r="CZ5" s="32" t="s">
         <v>302</v>
       </c>
-      <c r="DA5" s="33" t="s">
+      <c r="DA5" s="32" t="s">
         <v>303</v>
       </c>
-      <c r="DB5" s="33" t="s">
+      <c r="DB5" s="32" t="s">
         <v>304</v>
       </c>
-      <c r="DC5" s="33" t="s">
+      <c r="DC5" s="32" t="s">
         <v>305</v>
       </c>
-      <c r="DD5" s="33" t="s">
+      <c r="DD5" s="32" t="s">
         <v>306</v>
       </c>
-      <c r="DE5" s="33" t="s">
+      <c r="DE5" s="32" t="s">
         <v>307</v>
       </c>
-      <c r="DF5" s="33" t="s">
+      <c r="DF5" s="32" t="s">
         <v>308</v>
       </c>
-      <c r="DG5" s="33" t="s">
+      <c r="DG5" s="32" t="s">
         <v>309</v>
       </c>
-      <c r="DH5" s="33" t="s">
+      <c r="DH5" s="32" t="s">
         <v>310</v>
       </c>
+      <c r="DI5" s="32" t="s">
+        <v>324</v>
+      </c>
+      <c r="DJ5" s="33" t="s">
+        <v>325</v>
+      </c>
+      <c r="DK5" s="32" t="s">
+        <v>326</v>
+      </c>
+      <c r="DL5" s="32" t="s">
+        <v>322</v>
+      </c>
+      <c r="DM5" s="32" t="s">
+        <v>323</v>
+      </c>
+      <c r="DN5" s="32" t="s">
+        <v>327</v>
+      </c>
+      <c r="DO5" s="32" t="s">
+        <v>328</v>
+      </c>
+      <c r="DP5" s="32" t="s">
+        <v>329</v>
+      </c>
     </row>
-    <row r="6" spans="1:112" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:120" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations disablePrompts="1" count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1 L5" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"cartographic,mixed_materials,moving_image,notated_music,software_multimedia,sound_recording,sound_recording_musical,sound_recording_nonmusical,still_image,text"</formula1>
       <formula2>0</formula2>

</xml_diff>

<commit_message>
ANW-2999 address PR review comments
</commit_message>
<xml_diff>
--- a/frontend/public/bulk_import_templates/bulk_import_DO_template.xlsx
+++ b/frontend/public/bulk_import_templates/bulk_import_DO_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zeffmorgan/src/lyrasis/archivesspace/frontend/public/bulk_import_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE98F79A-CF01-AB40-B951-70ED553D211C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A3F0B3C-95CC-324D-BFD6-D75E20C2F837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34560" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="340">
   <si>
     <t>This is the template for use with the bulk_import ("Load SpreadSheet") for importing digital ob jects to associate with archival objects .  You may replace this line with something of your choosing after you've copied the file for your use.</t>
   </si>
@@ -173,9 +173,6 @@
   </si>
   <si>
     <t>Content</t>
-  </si>
-  <si>
-    <t>Agent Type (agent_person/agent_family/agent_corporate_entity)</t>
   </si>
   <si>
     <t>Agent Record ID
@@ -970,10 +967,6 @@
 Duplicate the columns  and increment the index to add more versions.
 file_version_2_*
 file_version_3_*, etc.</t>
-  </si>
-  <si>
-    <t>Agent Type (agent_person/agent_family/agent_corporate_entity)
-Replaces the</t>
   </si>
   <si>
     <t>Event</t>
@@ -1044,78 +1037,6 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> with an explicit Agent Record ID</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>REQUIRED</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> for numeric ID
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">LEAVE BLANK </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>for URI</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Numeric ID or canonical URI
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">MUST </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>be an existing agent</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">
-If all Agent fields are blank, uses the ArchivesSpace software Agent with the `executing_program` role.</t>
     </r>
   </si>
   <si>
@@ -1262,6 +1183,101 @@
   <si>
     <t>Optional. TRUE makes the thumbnail or icon link to this file. Publishes the file version. 
 TRUE/FALSE, YES/NO, Y/N, T/F, 1/0; blank = FALSE.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Numeric ID or canonical URI
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">MUST </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>be an existing agent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+If all Agent fields are blank, uses the ArchivesSpace software Agent with the executing_program role</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>REQUIRED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> for numeric ID
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">LEAVE BLANK </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">for URI
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Accepted:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> person, family, corporate_entity, software</t>
+    </r>
+  </si>
+  <si>
+    <t>Accepted Types: 
+person, family, corporate_entity</t>
   </si>
 </sst>
 </file>
@@ -2107,7 +2123,8 @@
     <col min="37" max="37" width="21.83203125" style="2" customWidth="1"/>
     <col min="38" max="38" width="9.33203125" style="2" customWidth="1"/>
     <col min="39" max="46" width="17.6640625" style="2" customWidth="1"/>
-    <col min="47" max="48" width="9.1640625" style="2" customWidth="1"/>
+    <col min="47" max="47" width="16" style="2" customWidth="1"/>
+    <col min="48" max="48" width="11.33203125" style="2" customWidth="1"/>
     <col min="49" max="49" width="15.1640625" style="2" customWidth="1"/>
     <col min="50" max="50" width="20.1640625" style="2" customWidth="1"/>
     <col min="51" max="51" width="15.33203125" style="2" customWidth="1"/>
@@ -2486,28 +2503,28 @@
         <v>15</v>
       </c>
       <c r="DJ2" s="44" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="DK2" s="45" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="DL2" s="44" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="DM2" s="44" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="DN2" s="44" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="DO2" s="44" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="DP2" s="44" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="DQ2" s="44" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3" spans="1:121" ht="132" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -2587,7 +2604,7 @@
         <v>34</v>
       </c>
       <c r="Z3" s="35" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AA3" s="35" t="s">
         <v>35</v>
@@ -2617,10 +2634,10 @@
         <v>43</v>
       </c>
       <c r="AJ3" s="35" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="AK3" s="35" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="AL3" s="35" t="s">
         <v>44</v>
@@ -2650,959 +2667,959 @@
         <v>48</v>
       </c>
       <c r="AU3" s="23" t="s">
+        <v>339</v>
+      </c>
+      <c r="AV3" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="AV3" s="23" t="s">
+      <c r="AW3" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="AW3" s="23" t="s">
+      <c r="AX3" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="AX3" s="23" t="s">
+      <c r="AY3" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="AY3" s="23" t="s">
+      <c r="AZ3" s="23" t="s">
+        <v>339</v>
+      </c>
+      <c r="BA3" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="BB3" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="BC3" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="BD3" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="BE3" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="AZ3" s="23" t="s">
-        <v>309</v>
-      </c>
-      <c r="BA3" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="BB3" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="BC3" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="BD3" s="23" t="s">
+      <c r="BF3" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="BG3" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="BH3" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="BI3" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="BE3" s="24" t="s">
+      <c r="BJ3" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="BF3" s="24" t="s">
+      <c r="BK3" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="BG3" s="24" t="s">
+      <c r="BL3" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="BH3" s="24" t="s">
+      <c r="BM3" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="BI3" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="BJ3" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="BK3" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="BL3" s="24" t="s">
+      <c r="BN3" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="BO3" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="BP3" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="BQ3" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="BR3" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="BS3" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="BM3" s="20" t="s">
+      <c r="BT3" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="BN3" s="20" t="s">
+      <c r="BU3" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="BO3" s="20" t="s">
+      <c r="BV3" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="BP3" s="21" t="s">
+      <c r="BW3" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="BQ3" s="21" t="s">
+      <c r="BX3" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="BR3" s="43" t="s">
+      <c r="BY3" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="BS3" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="BT3" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="BU3" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="BV3" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="BW3" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="BX3" s="22" t="s">
-        <v>63</v>
-      </c>
-      <c r="BY3" s="37" t="s">
+      <c r="BZ3" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="BZ3" s="37" t="s">
+      <c r="CA3" s="39" t="s">
         <v>65</v>
       </c>
-      <c r="CA3" s="39" t="s">
+      <c r="CB3" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="CC3" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="CD3" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="CB3" s="39" t="s">
+      <c r="CE3" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="CC3" s="39" t="s">
+      <c r="CF3" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="CD3" s="39" t="s">
+      <c r="CG3" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="CE3" s="39" t="s">
+      <c r="CH3" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="CF3" s="39" t="s">
+      <c r="CI3" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="CG3" s="39" t="s">
+      <c r="CJ3" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="CH3" s="39" t="s">
+      <c r="CK3" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="CI3" s="39" t="s">
+      <c r="CL3" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="CJ3" s="39" t="s">
+      <c r="CM3" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="CK3" s="39" t="s">
+      <c r="CN3" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="CL3" s="39" t="s">
+      <c r="CO3" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="CM3" s="39" t="s">
+      <c r="CP3" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="CQ3" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="CN3" s="39" t="s">
+      <c r="CR3" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="CO3" s="39" t="s">
+      <c r="CS3" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="CP3" s="39" t="s">
+      <c r="CT3" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="CQ3" s="39" t="s">
+      <c r="CU3" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="CV3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="CR3" s="39" t="s">
-        <v>71</v>
-      </c>
-      <c r="CS3" s="39" t="s">
-        <v>71</v>
-      </c>
-      <c r="CT3" s="39" t="s">
-        <v>71</v>
-      </c>
-      <c r="CU3" s="39" t="s">
-        <v>71</v>
-      </c>
-      <c r="CV3" s="39" t="s">
+      <c r="CW3" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="CW3" s="39" t="s">
+      <c r="CX3" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="CX3" s="39" t="s">
+      <c r="CY3" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="CY3" s="39" t="s">
+      <c r="CZ3" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="CZ3" s="25" t="s">
+      <c r="DA3" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="DA3" s="25" t="s">
+      <c r="DB3" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="DB3" s="25" t="s">
+      <c r="DC3" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="DC3" s="25" t="s">
+      <c r="DD3" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="DD3" s="25" t="s">
+      <c r="DE3" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="DE3" s="25" t="s">
+      <c r="DF3" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="DF3" s="25" t="s">
+      <c r="DG3" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="DG3" s="25" t="s">
+      <c r="DH3" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="DH3" s="25" t="s">
+      <c r="DI3" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="DI3" s="25" t="s">
-        <v>85</v>
-      </c>
       <c r="DJ3" s="46" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="DK3" s="47" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="DL3" s="48" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="DM3" s="48" t="s">
+        <v>326</v>
+      </c>
+      <c r="DN3" s="48" t="s">
         <v>330</v>
       </c>
-      <c r="DN3" s="48" t="s">
-        <v>334</v>
-      </c>
       <c r="DO3" s="48" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="DP3" s="46" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="DQ3" s="46" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" spans="1:121" s="27" customFormat="1" ht="41.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="40" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="C4" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="D4" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="E4" s="27" t="s">
         <v>89</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="F4" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="G4" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="H4" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="I4" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="I4" s="27" t="s">
+      <c r="J4" s="27" t="s">
         <v>94</v>
       </c>
-      <c r="J4" s="27" t="s">
+      <c r="K4" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="K4" s="27" t="s">
+      <c r="L4" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="L4" s="27" t="s">
+      <c r="M4" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="M4" s="27" t="s">
+      <c r="N4" s="27" t="s">
         <v>98</v>
       </c>
-      <c r="N4" s="27" t="s">
+      <c r="O4" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="P4" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="P4" s="28" t="s">
+      <c r="Q4" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="Q4" s="27" t="s">
+      <c r="R4" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="R4" s="28" t="s">
+      <c r="S4" s="27" t="s">
         <v>103</v>
       </c>
-      <c r="S4" s="27" t="s">
+      <c r="T4" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="T4" s="27" t="s">
+      <c r="U4" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="U4" s="28" t="s">
+      <c r="V4" s="28" t="s">
         <v>106</v>
       </c>
-      <c r="V4" s="28" t="s">
+      <c r="W4" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="W4" s="27" t="s">
+      <c r="X4" s="28" t="s">
         <v>108</v>
       </c>
-      <c r="X4" s="28" t="s">
+      <c r="Y4" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="Y4" s="27" t="s">
+      <c r="Z4" s="27" t="s">
         <v>110</v>
       </c>
-      <c r="Z4" s="27" t="s">
+      <c r="AA4" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="AA4" s="27" t="s">
+      <c r="AB4" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="AB4" s="27" t="s">
+      <c r="AC4" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="AC4" s="27" t="s">
+      <c r="AD4" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="AD4" s="27" t="s">
+      <c r="AE4" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="AE4" s="27" t="s">
+      <c r="AF4" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="AF4" s="27" t="s">
+      <c r="AG4" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="AG4" s="27" t="s">
+      <c r="AH4" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="AH4" s="27" t="s">
+      <c r="AI4" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="AI4" s="27" t="s">
+      <c r="AJ4" s="27" t="s">
+        <v>331</v>
+      </c>
+      <c r="AK4" s="27" t="s">
+        <v>332</v>
+      </c>
+      <c r="AL4" s="27" t="s">
         <v>120</v>
       </c>
-      <c r="AJ4" s="27" t="s">
-        <v>335</v>
-      </c>
-      <c r="AK4" s="27" t="s">
-        <v>336</v>
-      </c>
-      <c r="AL4" s="27" t="s">
+      <c r="AM4" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="AM4" s="27" t="s">
+      <c r="AN4" s="27" t="s">
         <v>122</v>
       </c>
-      <c r="AN4" s="27" t="s">
+      <c r="AO4" s="27" t="s">
         <v>123</v>
       </c>
-      <c r="AO4" s="27" t="s">
+      <c r="AP4" s="27" t="s">
         <v>124</v>
       </c>
-      <c r="AP4" s="27" t="s">
+      <c r="AQ4" s="27" t="s">
         <v>125</v>
       </c>
-      <c r="AQ4" s="27" t="s">
+      <c r="AR4" s="27" t="s">
         <v>126</v>
       </c>
-      <c r="AR4" s="27" t="s">
+      <c r="AS4" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="AS4" s="27" t="s">
+      <c r="AT4" s="27" t="s">
         <v>128</v>
       </c>
-      <c r="AT4" s="27" t="s">
+      <c r="AU4" s="27" t="s">
         <v>129</v>
       </c>
-      <c r="AU4" s="27" t="s">
+      <c r="AV4" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="AV4" s="27" t="s">
+      <c r="AW4" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="AW4" s="27" t="s">
+      <c r="AX4" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="AX4" s="27" t="s">
+      <c r="AY4" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="AY4" s="27" t="s">
+      <c r="AZ4" s="27" t="s">
         <v>134</v>
       </c>
-      <c r="AZ4" s="27" t="s">
+      <c r="BA4" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="BA4" s="27" t="s">
+      <c r="BB4" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="BB4" s="27" t="s">
+      <c r="BC4" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="BC4" s="27" t="s">
+      <c r="BD4" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="BD4" s="27" t="s">
+      <c r="BE4" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="BE4" s="27" t="s">
+      <c r="BF4" s="27" t="s">
         <v>140</v>
       </c>
-      <c r="BF4" s="27" t="s">
+      <c r="BG4" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="BG4" s="27" t="s">
+      <c r="BH4" s="27" t="s">
         <v>142</v>
       </c>
-      <c r="BH4" s="27" t="s">
+      <c r="BI4" s="27" t="s">
         <v>143</v>
       </c>
-      <c r="BI4" s="27" t="s">
+      <c r="BJ4" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="BJ4" s="27" t="s">
+      <c r="BK4" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="BK4" s="27" t="s">
+      <c r="BL4" s="27" t="s">
         <v>146</v>
       </c>
-      <c r="BL4" s="27" t="s">
+      <c r="BM4" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="BM4" s="27" t="s">
+      <c r="BN4" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="BN4" s="27" t="s">
+      <c r="BO4" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="BO4" s="27" t="s">
+      <c r="BP4" s="27" t="s">
         <v>150</v>
       </c>
-      <c r="BP4" s="27" t="s">
+      <c r="BQ4" s="27" t="s">
         <v>151</v>
       </c>
-      <c r="BQ4" s="27" t="s">
+      <c r="BR4" s="29" t="s">
         <v>152</v>
       </c>
-      <c r="BR4" s="29" t="s">
+      <c r="BS4" s="27" t="s">
         <v>153</v>
       </c>
-      <c r="BS4" s="27" t="s">
+      <c r="BT4" s="27" t="s">
         <v>154</v>
       </c>
-      <c r="BT4" s="27" t="s">
+      <c r="BU4" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="BU4" s="27" t="s">
+      <c r="BV4" s="27" t="s">
         <v>156</v>
       </c>
-      <c r="BV4" s="27" t="s">
+      <c r="BW4" s="27" t="s">
         <v>157</v>
       </c>
-      <c r="BW4" s="27" t="s">
+      <c r="BX4" s="42" t="s">
         <v>158</v>
       </c>
-      <c r="BX4" s="42" t="s">
+      <c r="BY4" s="27" t="s">
         <v>159</v>
       </c>
-      <c r="BY4" s="27" t="s">
+      <c r="BZ4" s="27" t="s">
         <v>160</v>
       </c>
-      <c r="BZ4" s="27" t="s">
+      <c r="CA4" s="27" t="s">
         <v>161</v>
       </c>
-      <c r="CA4" s="27" t="s">
+      <c r="CB4" s="27" t="s">
         <v>162</v>
       </c>
-      <c r="CB4" s="27" t="s">
+      <c r="CC4" s="27" t="s">
         <v>163</v>
       </c>
-      <c r="CC4" s="27" t="s">
+      <c r="CD4" s="27" t="s">
         <v>164</v>
       </c>
-      <c r="CD4" s="27" t="s">
+      <c r="CE4" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="CE4" s="27" t="s">
+      <c r="CF4" s="27" t="s">
         <v>166</v>
       </c>
-      <c r="CF4" s="27" t="s">
+      <c r="CG4" s="27" t="s">
         <v>167</v>
       </c>
-      <c r="CG4" s="27" t="s">
+      <c r="CH4" s="27" t="s">
         <v>168</v>
       </c>
-      <c r="CH4" s="27" t="s">
+      <c r="CI4" s="27" t="s">
         <v>169</v>
       </c>
-      <c r="CI4" s="27" t="s">
+      <c r="CJ4" s="27" t="s">
         <v>170</v>
       </c>
-      <c r="CJ4" s="27" t="s">
+      <c r="CK4" s="27" t="s">
         <v>171</v>
       </c>
-      <c r="CK4" s="27" t="s">
+      <c r="CL4" s="27" t="s">
         <v>172</v>
       </c>
-      <c r="CL4" s="27" t="s">
+      <c r="CM4" s="27" t="s">
         <v>173</v>
       </c>
-      <c r="CM4" s="27" t="s">
+      <c r="CN4" s="27" t="s">
         <v>174</v>
       </c>
-      <c r="CN4" s="27" t="s">
+      <c r="CO4" s="27" t="s">
         <v>175</v>
       </c>
-      <c r="CO4" s="27" t="s">
+      <c r="CP4" s="27" t="s">
         <v>176</v>
       </c>
-      <c r="CP4" s="27" t="s">
+      <c r="CQ4" s="27" t="s">
         <v>177</v>
       </c>
-      <c r="CQ4" s="27" t="s">
+      <c r="CR4" s="27" t="s">
         <v>178</v>
       </c>
-      <c r="CR4" s="27" t="s">
+      <c r="CS4" s="27" t="s">
         <v>179</v>
       </c>
-      <c r="CS4" s="27" t="s">
+      <c r="CT4" s="27" t="s">
         <v>180</v>
       </c>
-      <c r="CT4" s="27" t="s">
+      <c r="CU4" s="27" t="s">
         <v>181</v>
       </c>
-      <c r="CU4" s="27" t="s">
+      <c r="CV4" s="27" t="s">
         <v>182</v>
       </c>
-      <c r="CV4" s="27" t="s">
+      <c r="CW4" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="CW4" s="27" t="s">
+      <c r="CX4" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="CX4" s="27" t="s">
+      <c r="CY4" s="27" t="s">
         <v>185</v>
       </c>
-      <c r="CY4" s="27" t="s">
+      <c r="CZ4" s="27" t="s">
         <v>186</v>
       </c>
-      <c r="CZ4" s="27" t="s">
+      <c r="DA4" s="27" t="s">
         <v>187</v>
       </c>
-      <c r="DA4" s="27" t="s">
+      <c r="DB4" s="27" t="s">
         <v>188</v>
       </c>
-      <c r="DB4" s="27" t="s">
+      <c r="DC4" s="27" t="s">
         <v>189</v>
       </c>
-      <c r="DC4" s="27" t="s">
+      <c r="DD4" s="27" t="s">
         <v>190</v>
       </c>
-      <c r="DD4" s="27" t="s">
+      <c r="DE4" s="27" t="s">
         <v>191</v>
       </c>
-      <c r="DE4" s="27" t="s">
+      <c r="DF4" s="27" t="s">
         <v>192</v>
       </c>
-      <c r="DF4" s="27" t="s">
+      <c r="DG4" s="27" t="s">
         <v>193</v>
       </c>
-      <c r="DG4" s="27" t="s">
+      <c r="DH4" s="27" t="s">
         <v>194</v>
       </c>
-      <c r="DH4" s="27" t="s">
+      <c r="DI4" s="27" t="s">
         <v>195</v>
       </c>
-      <c r="DI4" s="27" t="s">
-        <v>196</v>
-      </c>
       <c r="DJ4" s="27" t="s">
+        <v>309</v>
+      </c>
+      <c r="DK4" s="28" t="s">
+        <v>310</v>
+      </c>
+      <c r="DL4" s="27" t="s">
         <v>311</v>
       </c>
-      <c r="DK4" s="28" t="s">
+      <c r="DM4" s="27" t="s">
         <v>312</v>
       </c>
-      <c r="DL4" s="27" t="s">
+      <c r="DN4" s="27" t="s">
         <v>313</v>
       </c>
-      <c r="DM4" s="27" t="s">
+      <c r="DO4" s="27" t="s">
         <v>314</v>
       </c>
-      <c r="DN4" s="27" t="s">
+      <c r="DP4" s="27" t="s">
         <v>315</v>
       </c>
-      <c r="DO4" s="27" t="s">
+      <c r="DQ4" s="27" t="s">
         <v>316</v>
-      </c>
-      <c r="DP4" s="27" t="s">
-        <v>317</v>
-      </c>
-      <c r="DQ4" s="27" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="5" spans="1:121" ht="82" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
+        <v>196</v>
+      </c>
+      <c r="B5" s="41" t="s">
         <v>197</v>
       </c>
-      <c r="B5" s="41" t="s">
+      <c r="C5" s="31" t="s">
         <v>198</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="D5" s="32" t="s">
         <v>199</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="E5" s="31" t="s">
         <v>200</v>
       </c>
-      <c r="E5" s="31" t="s">
+      <c r="F5" s="31" t="s">
         <v>201</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="G5" s="31" t="s">
         <v>202</v>
       </c>
-      <c r="G5" s="31" t="s">
+      <c r="H5" s="32" t="s">
         <v>203</v>
       </c>
-      <c r="H5" s="32" t="s">
+      <c r="I5" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="I5" s="32" t="s">
+      <c r="J5" s="32" t="s">
         <v>205</v>
       </c>
-      <c r="J5" s="32" t="s">
+      <c r="K5" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="K5" s="32" t="s">
+      <c r="L5" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="L5" s="32" t="s">
+      <c r="M5" s="32" t="s">
         <v>208</v>
       </c>
-      <c r="M5" s="32" t="s">
+      <c r="N5" s="32" t="s">
         <v>209</v>
       </c>
-      <c r="N5" s="32" t="s">
+      <c r="O5" s="33" t="s">
         <v>210</v>
       </c>
-      <c r="O5" s="33" t="s">
+      <c r="P5" s="33" t="s">
         <v>211</v>
       </c>
-      <c r="P5" s="33" t="s">
+      <c r="Q5" s="31" t="s">
         <v>212</v>
       </c>
-      <c r="Q5" s="31" t="s">
+      <c r="R5" s="33" t="s">
         <v>213</v>
       </c>
-      <c r="R5" s="33" t="s">
+      <c r="S5" s="32" t="s">
         <v>214</v>
       </c>
-      <c r="S5" s="32" t="s">
+      <c r="T5" s="32" t="s">
         <v>215</v>
       </c>
-      <c r="T5" s="32" t="s">
+      <c r="U5" s="33" t="s">
         <v>216</v>
       </c>
-      <c r="U5" s="33" t="s">
+      <c r="V5" s="33" t="s">
         <v>217</v>
       </c>
-      <c r="V5" s="33" t="s">
+      <c r="W5" s="31" t="s">
         <v>218</v>
       </c>
-      <c r="W5" s="31" t="s">
+      <c r="X5" s="33" t="s">
         <v>219</v>
       </c>
-      <c r="X5" s="33" t="s">
+      <c r="Y5" s="32" t="s">
         <v>220</v>
       </c>
-      <c r="Y5" s="32" t="s">
+      <c r="Z5" s="32" t="s">
         <v>221</v>
       </c>
-      <c r="Z5" s="32" t="s">
+      <c r="AA5" s="32" t="s">
         <v>222</v>
       </c>
-      <c r="AA5" s="32" t="s">
+      <c r="AB5" s="32" t="s">
         <v>223</v>
       </c>
-      <c r="AB5" s="32" t="s">
+      <c r="AC5" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="AC5" s="32" t="s">
+      <c r="AD5" s="32" t="s">
         <v>225</v>
       </c>
-      <c r="AD5" s="32" t="s">
+      <c r="AE5" s="32" t="s">
         <v>226</v>
       </c>
-      <c r="AE5" s="32" t="s">
+      <c r="AF5" s="32" t="s">
         <v>227</v>
       </c>
-      <c r="AF5" s="32" t="s">
+      <c r="AG5" s="32" t="s">
         <v>228</v>
       </c>
-      <c r="AG5" s="32" t="s">
+      <c r="AH5" s="32" t="s">
         <v>229</v>
       </c>
-      <c r="AH5" s="32" t="s">
+      <c r="AI5" s="32" t="s">
         <v>230</v>
       </c>
-      <c r="AI5" s="32" t="s">
+      <c r="AJ5" s="32" t="s">
+        <v>333</v>
+      </c>
+      <c r="AK5" s="32" t="s">
+        <v>334</v>
+      </c>
+      <c r="AL5" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="AJ5" s="32" t="s">
-        <v>337</v>
-      </c>
-      <c r="AK5" s="32" t="s">
-        <v>338</v>
-      </c>
-      <c r="AL5" s="32" t="s">
+      <c r="AM5" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="AM5" s="32" t="s">
+      <c r="AN5" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="AN5" s="32" t="s">
+      <c r="AO5" s="32" t="s">
         <v>234</v>
       </c>
-      <c r="AO5" s="32" t="s">
+      <c r="AP5" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="AP5" s="32" t="s">
+      <c r="AQ5" s="32" t="s">
         <v>236</v>
       </c>
-      <c r="AQ5" s="32" t="s">
+      <c r="AR5" s="32" t="s">
         <v>237</v>
       </c>
-      <c r="AR5" s="32" t="s">
+      <c r="AS5" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="AS5" s="32" t="s">
+      <c r="AT5" s="32" t="s">
         <v>239</v>
       </c>
-      <c r="AT5" s="32" t="s">
+      <c r="AU5" s="32" t="s">
         <v>240</v>
       </c>
-      <c r="AU5" s="32" t="s">
+      <c r="AV5" s="32" t="s">
         <v>241</v>
       </c>
-      <c r="AV5" s="32" t="s">
+      <c r="AW5" s="32" t="s">
         <v>242</v>
       </c>
-      <c r="AW5" s="32" t="s">
+      <c r="AX5" s="32" t="s">
         <v>243</v>
       </c>
-      <c r="AX5" s="32" t="s">
+      <c r="AY5" s="32" t="s">
         <v>244</v>
       </c>
-      <c r="AY5" s="32" t="s">
+      <c r="AZ5" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="AZ5" s="32" t="s">
+      <c r="BA5" s="32" t="s">
         <v>246</v>
       </c>
-      <c r="BA5" s="32" t="s">
+      <c r="BB5" s="32" t="s">
         <v>247</v>
       </c>
-      <c r="BB5" s="32" t="s">
+      <c r="BC5" s="32" t="s">
         <v>248</v>
       </c>
-      <c r="BC5" s="32" t="s">
+      <c r="BD5" s="32" t="s">
         <v>249</v>
       </c>
-      <c r="BD5" s="32" t="s">
+      <c r="BE5" s="32" t="s">
         <v>250</v>
       </c>
-      <c r="BE5" s="32" t="s">
+      <c r="BF5" s="32" t="s">
         <v>251</v>
       </c>
-      <c r="BF5" s="32" t="s">
+      <c r="BG5" s="32" t="s">
         <v>252</v>
       </c>
-      <c r="BG5" s="32" t="s">
+      <c r="BH5" s="32" t="s">
         <v>253</v>
       </c>
-      <c r="BH5" s="32" t="s">
+      <c r="BI5" s="32" t="s">
         <v>254</v>
       </c>
-      <c r="BI5" s="32" t="s">
+      <c r="BJ5" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="BJ5" s="32" t="s">
+      <c r="BK5" s="32" t="s">
         <v>256</v>
       </c>
-      <c r="BK5" s="32" t="s">
+      <c r="BL5" s="32" t="s">
         <v>257</v>
       </c>
-      <c r="BL5" s="32" t="s">
+      <c r="BM5" s="32" t="s">
         <v>258</v>
       </c>
-      <c r="BM5" s="32" t="s">
+      <c r="BN5" s="31" t="s">
         <v>259</v>
       </c>
-      <c r="BN5" s="31" t="s">
+      <c r="BO5" s="31" t="s">
         <v>260</v>
       </c>
-      <c r="BO5" s="31" t="s">
+      <c r="BP5" s="32" t="s">
         <v>261</v>
       </c>
-      <c r="BP5" s="32" t="s">
+      <c r="BQ5" s="32" t="s">
         <v>262</v>
       </c>
-      <c r="BQ5" s="32" t="s">
+      <c r="BR5" s="32" t="s">
         <v>263</v>
       </c>
-      <c r="BR5" s="32" t="s">
+      <c r="BS5" s="32" t="s">
         <v>264</v>
       </c>
-      <c r="BS5" s="32" t="s">
+      <c r="BT5" s="31" t="s">
         <v>265</v>
       </c>
-      <c r="BT5" s="31" t="s">
+      <c r="BU5" s="31" t="s">
         <v>266</v>
       </c>
-      <c r="BU5" s="31" t="s">
+      <c r="BV5" s="32" t="s">
         <v>267</v>
       </c>
-      <c r="BV5" s="32" t="s">
+      <c r="BW5" s="32" t="s">
         <v>268</v>
       </c>
-      <c r="BW5" s="32" t="s">
+      <c r="BX5" s="32" t="s">
         <v>269</v>
       </c>
-      <c r="BX5" s="32" t="s">
+      <c r="BY5" s="32" t="s">
         <v>270</v>
       </c>
-      <c r="BY5" s="32" t="s">
+      <c r="BZ5" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="BZ5" s="32" t="s">
+      <c r="CA5" s="32" t="s">
         <v>272</v>
       </c>
-      <c r="CA5" s="32" t="s">
+      <c r="CB5" s="32" t="s">
         <v>273</v>
       </c>
-      <c r="CB5" s="32" t="s">
+      <c r="CC5" s="32" t="s">
         <v>274</v>
       </c>
-      <c r="CC5" s="32" t="s">
+      <c r="CD5" s="32" t="s">
         <v>275</v>
       </c>
-      <c r="CD5" s="32" t="s">
+      <c r="CE5" s="32" t="s">
         <v>276</v>
       </c>
-      <c r="CE5" s="32" t="s">
+      <c r="CF5" s="32" t="s">
         <v>277</v>
       </c>
-      <c r="CF5" s="32" t="s">
+      <c r="CG5" s="32" t="s">
         <v>278</v>
       </c>
-      <c r="CG5" s="32" t="s">
+      <c r="CH5" s="32" t="s">
         <v>279</v>
       </c>
-      <c r="CH5" s="32" t="s">
+      <c r="CI5" s="32" t="s">
         <v>280</v>
       </c>
-      <c r="CI5" s="32" t="s">
+      <c r="CJ5" s="32" t="s">
         <v>281</v>
       </c>
-      <c r="CJ5" s="32" t="s">
+      <c r="CK5" s="32" t="s">
         <v>282</v>
       </c>
-      <c r="CK5" s="32" t="s">
+      <c r="CL5" s="32" t="s">
         <v>283</v>
       </c>
-      <c r="CL5" s="32" t="s">
+      <c r="CM5" s="32" t="s">
         <v>284</v>
       </c>
-      <c r="CM5" s="32" t="s">
+      <c r="CN5" s="32" t="s">
         <v>285</v>
       </c>
-      <c r="CN5" s="32" t="s">
+      <c r="CO5" s="32" t="s">
         <v>286</v>
       </c>
-      <c r="CO5" s="32" t="s">
+      <c r="CP5" s="32" t="s">
         <v>287</v>
       </c>
-      <c r="CP5" s="32" t="s">
+      <c r="CQ5" s="32" t="s">
         <v>288</v>
       </c>
-      <c r="CQ5" s="32" t="s">
+      <c r="CR5" s="32" t="s">
         <v>289</v>
       </c>
-      <c r="CR5" s="32" t="s">
+      <c r="CS5" s="32" t="s">
         <v>290</v>
       </c>
-      <c r="CS5" s="32" t="s">
+      <c r="CT5" s="32" t="s">
         <v>291</v>
       </c>
-      <c r="CT5" s="32" t="s">
+      <c r="CU5" s="32" t="s">
         <v>292</v>
       </c>
-      <c r="CU5" s="32" t="s">
+      <c r="CV5" s="32" t="s">
         <v>293</v>
       </c>
-      <c r="CV5" s="32" t="s">
+      <c r="CW5" s="32" t="s">
         <v>294</v>
       </c>
-      <c r="CW5" s="32" t="s">
+      <c r="CX5" s="32" t="s">
         <v>295</v>
       </c>
-      <c r="CX5" s="32" t="s">
+      <c r="CY5" s="32" t="s">
         <v>296</v>
       </c>
-      <c r="CY5" s="32" t="s">
+      <c r="CZ5" s="32" t="s">
         <v>297</v>
       </c>
-      <c r="CZ5" s="32" t="s">
+      <c r="DA5" s="32" t="s">
         <v>298</v>
       </c>
-      <c r="DA5" s="32" t="s">
+      <c r="DB5" s="32" t="s">
         <v>299</v>
       </c>
-      <c r="DB5" s="32" t="s">
+      <c r="DC5" s="32" t="s">
         <v>300</v>
       </c>
-      <c r="DC5" s="32" t="s">
+      <c r="DD5" s="32" t="s">
         <v>301</v>
       </c>
-      <c r="DD5" s="32" t="s">
+      <c r="DE5" s="32" t="s">
         <v>302</v>
       </c>
-      <c r="DE5" s="32" t="s">
+      <c r="DF5" s="32" t="s">
         <v>303</v>
       </c>
-      <c r="DF5" s="32" t="s">
+      <c r="DG5" s="32" t="s">
         <v>304</v>
       </c>
-      <c r="DG5" s="32" t="s">
+      <c r="DH5" s="32" t="s">
         <v>305</v>
       </c>
-      <c r="DH5" s="32" t="s">
+      <c r="DI5" s="32" t="s">
         <v>306</v>
       </c>
-      <c r="DI5" s="32" t="s">
-        <v>307</v>
-      </c>
       <c r="DJ5" s="32" t="s">
+        <v>319</v>
+      </c>
+      <c r="DK5" s="33" t="s">
+        <v>320</v>
+      </c>
+      <c r="DL5" s="32" t="s">
         <v>321</v>
       </c>
-      <c r="DK5" s="33" t="s">
+      <c r="DM5" s="32" t="s">
+        <v>317</v>
+      </c>
+      <c r="DN5" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="DO5" s="32" t="s">
         <v>322</v>
       </c>
-      <c r="DL5" s="32" t="s">
+      <c r="DP5" s="32" t="s">
         <v>323</v>
       </c>
-      <c r="DM5" s="32" t="s">
-        <v>319</v>
-      </c>
-      <c r="DN5" s="32" t="s">
-        <v>320</v>
-      </c>
-      <c r="DO5" s="32" t="s">
+      <c r="DQ5" s="32" t="s">
         <v>324</v>
-      </c>
-      <c r="DP5" s="32" t="s">
-        <v>325</v>
-      </c>
-      <c r="DQ5" s="32" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="6" spans="1:121" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
ANW-2999 Add validated BDO Events to bulk import (#4321)
* ANW-2999 Add validated BDO Events to bulk import

Planning-assisted-by: Codex [GPT-5.6 Sol]
Code-assisted-by: Codex [GPT-5.6 Sol]
Tests-coauthored-by: Grok [Grok 4.7]

* ANW-2999 fix validate only path

* ANW-2999 fix event URI saved

* ANW-2999 apply performance suggestion

* ANW-2999 apply Agent type vocabulary suggestion

* ANW-2999 address PR review comments

* small performance fix: do not reload the controlled value list every time a value is looked up

---------

Co-authored-by: Thimios <thimios.dimopulos@lyrasis.org>
</commit_message>
<xml_diff>
--- a/frontend/public/bulk_import_templates/bulk_import_DO_template.xlsx
+++ b/frontend/public/bulk_import_templates/bulk_import_DO_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zeffmorgan/src/lyrasis/archivesspace/frontend/public/bulk_import_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6626C96-CED2-3646-9CBC-6C76BAC05211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A3F0B3C-95CC-324D-BFD6-D75E20C2F837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34560" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="340">
   <si>
     <t>This is the template for use with the bulk_import ("Load SpreadSheet") for importing digital ob jects to associate with archival objects .  You may replace this line with something of your choosing after you've copied the file for your use.</t>
   </si>
@@ -173,9 +173,6 @@
   </si>
   <si>
     <t>Content</t>
-  </si>
-  <si>
-    <t>Agent Type (agent_person/agent_family/agent_corporate_entity)</t>
   </si>
   <si>
     <t>Agent Record ID
@@ -972,33 +969,322 @@
 file_version_3_*, etc.</t>
   </si>
   <si>
-    <t>Agent Type (agent_person/agent_family/agent_corporate_entity)
-Replaces the</t>
-  </si>
-  <si>
-    <t>Make Display Thumbnail?</t>
+    <t>Event</t>
+  </si>
+  <si>
+    <t>event_1_type</t>
+  </si>
+  <si>
+    <t>event_1_date</t>
+  </si>
+  <si>
+    <t>event_1_date_label</t>
+  </si>
+  <si>
+    <t>event_1_outcome</t>
+  </si>
+  <si>
+    <t>event_1_outcome_note</t>
+  </si>
+  <si>
+    <t>event_1_agent_1_record_id</t>
+  </si>
+  <si>
+    <t>event_1_agent_1_agent_type</t>
+  </si>
+  <si>
+    <t>event_1_agent_1_role</t>
+  </si>
+  <si>
+    <t>Event(1) Outcome</t>
+  </si>
+  <si>
+    <t>Event(1) Outcome Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event(1) Type </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event(1) Date </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event(1) Date Label </t>
+  </si>
+  <si>
+    <t>Event(1) Agent(1) Record ID</t>
+  </si>
+  <si>
+    <t>Event(1) Agent(1) Type</t>
+  </si>
+  <si>
+    <t>Event(1) Agent(1) Role</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>REQUIRED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> with an explicit Agent Record ID</t>
+    </r>
+  </si>
+  <si>
+    <t>Event outcome (installation-wide controlled value; optional)
+Example: pass</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>REQUIRED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> if specifying Event
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+YYYY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>YYYY-MM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, or </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>YYYY-MM-DD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> e</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>ntered as text.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Excel can convert partial dates into numeric dates, losing the intended precision and causing an import error.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>REQUIRED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> if specifying Event
+Installation-wide controlled value. 
+Example: cataloged</t>
+    </r>
+  </si>
+  <si>
+    <t>Installation-wide controlled value. When a Date is supplied without a Date Label, ArchivesSpace stores 'other'.</t>
+  </si>
+  <si>
+    <t>Additional information about the event outcome (free text; optional; may be supplied without an Outcome)</t>
   </si>
   <si>
     <t>file_version_1_is_display_thumbnail</t>
   </si>
   <si>
+    <t>file_version_1_is_display_link</t>
+  </si>
+  <si>
     <t>File Version(1) Make Display Thumbnail</t>
   </si>
   <si>
-    <t>Make Display Link?</t>
-  </si>
-  <si>
-    <t>file_version_1_is_display_link</t>
-  </si>
-  <si>
     <t>File Version(1) Make Display Link</t>
+  </si>
+  <si>
+    <t>Optional. TRUE shows this file as the Digital Object's thumbnail (generic icon if it can't display). Publishes the file version. 
+TRUE/FALSE, YES/NO, Y/N, T/F, 1/0; blank = FALSE.</t>
+  </si>
+  <si>
+    <t>Optional. TRUE makes the thumbnail or icon link to this file. Publishes the file version. 
+TRUE/FALSE, YES/NO, Y/N, T/F, 1/0; blank = FALSE.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Numeric ID or canonical URI
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">MUST </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>be an existing agent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+If all Agent fields are blank, uses the ArchivesSpace software Agent with the executing_program role</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>REQUIRED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> for numeric ID
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">LEAVE BLANK </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">for URI
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Accepted:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> person, family, corporate_entity, software</t>
+    </r>
+  </si>
+  <si>
+    <t>Accepted Types: 
+person, family, corporate_entity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1064,8 +1350,19 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1129,6 +1426,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE8DDF2"/>
+        <bgColor rgb="FFE6E0EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor rgb="FFDCE6F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF2DF"/>
+        <bgColor rgb="FFFDEADA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF2DF"/>
         <bgColor rgb="FFE6E0EC"/>
       </patternFill>
     </fill>
@@ -1215,7 +1530,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1305,9 +1620,6 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1345,6 +1657,30 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1419,6 +1755,9 @@
       <rgbColor rgb="00333399"/>
       <rgbColor rgb="00333333"/>
     </indexedColors>
+    <mruColors>
+      <color rgb="FFEBF2DF"/>
+    </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1748,7 +2087,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DI6"/>
+  <dimension ref="A1:DQ6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.33203125" style="1" customWidth="1"/>
@@ -1780,11 +2119,12 @@
     <col min="31" max="33" width="9.33203125" style="2" customWidth="1"/>
     <col min="34" max="34" width="10.1640625" style="2" customWidth="1"/>
     <col min="35" max="35" width="9.33203125" style="2" customWidth="1"/>
-    <col min="36" max="36" width="14" style="2" customWidth="1"/>
-    <col min="37" max="37" width="14" style="2" customWidth="1"/>
+    <col min="36" max="36" width="24" style="2" customWidth="1"/>
+    <col min="37" max="37" width="21.83203125" style="2" customWidth="1"/>
     <col min="38" max="38" width="9.33203125" style="2" customWidth="1"/>
     <col min="39" max="46" width="17.6640625" style="2" customWidth="1"/>
-    <col min="47" max="48" width="9.1640625" style="2" customWidth="1"/>
+    <col min="47" max="47" width="16" style="2" customWidth="1"/>
+    <col min="48" max="48" width="11.33203125" style="2" customWidth="1"/>
     <col min="49" max="49" width="15.1640625" style="2" customWidth="1"/>
     <col min="50" max="50" width="20.1640625" style="2" customWidth="1"/>
     <col min="51" max="51" width="15.33203125" style="2" customWidth="1"/>
@@ -1810,16 +2150,19 @@
     <col min="108" max="108" width="17.33203125" style="2" customWidth="1"/>
     <col min="109" max="112" width="16" style="2" customWidth="1"/>
     <col min="113" max="113" width="13.5" style="2" customWidth="1"/>
+    <col min="114" max="114" width="21.5" style="2" customWidth="1"/>
+    <col min="115" max="115" width="21.5" style="3" customWidth="1"/>
+    <col min="116" max="121" width="21.5" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:113" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:121" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="BH1" s="2"/>
       <c r="BK1" s="2"/>
     </row>
-    <row r="2" spans="1:113" s="2" customFormat="1" ht="41.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:121" s="2" customFormat="1" ht="41.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1895,43 +2238,43 @@
       <c r="Y2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="Z2" s="35" t="s">
+      <c r="Z2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AA2" s="35" t="s">
+      <c r="AA2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AB2" s="35" t="s">
+      <c r="AB2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AC2" s="35" t="s">
+      <c r="AC2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AD2" s="35" t="s">
+      <c r="AD2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AE2" s="35" t="s">
+      <c r="AE2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AF2" s="35" t="s">
+      <c r="AF2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AG2" s="35" t="s">
+      <c r="AG2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AH2" s="35" t="s">
+      <c r="AH2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AI2" s="35" t="s">
+      <c r="AI2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AJ2" s="35" t="s">
+      <c r="AJ2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AK2" s="35" t="s">
+      <c r="AK2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AL2" s="35" t="s">
+      <c r="AL2" s="34" t="s">
         <v>5</v>
       </c>
       <c r="AM2" s="12" t="s">
@@ -2048,85 +2391,85 @@
       <c r="BX2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="BY2" s="37" t="s">
+      <c r="BY2" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="BZ2" s="37" t="s">
+      <c r="BZ2" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="CA2" s="39" t="s">
+      <c r="CA2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CB2" s="39" t="s">
+      <c r="CB2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CC2" s="39" t="s">
+      <c r="CC2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CD2" s="39" t="s">
+      <c r="CD2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CE2" s="39" t="s">
+      <c r="CE2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CF2" s="39" t="s">
+      <c r="CF2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CG2" s="39" t="s">
+      <c r="CG2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CH2" s="39" t="s">
+      <c r="CH2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CI2" s="39" t="s">
+      <c r="CI2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CJ2" s="39" t="s">
+      <c r="CJ2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CK2" s="39" t="s">
+      <c r="CK2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CL2" s="39" t="s">
+      <c r="CL2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CM2" s="39" t="s">
+      <c r="CM2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CN2" s="39" t="s">
+      <c r="CN2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CO2" s="39" t="s">
+      <c r="CO2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CP2" s="39" t="s">
+      <c r="CP2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CQ2" s="39" t="s">
+      <c r="CQ2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CR2" s="39" t="s">
+      <c r="CR2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CS2" s="39" t="s">
+      <c r="CS2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CT2" s="39" t="s">
+      <c r="CT2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CU2" s="39" t="s">
+      <c r="CU2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CV2" s="39" t="s">
+      <c r="CV2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CW2" s="39" t="s">
+      <c r="CW2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CX2" s="39" t="s">
+      <c r="CX2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CY2" s="39" t="s">
+      <c r="CY2" s="38" t="s">
         <v>14</v>
       </c>
       <c r="CZ2" s="12" t="s">
@@ -2159,8 +2502,32 @@
       <c r="DI2" s="12" t="s">
         <v>15</v>
       </c>
+      <c r="DJ2" s="44" t="s">
+        <v>308</v>
+      </c>
+      <c r="DK2" s="45" t="s">
+        <v>308</v>
+      </c>
+      <c r="DL2" s="44" t="s">
+        <v>308</v>
+      </c>
+      <c r="DM2" s="44" t="s">
+        <v>308</v>
+      </c>
+      <c r="DN2" s="44" t="s">
+        <v>308</v>
+      </c>
+      <c r="DO2" s="44" t="s">
+        <v>308</v>
+      </c>
+      <c r="DP2" s="44" t="s">
+        <v>308</v>
+      </c>
+      <c r="DQ2" s="44" t="s">
+        <v>308</v>
+      </c>
     </row>
-    <row r="3" spans="1:113" ht="132" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:121" ht="132" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>16</v>
       </c>
@@ -2236,43 +2603,43 @@
       <c r="Y3" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="Z3" s="36" t="s">
-        <v>308</v>
-      </c>
-      <c r="AA3" s="36" t="s">
+      <c r="Z3" s="35" t="s">
+        <v>307</v>
+      </c>
+      <c r="AA3" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="AB3" s="36" t="s">
+      <c r="AB3" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="AC3" s="36" t="s">
+      <c r="AC3" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="AD3" s="36" t="s">
+      <c r="AD3" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="AE3" s="36" t="s">
+      <c r="AE3" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="AF3" s="36" t="s">
+      <c r="AF3" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="AG3" s="36" t="s">
+      <c r="AG3" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="AH3" s="36" t="s">
+      <c r="AH3" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="AI3" s="36" t="s">
+      <c r="AI3" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="AJ3" s="36" t="s">
-        <v>310</v>
-      </c>
-      <c r="AK3" s="36" t="s">
-        <v>313</v>
-      </c>
-      <c r="AL3" s="36" t="s">
+      <c r="AJ3" s="35" t="s">
+        <v>335</v>
+      </c>
+      <c r="AK3" s="35" t="s">
+        <v>336</v>
+      </c>
+      <c r="AL3" s="35" t="s">
         <v>44</v>
       </c>
       <c r="AM3" s="25" t="s">
@@ -2300,890 +2667,962 @@
         <v>48</v>
       </c>
       <c r="AU3" s="23" t="s">
+        <v>339</v>
+      </c>
+      <c r="AV3" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="AV3" s="23" t="s">
+      <c r="AW3" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="AW3" s="23" t="s">
+      <c r="AX3" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="AX3" s="23" t="s">
+      <c r="AY3" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="AY3" s="23" t="s">
+      <c r="AZ3" s="23" t="s">
+        <v>339</v>
+      </c>
+      <c r="BA3" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="BB3" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="BC3" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="BD3" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="BE3" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="AZ3" s="23" t="s">
+      <c r="BF3" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="BG3" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="BH3" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="BI3" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="BJ3" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="BK3" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="BL3" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="BM3" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="BN3" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="BO3" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="BP3" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="BQ3" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="BR3" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="BS3" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="BT3" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="BU3" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="BV3" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="BW3" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="BX3" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="BY3" s="37" t="s">
+        <v>63</v>
+      </c>
+      <c r="BZ3" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="CA3" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="CB3" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="CC3" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="CD3" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="CE3" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="CF3" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="CG3" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="CH3" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="CI3" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="CJ3" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="CK3" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="CL3" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="CM3" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="CN3" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="CO3" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="CP3" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="CQ3" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="CR3" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="CS3" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="CT3" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="CU3" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="CV3" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="CW3" s="39" t="s">
+        <v>72</v>
+      </c>
+      <c r="CX3" s="39" t="s">
+        <v>73</v>
+      </c>
+      <c r="CY3" s="39" t="s">
+        <v>74</v>
+      </c>
+      <c r="CZ3" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="DA3" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="DB3" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="DC3" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="DD3" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="DE3" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="DF3" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="DG3" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="DH3" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="DI3" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="DJ3" s="46" t="s">
+        <v>328</v>
+      </c>
+      <c r="DK3" s="47" t="s">
+        <v>327</v>
+      </c>
+      <c r="DL3" s="48" t="s">
+        <v>329</v>
+      </c>
+      <c r="DM3" s="48" t="s">
+        <v>326</v>
+      </c>
+      <c r="DN3" s="48" t="s">
+        <v>330</v>
+      </c>
+      <c r="DO3" s="48" t="s">
+        <v>337</v>
+      </c>
+      <c r="DP3" s="46" t="s">
+        <v>338</v>
+      </c>
+      <c r="DQ3" s="46" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="4" spans="1:121" s="27" customFormat="1" ht="41.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G4" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="H4" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="I4" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="J4" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="K4" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="L4" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="M4" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="N4" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="O4" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="P4" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q4" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="R4" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="S4" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="T4" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="U4" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="V4" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="W4" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="X4" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="Y4" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="Z4" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="AA4" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="AB4" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="AC4" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="AD4" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="AE4" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="AF4" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG4" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="AH4" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="AI4" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="AJ4" s="27" t="s">
+        <v>331</v>
+      </c>
+      <c r="AK4" s="27" t="s">
+        <v>332</v>
+      </c>
+      <c r="AL4" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="AM4" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="AN4" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="AO4" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="AP4" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="AQ4" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="AR4" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="AS4" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="AT4" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AU4" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="AV4" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="AW4" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="AX4" s="27" t="s">
+        <v>132</v>
+      </c>
+      <c r="AY4" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="AZ4" s="27" t="s">
+        <v>134</v>
+      </c>
+      <c r="BA4" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="BB4" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="BC4" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="BD4" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="BE4" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="BF4" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="BG4" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="BH4" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="BI4" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="BJ4" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="BK4" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="BL4" s="27" t="s">
+        <v>146</v>
+      </c>
+      <c r="BM4" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="BN4" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="BO4" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="BP4" s="27" t="s">
+        <v>150</v>
+      </c>
+      <c r="BQ4" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="BR4" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS4" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="BT4" s="27" t="s">
+        <v>154</v>
+      </c>
+      <c r="BU4" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="BV4" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="BW4" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="BX4" s="42" t="s">
+        <v>158</v>
+      </c>
+      <c r="BY4" s="27" t="s">
+        <v>159</v>
+      </c>
+      <c r="BZ4" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="CA4" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="CB4" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="CC4" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="CD4" s="27" t="s">
+        <v>164</v>
+      </c>
+      <c r="CE4" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="CF4" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="CG4" s="27" t="s">
+        <v>167</v>
+      </c>
+      <c r="CH4" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="CI4" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="CJ4" s="27" t="s">
+        <v>170</v>
+      </c>
+      <c r="CK4" s="27" t="s">
+        <v>171</v>
+      </c>
+      <c r="CL4" s="27" t="s">
+        <v>172</v>
+      </c>
+      <c r="CM4" s="27" t="s">
+        <v>173</v>
+      </c>
+      <c r="CN4" s="27" t="s">
+        <v>174</v>
+      </c>
+      <c r="CO4" s="27" t="s">
+        <v>175</v>
+      </c>
+      <c r="CP4" s="27" t="s">
+        <v>176</v>
+      </c>
+      <c r="CQ4" s="27" t="s">
+        <v>177</v>
+      </c>
+      <c r="CR4" s="27" t="s">
+        <v>178</v>
+      </c>
+      <c r="CS4" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="CT4" s="27" t="s">
+        <v>180</v>
+      </c>
+      <c r="CU4" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="CV4" s="27" t="s">
+        <v>182</v>
+      </c>
+      <c r="CW4" s="27" t="s">
+        <v>183</v>
+      </c>
+      <c r="CX4" s="27" t="s">
+        <v>184</v>
+      </c>
+      <c r="CY4" s="27" t="s">
+        <v>185</v>
+      </c>
+      <c r="CZ4" s="27" t="s">
+        <v>186</v>
+      </c>
+      <c r="DA4" s="27" t="s">
+        <v>187</v>
+      </c>
+      <c r="DB4" s="27" t="s">
+        <v>188</v>
+      </c>
+      <c r="DC4" s="27" t="s">
+        <v>189</v>
+      </c>
+      <c r="DD4" s="27" t="s">
+        <v>190</v>
+      </c>
+      <c r="DE4" s="27" t="s">
+        <v>191</v>
+      </c>
+      <c r="DF4" s="27" t="s">
+        <v>192</v>
+      </c>
+      <c r="DG4" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="DH4" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="DI4" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="DJ4" s="27" t="s">
         <v>309</v>
       </c>
-      <c r="BA3" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="BB3" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="BC3" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="BD3" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="BE3" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="BF3" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="BG3" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="BH3" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="BI3" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="BJ3" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="BK3" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="BL3" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="BM3" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="BN3" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="BO3" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="BP3" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="BQ3" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="BR3" s="22" t="s">
-        <v>63</v>
-      </c>
-      <c r="BS3" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="BT3" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="BU3" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="BV3" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="BW3" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="BX3" s="22" t="s">
-        <v>63</v>
-      </c>
-      <c r="BY3" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="BZ3" s="38" t="s">
-        <v>65</v>
-      </c>
-      <c r="CA3" s="40" t="s">
-        <v>66</v>
-      </c>
-      <c r="CB3" s="40" t="s">
-        <v>66</v>
-      </c>
-      <c r="CC3" s="40" t="s">
-        <v>66</v>
-      </c>
-      <c r="CD3" s="40" t="s">
-        <v>67</v>
-      </c>
-      <c r="CE3" s="40" t="s">
-        <v>67</v>
-      </c>
-      <c r="CF3" s="40" t="s">
-        <v>67</v>
-      </c>
-      <c r="CG3" s="40" t="s">
-        <v>68</v>
-      </c>
-      <c r="CH3" s="40" t="s">
-        <v>68</v>
-      </c>
-      <c r="CI3" s="40" t="s">
-        <v>68</v>
-      </c>
-      <c r="CJ3" s="40" t="s">
-        <v>69</v>
-      </c>
-      <c r="CK3" s="40" t="s">
-        <v>69</v>
-      </c>
-      <c r="CL3" s="40" t="s">
-        <v>69</v>
-      </c>
-      <c r="CM3" s="40" t="s">
-        <v>70</v>
-      </c>
-      <c r="CN3" s="40" t="s">
-        <v>70</v>
-      </c>
-      <c r="CO3" s="40" t="s">
-        <v>70</v>
-      </c>
-      <c r="CP3" s="40" t="s">
-        <v>70</v>
-      </c>
-      <c r="CQ3" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="CR3" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="CS3" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="CT3" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="CU3" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="CV3" s="40" t="s">
-        <v>72</v>
-      </c>
-      <c r="CW3" s="40" t="s">
-        <v>73</v>
-      </c>
-      <c r="CX3" s="40" t="s">
-        <v>74</v>
-      </c>
-      <c r="CY3" s="40" t="s">
-        <v>75</v>
-      </c>
-      <c r="CZ3" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="DA3" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="DB3" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="DC3" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="DD3" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="DE3" s="25" t="s">
-        <v>81</v>
-      </c>
-      <c r="DF3" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="DG3" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="DH3" s="25" t="s">
-        <v>84</v>
-      </c>
-      <c r="DI3" s="25" t="s">
-        <v>85</v>
+      <c r="DK4" s="28" t="s">
+        <v>310</v>
+      </c>
+      <c r="DL4" s="27" t="s">
+        <v>311</v>
+      </c>
+      <c r="DM4" s="27" t="s">
+        <v>312</v>
+      </c>
+      <c r="DN4" s="27" t="s">
+        <v>313</v>
+      </c>
+      <c r="DO4" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="DP4" s="27" t="s">
+        <v>315</v>
+      </c>
+      <c r="DQ4" s="27" t="s">
+        <v>316</v>
       </c>
     </row>
-    <row r="4" spans="1:113" s="27" customFormat="1" ht="41.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="41" t="s">
-        <v>87</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>88</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>89</v>
-      </c>
-      <c r="E4" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="F4" s="27" t="s">
-        <v>91</v>
-      </c>
-      <c r="G4" s="27" t="s">
-        <v>92</v>
-      </c>
-      <c r="H4" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="I4" s="27" t="s">
-        <v>94</v>
-      </c>
-      <c r="J4" s="27" t="s">
-        <v>95</v>
-      </c>
-      <c r="K4" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="L4" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="M4" s="27" t="s">
-        <v>98</v>
-      </c>
-      <c r="N4" s="27" t="s">
-        <v>99</v>
-      </c>
-      <c r="O4" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="P4" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="Q4" s="27" t="s">
-        <v>102</v>
-      </c>
-      <c r="R4" s="28" t="s">
-        <v>103</v>
-      </c>
-      <c r="S4" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="T4" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="U4" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="V4" s="28" t="s">
-        <v>107</v>
-      </c>
-      <c r="W4" s="27" t="s">
-        <v>108</v>
-      </c>
-      <c r="X4" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="Y4" s="27" t="s">
-        <v>110</v>
-      </c>
-      <c r="Z4" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="AA4" s="27" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB4" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="AC4" s="27" t="s">
-        <v>114</v>
-      </c>
-      <c r="AD4" s="27" t="s">
-        <v>115</v>
-      </c>
-      <c r="AE4" s="27" t="s">
-        <v>116</v>
-      </c>
-      <c r="AF4" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="AG4" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="AH4" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="AI4" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="AJ4" s="27" t="s">
-        <v>311</v>
-      </c>
-      <c r="AK4" s="27" t="s">
-        <v>314</v>
-      </c>
-      <c r="AL4" s="27" t="s">
-        <v>121</v>
-      </c>
-      <c r="AM4" s="27" t="s">
-        <v>122</v>
-      </c>
-      <c r="AN4" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="AO4" s="27" t="s">
-        <v>124</v>
-      </c>
-      <c r="AP4" s="27" t="s">
-        <v>125</v>
-      </c>
-      <c r="AQ4" s="27" t="s">
-        <v>126</v>
-      </c>
-      <c r="AR4" s="27" t="s">
-        <v>127</v>
-      </c>
-      <c r="AS4" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="AT4" s="27" t="s">
-        <v>129</v>
-      </c>
-      <c r="AU4" s="27" t="s">
-        <v>130</v>
-      </c>
-      <c r="AV4" s="27" t="s">
-        <v>131</v>
-      </c>
-      <c r="AW4" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="AX4" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="AY4" s="27" t="s">
-        <v>134</v>
-      </c>
-      <c r="AZ4" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="BA4" s="27" t="s">
-        <v>136</v>
-      </c>
-      <c r="BB4" s="27" t="s">
-        <v>137</v>
-      </c>
-      <c r="BC4" s="27" t="s">
-        <v>138</v>
-      </c>
-      <c r="BD4" s="27" t="s">
-        <v>139</v>
-      </c>
-      <c r="BE4" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="BF4" s="27" t="s">
-        <v>141</v>
-      </c>
-      <c r="BG4" s="27" t="s">
-        <v>142</v>
-      </c>
-      <c r="BH4" s="27" t="s">
-        <v>143</v>
-      </c>
-      <c r="BI4" s="27" t="s">
-        <v>144</v>
-      </c>
-      <c r="BJ4" s="27" t="s">
-        <v>145</v>
-      </c>
-      <c r="BK4" s="27" t="s">
-        <v>146</v>
-      </c>
-      <c r="BL4" s="27" t="s">
-        <v>147</v>
-      </c>
-      <c r="BM4" s="27" t="s">
-        <v>148</v>
-      </c>
-      <c r="BN4" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="BO4" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="BP4" s="27" t="s">
-        <v>151</v>
-      </c>
-      <c r="BQ4" s="27" t="s">
-        <v>152</v>
-      </c>
-      <c r="BR4" s="29" t="s">
-        <v>153</v>
-      </c>
-      <c r="BS4" s="27" t="s">
-        <v>154</v>
-      </c>
-      <c r="BT4" s="27" t="s">
-        <v>155</v>
-      </c>
-      <c r="BU4" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="BV4" s="27" t="s">
-        <v>157</v>
-      </c>
-      <c r="BW4" s="27" t="s">
-        <v>158</v>
-      </c>
-      <c r="BX4" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="BY4" s="27" t="s">
-        <v>160</v>
-      </c>
-      <c r="BZ4" s="27" t="s">
-        <v>161</v>
-      </c>
-      <c r="CA4" s="27" t="s">
-        <v>162</v>
-      </c>
-      <c r="CB4" s="27" t="s">
-        <v>163</v>
-      </c>
-      <c r="CC4" s="27" t="s">
-        <v>164</v>
-      </c>
-      <c r="CD4" s="27" t="s">
-        <v>165</v>
-      </c>
-      <c r="CE4" s="27" t="s">
-        <v>166</v>
-      </c>
-      <c r="CF4" s="27" t="s">
-        <v>167</v>
-      </c>
-      <c r="CG4" s="27" t="s">
-        <v>168</v>
-      </c>
-      <c r="CH4" s="27" t="s">
-        <v>169</v>
-      </c>
-      <c r="CI4" s="27" t="s">
-        <v>170</v>
-      </c>
-      <c r="CJ4" s="27" t="s">
-        <v>171</v>
-      </c>
-      <c r="CK4" s="27" t="s">
-        <v>172</v>
-      </c>
-      <c r="CL4" s="27" t="s">
-        <v>173</v>
-      </c>
-      <c r="CM4" s="27" t="s">
-        <v>174</v>
-      </c>
-      <c r="CN4" s="27" t="s">
-        <v>175</v>
-      </c>
-      <c r="CO4" s="27" t="s">
-        <v>176</v>
-      </c>
-      <c r="CP4" s="27" t="s">
-        <v>177</v>
-      </c>
-      <c r="CQ4" s="27" t="s">
-        <v>178</v>
-      </c>
-      <c r="CR4" s="27" t="s">
-        <v>179</v>
-      </c>
-      <c r="CS4" s="27" t="s">
-        <v>180</v>
-      </c>
-      <c r="CT4" s="27" t="s">
-        <v>181</v>
-      </c>
-      <c r="CU4" s="27" t="s">
-        <v>182</v>
-      </c>
-      <c r="CV4" s="27" t="s">
-        <v>183</v>
-      </c>
-      <c r="CW4" s="27" t="s">
-        <v>184</v>
-      </c>
-      <c r="CX4" s="27" t="s">
-        <v>185</v>
-      </c>
-      <c r="CY4" s="27" t="s">
-        <v>186</v>
-      </c>
-      <c r="CZ4" s="27" t="s">
-        <v>187</v>
-      </c>
-      <c r="DA4" s="27" t="s">
-        <v>188</v>
-      </c>
-      <c r="DB4" s="27" t="s">
-        <v>189</v>
-      </c>
-      <c r="DC4" s="27" t="s">
-        <v>190</v>
-      </c>
-      <c r="DD4" s="27" t="s">
-        <v>191</v>
-      </c>
-      <c r="DE4" s="27" t="s">
-        <v>192</v>
-      </c>
-      <c r="DF4" s="27" t="s">
-        <v>193</v>
-      </c>
-      <c r="DG4" s="27" t="s">
-        <v>194</v>
-      </c>
-      <c r="DH4" s="27" t="s">
-        <v>195</v>
-      </c>
-      <c r="DI4" s="27" t="s">
+    <row r="5" spans="1:121" ht="82" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="30" t="s">
         <v>196</v>
       </c>
+      <c r="B5" s="41" t="s">
+        <v>197</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>198</v>
+      </c>
+      <c r="D5" s="32" t="s">
+        <v>199</v>
+      </c>
+      <c r="E5" s="31" t="s">
+        <v>200</v>
+      </c>
+      <c r="F5" s="31" t="s">
+        <v>201</v>
+      </c>
+      <c r="G5" s="31" t="s">
+        <v>202</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>203</v>
+      </c>
+      <c r="I5" s="32" t="s">
+        <v>204</v>
+      </c>
+      <c r="J5" s="32" t="s">
+        <v>205</v>
+      </c>
+      <c r="K5" s="32" t="s">
+        <v>206</v>
+      </c>
+      <c r="L5" s="32" t="s">
+        <v>207</v>
+      </c>
+      <c r="M5" s="32" t="s">
+        <v>208</v>
+      </c>
+      <c r="N5" s="32" t="s">
+        <v>209</v>
+      </c>
+      <c r="O5" s="33" t="s">
+        <v>210</v>
+      </c>
+      <c r="P5" s="33" t="s">
+        <v>211</v>
+      </c>
+      <c r="Q5" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="R5" s="33" t="s">
+        <v>213</v>
+      </c>
+      <c r="S5" s="32" t="s">
+        <v>214</v>
+      </c>
+      <c r="T5" s="32" t="s">
+        <v>215</v>
+      </c>
+      <c r="U5" s="33" t="s">
+        <v>216</v>
+      </c>
+      <c r="V5" s="33" t="s">
+        <v>217</v>
+      </c>
+      <c r="W5" s="31" t="s">
+        <v>218</v>
+      </c>
+      <c r="X5" s="33" t="s">
+        <v>219</v>
+      </c>
+      <c r="Y5" s="32" t="s">
+        <v>220</v>
+      </c>
+      <c r="Z5" s="32" t="s">
+        <v>221</v>
+      </c>
+      <c r="AA5" s="32" t="s">
+        <v>222</v>
+      </c>
+      <c r="AB5" s="32" t="s">
+        <v>223</v>
+      </c>
+      <c r="AC5" s="32" t="s">
+        <v>224</v>
+      </c>
+      <c r="AD5" s="32" t="s">
+        <v>225</v>
+      </c>
+      <c r="AE5" s="32" t="s">
+        <v>226</v>
+      </c>
+      <c r="AF5" s="32" t="s">
+        <v>227</v>
+      </c>
+      <c r="AG5" s="32" t="s">
+        <v>228</v>
+      </c>
+      <c r="AH5" s="32" t="s">
+        <v>229</v>
+      </c>
+      <c r="AI5" s="32" t="s">
+        <v>230</v>
+      </c>
+      <c r="AJ5" s="32" t="s">
+        <v>333</v>
+      </c>
+      <c r="AK5" s="32" t="s">
+        <v>334</v>
+      </c>
+      <c r="AL5" s="32" t="s">
+        <v>231</v>
+      </c>
+      <c r="AM5" s="32" t="s">
+        <v>232</v>
+      </c>
+      <c r="AN5" s="32" t="s">
+        <v>233</v>
+      </c>
+      <c r="AO5" s="32" t="s">
+        <v>234</v>
+      </c>
+      <c r="AP5" s="32" t="s">
+        <v>235</v>
+      </c>
+      <c r="AQ5" s="32" t="s">
+        <v>236</v>
+      </c>
+      <c r="AR5" s="32" t="s">
+        <v>237</v>
+      </c>
+      <c r="AS5" s="32" t="s">
+        <v>238</v>
+      </c>
+      <c r="AT5" s="32" t="s">
+        <v>239</v>
+      </c>
+      <c r="AU5" s="32" t="s">
+        <v>240</v>
+      </c>
+      <c r="AV5" s="32" t="s">
+        <v>241</v>
+      </c>
+      <c r="AW5" s="32" t="s">
+        <v>242</v>
+      </c>
+      <c r="AX5" s="32" t="s">
+        <v>243</v>
+      </c>
+      <c r="AY5" s="32" t="s">
+        <v>244</v>
+      </c>
+      <c r="AZ5" s="32" t="s">
+        <v>245</v>
+      </c>
+      <c r="BA5" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="BB5" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="BC5" s="32" t="s">
+        <v>248</v>
+      </c>
+      <c r="BD5" s="32" t="s">
+        <v>249</v>
+      </c>
+      <c r="BE5" s="32" t="s">
+        <v>250</v>
+      </c>
+      <c r="BF5" s="32" t="s">
+        <v>251</v>
+      </c>
+      <c r="BG5" s="32" t="s">
+        <v>252</v>
+      </c>
+      <c r="BH5" s="32" t="s">
+        <v>253</v>
+      </c>
+      <c r="BI5" s="32" t="s">
+        <v>254</v>
+      </c>
+      <c r="BJ5" s="32" t="s">
+        <v>255</v>
+      </c>
+      <c r="BK5" s="32" t="s">
+        <v>256</v>
+      </c>
+      <c r="BL5" s="32" t="s">
+        <v>257</v>
+      </c>
+      <c r="BM5" s="32" t="s">
+        <v>258</v>
+      </c>
+      <c r="BN5" s="31" t="s">
+        <v>259</v>
+      </c>
+      <c r="BO5" s="31" t="s">
+        <v>260</v>
+      </c>
+      <c r="BP5" s="32" t="s">
+        <v>261</v>
+      </c>
+      <c r="BQ5" s="32" t="s">
+        <v>262</v>
+      </c>
+      <c r="BR5" s="32" t="s">
+        <v>263</v>
+      </c>
+      <c r="BS5" s="32" t="s">
+        <v>264</v>
+      </c>
+      <c r="BT5" s="31" t="s">
+        <v>265</v>
+      </c>
+      <c r="BU5" s="31" t="s">
+        <v>266</v>
+      </c>
+      <c r="BV5" s="32" t="s">
+        <v>267</v>
+      </c>
+      <c r="BW5" s="32" t="s">
+        <v>268</v>
+      </c>
+      <c r="BX5" s="32" t="s">
+        <v>269</v>
+      </c>
+      <c r="BY5" s="32" t="s">
+        <v>270</v>
+      </c>
+      <c r="BZ5" s="32" t="s">
+        <v>271</v>
+      </c>
+      <c r="CA5" s="32" t="s">
+        <v>272</v>
+      </c>
+      <c r="CB5" s="32" t="s">
+        <v>273</v>
+      </c>
+      <c r="CC5" s="32" t="s">
+        <v>274</v>
+      </c>
+      <c r="CD5" s="32" t="s">
+        <v>275</v>
+      </c>
+      <c r="CE5" s="32" t="s">
+        <v>276</v>
+      </c>
+      <c r="CF5" s="32" t="s">
+        <v>277</v>
+      </c>
+      <c r="CG5" s="32" t="s">
+        <v>278</v>
+      </c>
+      <c r="CH5" s="32" t="s">
+        <v>279</v>
+      </c>
+      <c r="CI5" s="32" t="s">
+        <v>280</v>
+      </c>
+      <c r="CJ5" s="32" t="s">
+        <v>281</v>
+      </c>
+      <c r="CK5" s="32" t="s">
+        <v>282</v>
+      </c>
+      <c r="CL5" s="32" t="s">
+        <v>283</v>
+      </c>
+      <c r="CM5" s="32" t="s">
+        <v>284</v>
+      </c>
+      <c r="CN5" s="32" t="s">
+        <v>285</v>
+      </c>
+      <c r="CO5" s="32" t="s">
+        <v>286</v>
+      </c>
+      <c r="CP5" s="32" t="s">
+        <v>287</v>
+      </c>
+      <c r="CQ5" s="32" t="s">
+        <v>288</v>
+      </c>
+      <c r="CR5" s="32" t="s">
+        <v>289</v>
+      </c>
+      <c r="CS5" s="32" t="s">
+        <v>290</v>
+      </c>
+      <c r="CT5" s="32" t="s">
+        <v>291</v>
+      </c>
+      <c r="CU5" s="32" t="s">
+        <v>292</v>
+      </c>
+      <c r="CV5" s="32" t="s">
+        <v>293</v>
+      </c>
+      <c r="CW5" s="32" t="s">
+        <v>294</v>
+      </c>
+      <c r="CX5" s="32" t="s">
+        <v>295</v>
+      </c>
+      <c r="CY5" s="32" t="s">
+        <v>296</v>
+      </c>
+      <c r="CZ5" s="32" t="s">
+        <v>297</v>
+      </c>
+      <c r="DA5" s="32" t="s">
+        <v>298</v>
+      </c>
+      <c r="DB5" s="32" t="s">
+        <v>299</v>
+      </c>
+      <c r="DC5" s="32" t="s">
+        <v>300</v>
+      </c>
+      <c r="DD5" s="32" t="s">
+        <v>301</v>
+      </c>
+      <c r="DE5" s="32" t="s">
+        <v>302</v>
+      </c>
+      <c r="DF5" s="32" t="s">
+        <v>303</v>
+      </c>
+      <c r="DG5" s="32" t="s">
+        <v>304</v>
+      </c>
+      <c r="DH5" s="32" t="s">
+        <v>305</v>
+      </c>
+      <c r="DI5" s="32" t="s">
+        <v>306</v>
+      </c>
+      <c r="DJ5" s="32" t="s">
+        <v>319</v>
+      </c>
+      <c r="DK5" s="33" t="s">
+        <v>320</v>
+      </c>
+      <c r="DL5" s="32" t="s">
+        <v>321</v>
+      </c>
+      <c r="DM5" s="32" t="s">
+        <v>317</v>
+      </c>
+      <c r="DN5" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="DO5" s="32" t="s">
+        <v>322</v>
+      </c>
+      <c r="DP5" s="32" t="s">
+        <v>323</v>
+      </c>
+      <c r="DQ5" s="32" t="s">
+        <v>324</v>
+      </c>
     </row>
-    <row r="5" spans="1:113" ht="31" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
-        <v>197</v>
-      </c>
-      <c r="B5" s="42" t="s">
-        <v>198</v>
-      </c>
-      <c r="C5" s="32" t="s">
-        <v>199</v>
-      </c>
-      <c r="D5" s="33" t="s">
-        <v>200</v>
-      </c>
-      <c r="E5" s="32" t="s">
-        <v>201</v>
-      </c>
-      <c r="F5" s="32" t="s">
-        <v>202</v>
-      </c>
-      <c r="G5" s="32" t="s">
-        <v>203</v>
-      </c>
-      <c r="H5" s="33" t="s">
-        <v>204</v>
-      </c>
-      <c r="I5" s="33" t="s">
-        <v>205</v>
-      </c>
-      <c r="J5" s="33" t="s">
-        <v>206</v>
-      </c>
-      <c r="K5" s="33" t="s">
-        <v>207</v>
-      </c>
-      <c r="L5" s="33" t="s">
-        <v>208</v>
-      </c>
-      <c r="M5" s="33" t="s">
-        <v>209</v>
-      </c>
-      <c r="N5" s="33" t="s">
-        <v>210</v>
-      </c>
-      <c r="O5" s="34" t="s">
-        <v>211</v>
-      </c>
-      <c r="P5" s="34" t="s">
-        <v>212</v>
-      </c>
-      <c r="Q5" s="32" t="s">
-        <v>213</v>
-      </c>
-      <c r="R5" s="34" t="s">
-        <v>214</v>
-      </c>
-      <c r="S5" s="33" t="s">
-        <v>215</v>
-      </c>
-      <c r="T5" s="33" t="s">
-        <v>216</v>
-      </c>
-      <c r="U5" s="34" t="s">
-        <v>217</v>
-      </c>
-      <c r="V5" s="34" t="s">
-        <v>218</v>
-      </c>
-      <c r="W5" s="32" t="s">
-        <v>219</v>
-      </c>
-      <c r="X5" s="34" t="s">
-        <v>220</v>
-      </c>
-      <c r="Y5" s="33" t="s">
-        <v>221</v>
-      </c>
-      <c r="Z5" s="33" t="s">
-        <v>222</v>
-      </c>
-      <c r="AA5" s="33" t="s">
-        <v>223</v>
-      </c>
-      <c r="AB5" s="33" t="s">
-        <v>224</v>
-      </c>
-      <c r="AC5" s="33" t="s">
-        <v>225</v>
-      </c>
-      <c r="AD5" s="33" t="s">
-        <v>226</v>
-      </c>
-      <c r="AE5" s="33" t="s">
-        <v>227</v>
-      </c>
-      <c r="AF5" s="33" t="s">
-        <v>228</v>
-      </c>
-      <c r="AG5" s="33" t="s">
-        <v>229</v>
-      </c>
-      <c r="AH5" s="33" t="s">
-        <v>230</v>
-      </c>
-      <c r="AI5" s="33" t="s">
-        <v>231</v>
-      </c>
-      <c r="AJ5" s="33" t="s">
-        <v>312</v>
-      </c>
-      <c r="AK5" s="33" t="s">
-        <v>315</v>
-      </c>
-      <c r="AL5" s="33" t="s">
-        <v>232</v>
-      </c>
-      <c r="AM5" s="33" t="s">
-        <v>233</v>
-      </c>
-      <c r="AN5" s="33" t="s">
-        <v>234</v>
-      </c>
-      <c r="AO5" s="33" t="s">
-        <v>235</v>
-      </c>
-      <c r="AP5" s="33" t="s">
-        <v>236</v>
-      </c>
-      <c r="AQ5" s="33" t="s">
-        <v>237</v>
-      </c>
-      <c r="AR5" s="33" t="s">
-        <v>238</v>
-      </c>
-      <c r="AS5" s="33" t="s">
-        <v>239</v>
-      </c>
-      <c r="AT5" s="33" t="s">
-        <v>240</v>
-      </c>
-      <c r="AU5" s="33" t="s">
-        <v>241</v>
-      </c>
-      <c r="AV5" s="33" t="s">
-        <v>242</v>
-      </c>
-      <c r="AW5" s="33" t="s">
-        <v>243</v>
-      </c>
-      <c r="AX5" s="33" t="s">
-        <v>244</v>
-      </c>
-      <c r="AY5" s="33" t="s">
-        <v>245</v>
-      </c>
-      <c r="AZ5" s="33" t="s">
-        <v>246</v>
-      </c>
-      <c r="BA5" s="33" t="s">
-        <v>247</v>
-      </c>
-      <c r="BB5" s="33" t="s">
-        <v>248</v>
-      </c>
-      <c r="BC5" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="BD5" s="33" t="s">
-        <v>250</v>
-      </c>
-      <c r="BE5" s="33" t="s">
-        <v>251</v>
-      </c>
-      <c r="BF5" s="33" t="s">
-        <v>252</v>
-      </c>
-      <c r="BG5" s="33" t="s">
-        <v>253</v>
-      </c>
-      <c r="BH5" s="33" t="s">
-        <v>254</v>
-      </c>
-      <c r="BI5" s="33" t="s">
-        <v>255</v>
-      </c>
-      <c r="BJ5" s="33" t="s">
-        <v>256</v>
-      </c>
-      <c r="BK5" s="33" t="s">
-        <v>257</v>
-      </c>
-      <c r="BL5" s="33" t="s">
-        <v>258</v>
-      </c>
-      <c r="BM5" s="33" t="s">
-        <v>259</v>
-      </c>
-      <c r="BN5" s="32" t="s">
-        <v>260</v>
-      </c>
-      <c r="BO5" s="32" t="s">
-        <v>261</v>
-      </c>
-      <c r="BP5" s="33" t="s">
-        <v>262</v>
-      </c>
-      <c r="BQ5" s="33" t="s">
-        <v>263</v>
-      </c>
-      <c r="BR5" s="33" t="s">
-        <v>264</v>
-      </c>
-      <c r="BS5" s="33" t="s">
-        <v>265</v>
-      </c>
-      <c r="BT5" s="32" t="s">
-        <v>266</v>
-      </c>
-      <c r="BU5" s="32" t="s">
-        <v>267</v>
-      </c>
-      <c r="BV5" s="33" t="s">
-        <v>268</v>
-      </c>
-      <c r="BW5" s="33" t="s">
-        <v>269</v>
-      </c>
-      <c r="BX5" s="33" t="s">
-        <v>270</v>
-      </c>
-      <c r="BY5" s="33" t="s">
-        <v>271</v>
-      </c>
-      <c r="BZ5" s="33" t="s">
-        <v>272</v>
-      </c>
-      <c r="CA5" s="33" t="s">
-        <v>273</v>
-      </c>
-      <c r="CB5" s="33" t="s">
-        <v>274</v>
-      </c>
-      <c r="CC5" s="33" t="s">
-        <v>275</v>
-      </c>
-      <c r="CD5" s="33" t="s">
-        <v>276</v>
-      </c>
-      <c r="CE5" s="33" t="s">
-        <v>277</v>
-      </c>
-      <c r="CF5" s="33" t="s">
-        <v>278</v>
-      </c>
-      <c r="CG5" s="33" t="s">
-        <v>279</v>
-      </c>
-      <c r="CH5" s="33" t="s">
-        <v>280</v>
-      </c>
-      <c r="CI5" s="33" t="s">
-        <v>281</v>
-      </c>
-      <c r="CJ5" s="33" t="s">
-        <v>282</v>
-      </c>
-      <c r="CK5" s="33" t="s">
-        <v>283</v>
-      </c>
-      <c r="CL5" s="33" t="s">
-        <v>284</v>
-      </c>
-      <c r="CM5" s="33" t="s">
-        <v>285</v>
-      </c>
-      <c r="CN5" s="33" t="s">
-        <v>286</v>
-      </c>
-      <c r="CO5" s="33" t="s">
-        <v>287</v>
-      </c>
-      <c r="CP5" s="33" t="s">
-        <v>288</v>
-      </c>
-      <c r="CQ5" s="33" t="s">
-        <v>289</v>
-      </c>
-      <c r="CR5" s="33" t="s">
-        <v>290</v>
-      </c>
-      <c r="CS5" s="33" t="s">
-        <v>291</v>
-      </c>
-      <c r="CT5" s="33" t="s">
-        <v>292</v>
-      </c>
-      <c r="CU5" s="33" t="s">
-        <v>293</v>
-      </c>
-      <c r="CV5" s="33" t="s">
-        <v>294</v>
-      </c>
-      <c r="CW5" s="33" t="s">
-        <v>295</v>
-      </c>
-      <c r="CX5" s="33" t="s">
-        <v>296</v>
-      </c>
-      <c r="CY5" s="33" t="s">
-        <v>297</v>
-      </c>
-      <c r="CZ5" s="33" t="s">
-        <v>298</v>
-      </c>
-      <c r="DA5" s="33" t="s">
-        <v>299</v>
-      </c>
-      <c r="DB5" s="33" t="s">
-        <v>300</v>
-      </c>
-      <c r="DC5" s="33" t="s">
-        <v>301</v>
-      </c>
-      <c r="DD5" s="33" t="s">
-        <v>302</v>
-      </c>
-      <c r="DE5" s="33" t="s">
-        <v>303</v>
-      </c>
-      <c r="DF5" s="33" t="s">
-        <v>304</v>
-      </c>
-      <c r="DG5" s="33" t="s">
-        <v>305</v>
-      </c>
-      <c r="DH5" s="33" t="s">
-        <v>306</v>
-      </c>
-      <c r="DI5" s="33" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="6" spans="1:113" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:121" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1 L5" xr:uid="{00000000-0002-0000-0000-000004000000}">

</xml_diff>

<commit_message>
ANW-3085 Add a column to make the imported digital object instance representative
The digital object import links each digital object it creates to an
existing archival object, but could not make that instance representative,
and an archival object only shows a thumbnail through its representative
instance. The digital_object_is_representative column (FALSE/TRUE, blank
for FALSE), already in the archival object import, now marks it in the
CSV and Excel digital object templates too.

An archival object has one representative instance at most. When it
already has one, or an earlier row of the spreadsheet made one
representative, the digital object of the row is still linked to the
archival object, but not as representative, and the row logs an error.
A validation run saves nothing, so it remembers the archival objects its
earlier rows made representative to report the same rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/bulk_import_templates/bulk_import_DO_template.xlsx
+++ b/frontend/public/bulk_import_templates/bulk_import_DO_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="343">
   <si>
     <t>This is the template for use with the bulk_import ("Load SpreadSheet") for importing digital ob jects to associate with archival objects .  You may replace this line with something of your choosing after you've copied the file for your use.</t>
   </si>
@@ -1278,6 +1278,15 @@
   <si>
     <t>Accepted Types: 
 person, family, corporate_entity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make the instance linking the archival object to the digital object representative (FALSE/TRUE)? The archival object then shows the thumbnail of the digital object. An archival object can have only one representative instance, so if it already has one, the digital object is linked but not made representative. Leave this blank to get the default value FALSE.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">digital_object_is_representative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make Digital Object Instance Representative</t>
   </si>
 </sst>
 </file>
@@ -2087,7 +2096,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DQ6"/>
+  <dimension ref="A1:DR6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.33203125" style="1" customWidth="1"/>
@@ -2099,70 +2108,71 @@
     <col min="8" max="8" width="29.33203125" style="2" customWidth="1"/>
     <col min="9" max="9" width="25.1640625" style="2" customWidth="1"/>
     <col min="10" max="10" width="22.6640625" customWidth="1"/>
-    <col min="11" max="12" width="17.33203125" customWidth="1"/>
-    <col min="13" max="13" width="20.6640625" customWidth="1"/>
-    <col min="14" max="14" width="20.5" style="2" customWidth="1"/>
-    <col min="15" max="15" width="11" style="3" customWidth="1"/>
-    <col min="16" max="16" width="10.5" style="3" customWidth="1"/>
-    <col min="17" max="17" width="23.83203125" style="2" customWidth="1"/>
-    <col min="18" max="18" width="15.1640625" style="3" customWidth="1"/>
-    <col min="19" max="19" width="26.83203125" style="2" customWidth="1"/>
-    <col min="20" max="20" width="20.5" style="2" customWidth="1"/>
-    <col min="21" max="21" width="11" style="3" customWidth="1"/>
-    <col min="22" max="22" width="10.5" style="3" customWidth="1"/>
-    <col min="23" max="23" width="23.83203125" style="2" customWidth="1"/>
-    <col min="24" max="24" width="15.1640625" style="3" customWidth="1"/>
-    <col min="25" max="25" width="26.83203125" style="2" customWidth="1"/>
-    <col min="26" max="27" width="17.33203125" style="2" customWidth="1"/>
-    <col min="28" max="29" width="17.5" style="2" customWidth="1"/>
-    <col min="30" max="30" width="15.83203125" style="2" customWidth="1"/>
-    <col min="31" max="33" width="9.33203125" style="2" customWidth="1"/>
-    <col min="34" max="34" width="10.1640625" style="2" customWidth="1"/>
-    <col min="35" max="35" width="9.33203125" style="2" customWidth="1"/>
-    <col min="36" max="36" width="24" style="2" customWidth="1"/>
-    <col min="37" max="37" width="21.83203125" style="2" customWidth="1"/>
-    <col min="38" max="38" width="9.33203125" style="2" customWidth="1"/>
-    <col min="39" max="46" width="17.6640625" style="2" customWidth="1"/>
-    <col min="47" max="47" width="16" style="2" customWidth="1"/>
-    <col min="48" max="48" width="11.33203125" style="2" customWidth="1"/>
-    <col min="49" max="49" width="15.1640625" style="2" customWidth="1"/>
-    <col min="50" max="50" width="20.1640625" style="2" customWidth="1"/>
-    <col min="51" max="51" width="15.33203125" style="2" customWidth="1"/>
-    <col min="52" max="53" width="12.83203125" style="2" customWidth="1"/>
-    <col min="54" max="54" width="15.1640625" style="2" customWidth="1"/>
-    <col min="55" max="55" width="20.1640625" style="2" customWidth="1"/>
-    <col min="56" max="56" width="15.33203125" style="2" customWidth="1"/>
-    <col min="57" max="57" width="15.5" style="2" customWidth="1"/>
-    <col min="58" max="58" width="16.83203125" style="2" customWidth="1"/>
-    <col min="59" max="59" width="17.6640625" style="2" customWidth="1"/>
-    <col min="60" max="60" width="17.6640625" customWidth="1"/>
-    <col min="61" max="61" width="17" style="2" customWidth="1"/>
-    <col min="62" max="62" width="17.6640625" style="2" customWidth="1"/>
-    <col min="63" max="63" width="17.6640625" customWidth="1"/>
-    <col min="64" max="64" width="17.6640625" style="2" customWidth="1"/>
-    <col min="65" max="76" width="26.83203125" style="2" customWidth="1"/>
-    <col min="77" max="78" width="16.83203125" style="2" customWidth="1"/>
-    <col min="79" max="79" width="23.33203125" style="2" customWidth="1"/>
-    <col min="80" max="103" width="12.83203125" style="2" customWidth="1"/>
-    <col min="104" max="104" width="15.33203125" style="2" customWidth="1"/>
-    <col min="105" max="105" width="16.6640625" style="2" customWidth="1"/>
-    <col min="106" max="107" width="13.5" style="2" customWidth="1"/>
-    <col min="108" max="108" width="17.33203125" style="2" customWidth="1"/>
-    <col min="109" max="112" width="16" style="2" customWidth="1"/>
-    <col min="113" max="113" width="13.5" style="2" customWidth="1"/>
-    <col min="114" max="114" width="21.5" style="2" customWidth="1"/>
-    <col min="115" max="115" width="21.5" style="3" customWidth="1"/>
-    <col min="116" max="121" width="21.5" style="2" customWidth="1"/>
+    <col min="11" max="11" width="29.33203125" customWidth="1"/>
+    <col min="12" max="13" width="17.33203125" customWidth="1"/>
+    <col min="14" max="14" width="20.6640625" customWidth="1"/>
+    <col min="15" max="15" width="20.5" style="2" customWidth="1"/>
+    <col min="16" max="16" width="11" style="3" customWidth="1"/>
+    <col min="17" max="17" width="10.5" style="3" customWidth="1"/>
+    <col min="18" max="18" width="23.83203125" style="2" customWidth="1"/>
+    <col min="19" max="19" width="15.1640625" style="3" customWidth="1"/>
+    <col min="20" max="20" width="26.83203125" style="2" customWidth="1"/>
+    <col min="21" max="21" width="20.5" style="2" customWidth="1"/>
+    <col min="22" max="22" width="11" style="3" customWidth="1"/>
+    <col min="23" max="23" width="10.5" style="3" customWidth="1"/>
+    <col min="24" max="24" width="23.83203125" style="2" customWidth="1"/>
+    <col min="25" max="25" width="15.1640625" style="3" customWidth="1"/>
+    <col min="26" max="26" width="26.83203125" style="2" customWidth="1"/>
+    <col min="27" max="28" width="17.33203125" style="2" customWidth="1"/>
+    <col min="29" max="30" width="17.5" style="2" customWidth="1"/>
+    <col min="31" max="31" width="15.83203125" style="2" customWidth="1"/>
+    <col min="32" max="34" width="9.33203125" style="2" customWidth="1"/>
+    <col min="35" max="35" width="10.1640625" style="2" customWidth="1"/>
+    <col min="36" max="36" width="9.33203125" style="2" customWidth="1"/>
+    <col min="37" max="37" width="24" style="2" customWidth="1"/>
+    <col min="38" max="38" width="21.83203125" style="2" customWidth="1"/>
+    <col min="39" max="39" width="9.33203125" style="2" customWidth="1"/>
+    <col min="40" max="47" width="17.6640625" style="2" customWidth="1"/>
+    <col min="48" max="48" width="16" style="2" customWidth="1"/>
+    <col min="49" max="49" width="11.33203125" style="2" customWidth="1"/>
+    <col min="50" max="50" width="15.1640625" style="2" customWidth="1"/>
+    <col min="51" max="51" width="20.1640625" style="2" customWidth="1"/>
+    <col min="52" max="52" width="15.33203125" style="2" customWidth="1"/>
+    <col min="53" max="54" width="12.83203125" style="2" customWidth="1"/>
+    <col min="55" max="55" width="15.1640625" style="2" customWidth="1"/>
+    <col min="56" max="56" width="20.1640625" style="2" customWidth="1"/>
+    <col min="57" max="57" width="15.33203125" style="2" customWidth="1"/>
+    <col min="58" max="58" width="15.5" style="2" customWidth="1"/>
+    <col min="59" max="59" width="16.83203125" style="2" customWidth="1"/>
+    <col min="60" max="60" width="17.6640625" style="2" customWidth="1"/>
+    <col min="61" max="61" width="17.6640625" customWidth="1"/>
+    <col min="62" max="62" width="17" style="2" customWidth="1"/>
+    <col min="63" max="63" width="17.6640625" style="2" customWidth="1"/>
+    <col min="64" max="64" width="17.6640625" customWidth="1"/>
+    <col min="65" max="65" width="17.6640625" style="2" customWidth="1"/>
+    <col min="66" max="77" width="26.83203125" style="2" customWidth="1"/>
+    <col min="78" max="79" width="16.83203125" style="2" customWidth="1"/>
+    <col min="80" max="80" width="23.33203125" style="2" customWidth="1"/>
+    <col min="81" max="104" width="12.83203125" style="2" customWidth="1"/>
+    <col min="105" max="105" width="15.33203125" style="2" customWidth="1"/>
+    <col min="106" max="106" width="16.6640625" style="2" customWidth="1"/>
+    <col min="107" max="108" width="13.5" style="2" customWidth="1"/>
+    <col min="109" max="109" width="17.33203125" style="2" customWidth="1"/>
+    <col min="110" max="113" width="16" style="2" customWidth="1"/>
+    <col min="114" max="114" width="13.5" style="2" customWidth="1"/>
+    <col min="115" max="115" width="21.5" style="2" customWidth="1"/>
+    <col min="116" max="116" width="21.5" style="3" customWidth="1"/>
+    <col min="117" max="122" width="21.5" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:121" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:122" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="BH1" s="2"/>
-      <c r="BK1" s="2"/>
+      <c r="BI1" s="2"/>
+      <c r="BL1" s="2"/>
     </row>
-    <row r="2" spans="1:121" s="2" customFormat="1" ht="41.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:122" s="2" customFormat="1" ht="41.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -2202,44 +2212,44 @@
       <c r="M2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="O2" s="8" t="s">
+      <c r="N2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="O2" s="7" t="s">
         <v>6</v>
       </c>
       <c r="P2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="Q2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="R2" s="8" t="s">
+      <c r="R2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="S2" s="7" t="s">
+      <c r="S2" s="8" t="s">
         <v>6</v>
       </c>
       <c r="T2" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="U2" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="U2" s="7" t="s">
         <v>7</v>
       </c>
       <c r="V2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="W2" s="7" t="s">
+      <c r="W2" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="X2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="X2" s="8" t="s">
+      <c r="Y2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="Y2" s="7" t="s">
+      <c r="Z2" s="7" t="s">
         <v>7</v>
-      </c>
-      <c r="Z2" s="34" t="s">
-        <v>5</v>
       </c>
       <c r="AA2" s="34" t="s">
         <v>5</v>
@@ -2277,8 +2287,8 @@
       <c r="AL2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="AM2" s="12" t="s">
-        <v>9</v>
+      <c r="AM2" s="34" t="s">
+        <v>5</v>
       </c>
       <c r="AN2" s="12" t="s">
         <v>9</v>
@@ -2301,8 +2311,8 @@
       <c r="AT2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AU2" s="10" t="s">
-        <v>10</v>
+      <c r="AU2" s="12" t="s">
+        <v>9</v>
       </c>
       <c r="AV2" s="10" t="s">
         <v>10</v>
@@ -2331,8 +2341,8 @@
       <c r="BD2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="BE2" s="11" t="s">
-        <v>11</v>
+      <c r="BE2" s="10" t="s">
+        <v>10</v>
       </c>
       <c r="BF2" s="11" t="s">
         <v>11</v>
@@ -2355,8 +2365,8 @@
       <c r="BL2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="BM2" s="9" t="s">
-        <v>12</v>
+      <c r="BM2" s="11" t="s">
+        <v>11</v>
       </c>
       <c r="BN2" s="9" t="s">
         <v>12</v>
@@ -2391,14 +2401,14 @@
       <c r="BX2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="BY2" s="36" t="s">
-        <v>13</v>
+      <c r="BY2" s="9" t="s">
+        <v>12</v>
       </c>
       <c r="BZ2" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="CA2" s="38" t="s">
-        <v>14</v>
+      <c r="CA2" s="36" t="s">
+        <v>13</v>
       </c>
       <c r="CB2" s="38" t="s">
         <v>14</v>
@@ -2472,8 +2482,8 @@
       <c r="CY2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="CZ2" s="12" t="s">
-        <v>15</v>
+      <c r="CZ2" s="38" t="s">
+        <v>14</v>
       </c>
       <c r="DA2" s="12" t="s">
         <v>15</v>
@@ -2502,13 +2512,13 @@
       <c r="DI2" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="DJ2" s="44" t="s">
+      <c r="DJ2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="DK2" s="44" t="s">
         <v>308</v>
       </c>
-      <c r="DK2" s="45" t="s">
-        <v>308</v>
-      </c>
-      <c r="DL2" s="44" t="s">
+      <c r="DL2" s="45" t="s">
         <v>308</v>
       </c>
       <c r="DM2" s="44" t="s">
@@ -2526,8 +2536,11 @@
       <c r="DQ2" s="44" t="s">
         <v>308</v>
       </c>
+      <c r="DR2" s="44" t="s">
+        <v>308</v>
+      </c>
     </row>
-    <row r="3" spans="1:121" ht="132" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:122" ht="132" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>16</v>
       </c>
@@ -2559,211 +2572,211 @@
         <v>25</v>
       </c>
       <c r="K3" s="16" t="s">
+        <v>340</v>
+      </c>
+      <c r="L3" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="L3" s="16" t="s">
+      <c r="M3" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="M3" s="16" t="s">
+      <c r="N3" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="N3" s="17" t="s">
+      <c r="O3" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="O3" s="18" t="s">
+      <c r="P3" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="P3" s="18" t="s">
+      <c r="Q3" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="Q3" s="17" t="s">
+      <c r="R3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="R3" s="18" t="s">
+      <c r="S3" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="19" t="s">
+      <c r="T3" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="T3" s="17" t="s">
+      <c r="U3" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="U3" s="18" t="s">
+      <c r="V3" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="18" t="s">
+      <c r="W3" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="W3" s="17" t="s">
+      <c r="X3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="X3" s="18" t="s">
+      <c r="Y3" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="Y3" s="19" t="s">
+      <c r="Z3" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="Z3" s="35" t="s">
+      <c r="AA3" s="35" t="s">
         <v>307</v>
       </c>
-      <c r="AA3" s="35" t="s">
+      <c r="AB3" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="AB3" s="35" t="s">
+      <c r="AC3" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="AC3" s="35" t="s">
+      <c r="AD3" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="AD3" s="35" t="s">
+      <c r="AE3" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="AE3" s="35" t="s">
+      <c r="AF3" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="AF3" s="35" t="s">
+      <c r="AG3" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="AG3" s="35" t="s">
+      <c r="AH3" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="AH3" s="35" t="s">
+      <c r="AI3" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="AI3" s="35" t="s">
+      <c r="AJ3" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="AJ3" s="35" t="s">
+      <c r="AK3" s="35" t="s">
         <v>335</v>
       </c>
-      <c r="AK3" s="35" t="s">
+      <c r="AL3" s="35" t="s">
         <v>336</v>
       </c>
-      <c r="AL3" s="35" t="s">
+      <c r="AM3" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="AM3" s="25" t="s">
+      <c r="AN3" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="AN3" s="25" t="s">
+      <c r="AO3" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="AO3" s="25" t="s">
+      <c r="AP3" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="AP3" s="25" t="s">
+      <c r="AQ3" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="AQ3" s="25" t="s">
+      <c r="AR3" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="AR3" s="25" t="s">
+      <c r="AS3" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="AS3" s="25" t="s">
+      <c r="AT3" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="AT3" s="25" t="s">
+      <c r="AU3" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="AU3" s="23" t="s">
+      <c r="AV3" s="23" t="s">
         <v>339</v>
       </c>
-      <c r="AV3" s="23" t="s">
+      <c r="AW3" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="AW3" s="23" t="s">
+      <c r="AX3" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="AX3" s="23" t="s">
+      <c r="AY3" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="AY3" s="23" t="s">
+      <c r="AZ3" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="AZ3" s="23" t="s">
+      <c r="BA3" s="23" t="s">
         <v>339</v>
       </c>
-      <c r="BA3" s="23" t="s">
+      <c r="BB3" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="BB3" s="23" t="s">
+      <c r="BC3" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="BC3" s="23" t="s">
+      <c r="BD3" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="BD3" s="23" t="s">
+      <c r="BE3" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="BE3" s="24" t="s">
+      <c r="BF3" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="BF3" s="24" t="s">
+      <c r="BG3" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="BG3" s="24" t="s">
+      <c r="BH3" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="BH3" s="24" t="s">
+      <c r="BI3" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="BI3" s="24" t="s">
+      <c r="BJ3" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="BJ3" s="24" t="s">
+      <c r="BK3" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="BK3" s="24" t="s">
+      <c r="BL3" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="BL3" s="24" t="s">
+      <c r="BM3" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="BM3" s="20" t="s">
+      <c r="BN3" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="BN3" s="20" t="s">
+      <c r="BO3" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="BO3" s="20" t="s">
+      <c r="BP3" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="BP3" s="21" t="s">
+      <c r="BQ3" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="BQ3" s="21" t="s">
+      <c r="BR3" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="BR3" s="43" t="s">
+      <c r="BS3" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="BS3" s="20" t="s">
+      <c r="BT3" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="BT3" s="20" t="s">
+      <c r="BU3" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="BU3" s="20" t="s">
+      <c r="BV3" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="BV3" s="21" t="s">
+      <c r="BW3" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="BW3" s="21" t="s">
+      <c r="BX3" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="BX3" s="22" t="s">
+      <c r="BY3" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="BY3" s="37" t="s">
+      <c r="BZ3" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="BZ3" s="37" t="s">
+      <c r="CA3" s="37" t="s">
         <v>64</v>
-      </c>
-      <c r="CA3" s="39" t="s">
-        <v>65</v>
       </c>
       <c r="CB3" s="39" t="s">
         <v>65</v>
@@ -2772,7 +2785,7 @@
         <v>65</v>
       </c>
       <c r="CD3" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="CE3" s="39" t="s">
         <v>66</v>
@@ -2781,7 +2794,7 @@
         <v>66</v>
       </c>
       <c r="CG3" s="39" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="CH3" s="39" t="s">
         <v>67</v>
@@ -2790,7 +2803,7 @@
         <v>67</v>
       </c>
       <c r="CJ3" s="39" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="CK3" s="39" t="s">
         <v>68</v>
@@ -2799,7 +2812,7 @@
         <v>68</v>
       </c>
       <c r="CM3" s="39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="CN3" s="39" t="s">
         <v>69</v>
@@ -2811,7 +2824,7 @@
         <v>69</v>
       </c>
       <c r="CQ3" s="39" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="CR3" s="39" t="s">
         <v>70</v>
@@ -2826,73 +2839,76 @@
         <v>70</v>
       </c>
       <c r="CV3" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="CW3" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="CW3" s="39" t="s">
+      <c r="CX3" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="CX3" s="39" t="s">
+      <c r="CY3" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="CY3" s="39" t="s">
+      <c r="CZ3" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="CZ3" s="25" t="s">
+      <c r="DA3" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="DA3" s="25" t="s">
+      <c r="DB3" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="DB3" s="25" t="s">
+      <c r="DC3" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="DC3" s="25" t="s">
+      <c r="DD3" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="DD3" s="25" t="s">
+      <c r="DE3" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="DE3" s="25" t="s">
+      <c r="DF3" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="DF3" s="25" t="s">
+      <c r="DG3" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="DG3" s="25" t="s">
+      <c r="DH3" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="DH3" s="25" t="s">
+      <c r="DI3" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="DI3" s="25" t="s">
+      <c r="DJ3" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="DJ3" s="46" t="s">
+      <c r="DK3" s="46" t="s">
         <v>328</v>
       </c>
-      <c r="DK3" s="47" t="s">
+      <c r="DL3" s="47" t="s">
         <v>327</v>
       </c>
-      <c r="DL3" s="48" t="s">
+      <c r="DM3" s="48" t="s">
         <v>329</v>
       </c>
-      <c r="DM3" s="48" t="s">
+      <c r="DN3" s="48" t="s">
         <v>326</v>
       </c>
-      <c r="DN3" s="48" t="s">
+      <c r="DO3" s="48" t="s">
         <v>330</v>
       </c>
-      <c r="DO3" s="48" t="s">
+      <c r="DP3" s="48" t="s">
         <v>337</v>
       </c>
-      <c r="DP3" s="46" t="s">
+      <c r="DQ3" s="46" t="s">
         <v>338</v>
       </c>
-      <c r="DQ3" s="46" t="s">
+      <c r="DR3" s="46" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="4" spans="1:121" s="27" customFormat="1" ht="41.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:122" s="27" customFormat="1" ht="41.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
         <v>85</v>
       </c>
@@ -2924,340 +2940,343 @@
         <v>94</v>
       </c>
       <c r="K4" s="27" t="s">
+        <v>341</v>
+      </c>
+      <c r="L4" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="L4" s="27" t="s">
+      <c r="M4" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="M4" s="27" t="s">
+      <c r="N4" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="N4" s="27" t="s">
+      <c r="O4" s="27" t="s">
         <v>98</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="P4" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="P4" s="28" t="s">
+      <c r="Q4" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="Q4" s="27" t="s">
+      <c r="R4" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="R4" s="28" t="s">
+      <c r="S4" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="S4" s="27" t="s">
+      <c r="T4" s="27" t="s">
         <v>103</v>
       </c>
-      <c r="T4" s="27" t="s">
+      <c r="U4" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="U4" s="28" t="s">
+      <c r="V4" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="V4" s="28" t="s">
+      <c r="W4" s="28" t="s">
         <v>106</v>
       </c>
-      <c r="W4" s="27" t="s">
+      <c r="X4" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="X4" s="28" t="s">
+      <c r="Y4" s="28" t="s">
         <v>108</v>
       </c>
-      <c r="Y4" s="27" t="s">
+      <c r="Z4" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="Z4" s="27" t="s">
+      <c r="AA4" s="27" t="s">
         <v>110</v>
       </c>
-      <c r="AA4" s="27" t="s">
+      <c r="AB4" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="AB4" s="27" t="s">
+      <c r="AC4" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="AC4" s="27" t="s">
+      <c r="AD4" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="AD4" s="27" t="s">
+      <c r="AE4" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="AE4" s="27" t="s">
+      <c r="AF4" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="AF4" s="27" t="s">
+      <c r="AG4" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="AG4" s="27" t="s">
+      <c r="AH4" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="AH4" s="27" t="s">
+      <c r="AI4" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="AI4" s="27" t="s">
+      <c r="AJ4" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="AJ4" s="27" t="s">
+      <c r="AK4" s="27" t="s">
         <v>331</v>
       </c>
-      <c r="AK4" s="27" t="s">
+      <c r="AL4" s="27" t="s">
         <v>332</v>
       </c>
-      <c r="AL4" s="27" t="s">
+      <c r="AM4" s="27" t="s">
         <v>120</v>
       </c>
-      <c r="AM4" s="27" t="s">
+      <c r="AN4" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="AN4" s="27" t="s">
+      <c r="AO4" s="27" t="s">
         <v>122</v>
       </c>
-      <c r="AO4" s="27" t="s">
+      <c r="AP4" s="27" t="s">
         <v>123</v>
       </c>
-      <c r="AP4" s="27" t="s">
+      <c r="AQ4" s="27" t="s">
         <v>124</v>
       </c>
-      <c r="AQ4" s="27" t="s">
+      <c r="AR4" s="27" t="s">
         <v>125</v>
       </c>
-      <c r="AR4" s="27" t="s">
+      <c r="AS4" s="27" t="s">
         <v>126</v>
       </c>
-      <c r="AS4" s="27" t="s">
+      <c r="AT4" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="AT4" s="27" t="s">
+      <c r="AU4" s="27" t="s">
         <v>128</v>
       </c>
-      <c r="AU4" s="27" t="s">
+      <c r="AV4" s="27" t="s">
         <v>129</v>
       </c>
-      <c r="AV4" s="27" t="s">
+      <c r="AW4" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="AW4" s="27" t="s">
+      <c r="AX4" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="AX4" s="27" t="s">
+      <c r="AY4" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="AY4" s="27" t="s">
+      <c r="AZ4" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="AZ4" s="27" t="s">
+      <c r="BA4" s="27" t="s">
         <v>134</v>
       </c>
-      <c r="BA4" s="27" t="s">
+      <c r="BB4" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="BB4" s="27" t="s">
+      <c r="BC4" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="BC4" s="27" t="s">
+      <c r="BD4" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="BD4" s="27" t="s">
+      <c r="BE4" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="BE4" s="27" t="s">
+      <c r="BF4" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="BF4" s="27" t="s">
+      <c r="BG4" s="27" t="s">
         <v>140</v>
       </c>
-      <c r="BG4" s="27" t="s">
+      <c r="BH4" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="BH4" s="27" t="s">
+      <c r="BI4" s="27" t="s">
         <v>142</v>
       </c>
-      <c r="BI4" s="27" t="s">
+      <c r="BJ4" s="27" t="s">
         <v>143</v>
       </c>
-      <c r="BJ4" s="27" t="s">
+      <c r="BK4" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="BK4" s="27" t="s">
+      <c r="BL4" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="BL4" s="27" t="s">
+      <c r="BM4" s="27" t="s">
         <v>146</v>
       </c>
-      <c r="BM4" s="27" t="s">
+      <c r="BN4" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="BN4" s="27" t="s">
+      <c r="BO4" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="BO4" s="27" t="s">
+      <c r="BP4" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="BP4" s="27" t="s">
+      <c r="BQ4" s="27" t="s">
         <v>150</v>
       </c>
-      <c r="BQ4" s="27" t="s">
+      <c r="BR4" s="27" t="s">
         <v>151</v>
       </c>
-      <c r="BR4" s="29" t="s">
+      <c r="BS4" s="29" t="s">
         <v>152</v>
       </c>
-      <c r="BS4" s="27" t="s">
+      <c r="BT4" s="27" t="s">
         <v>153</v>
       </c>
-      <c r="BT4" s="27" t="s">
+      <c r="BU4" s="27" t="s">
         <v>154</v>
       </c>
-      <c r="BU4" s="27" t="s">
+      <c r="BV4" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="BV4" s="27" t="s">
+      <c r="BW4" s="27" t="s">
         <v>156</v>
       </c>
-      <c r="BW4" s="27" t="s">
+      <c r="BX4" s="27" t="s">
         <v>157</v>
       </c>
-      <c r="BX4" s="42" t="s">
+      <c r="BY4" s="42" t="s">
         <v>158</v>
       </c>
-      <c r="BY4" s="27" t="s">
+      <c r="BZ4" s="27" t="s">
         <v>159</v>
       </c>
-      <c r="BZ4" s="27" t="s">
+      <c r="CA4" s="27" t="s">
         <v>160</v>
       </c>
-      <c r="CA4" s="27" t="s">
+      <c r="CB4" s="27" t="s">
         <v>161</v>
       </c>
-      <c r="CB4" s="27" t="s">
+      <c r="CC4" s="27" t="s">
         <v>162</v>
       </c>
-      <c r="CC4" s="27" t="s">
+      <c r="CD4" s="27" t="s">
         <v>163</v>
       </c>
-      <c r="CD4" s="27" t="s">
+      <c r="CE4" s="27" t="s">
         <v>164</v>
       </c>
-      <c r="CE4" s="27" t="s">
+      <c r="CF4" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="CF4" s="27" t="s">
+      <c r="CG4" s="27" t="s">
         <v>166</v>
       </c>
-      <c r="CG4" s="27" t="s">
+      <c r="CH4" s="27" t="s">
         <v>167</v>
       </c>
-      <c r="CH4" s="27" t="s">
+      <c r="CI4" s="27" t="s">
         <v>168</v>
       </c>
-      <c r="CI4" s="27" t="s">
+      <c r="CJ4" s="27" t="s">
         <v>169</v>
       </c>
-      <c r="CJ4" s="27" t="s">
+      <c r="CK4" s="27" t="s">
         <v>170</v>
       </c>
-      <c r="CK4" s="27" t="s">
+      <c r="CL4" s="27" t="s">
         <v>171</v>
       </c>
-      <c r="CL4" s="27" t="s">
+      <c r="CM4" s="27" t="s">
         <v>172</v>
       </c>
-      <c r="CM4" s="27" t="s">
+      <c r="CN4" s="27" t="s">
         <v>173</v>
       </c>
-      <c r="CN4" s="27" t="s">
+      <c r="CO4" s="27" t="s">
         <v>174</v>
       </c>
-      <c r="CO4" s="27" t="s">
+      <c r="CP4" s="27" t="s">
         <v>175</v>
       </c>
-      <c r="CP4" s="27" t="s">
+      <c r="CQ4" s="27" t="s">
         <v>176</v>
       </c>
-      <c r="CQ4" s="27" t="s">
+      <c r="CR4" s="27" t="s">
         <v>177</v>
       </c>
-      <c r="CR4" s="27" t="s">
+      <c r="CS4" s="27" t="s">
         <v>178</v>
       </c>
-      <c r="CS4" s="27" t="s">
+      <c r="CT4" s="27" t="s">
         <v>179</v>
       </c>
-      <c r="CT4" s="27" t="s">
+      <c r="CU4" s="27" t="s">
         <v>180</v>
       </c>
-      <c r="CU4" s="27" t="s">
+      <c r="CV4" s="27" t="s">
         <v>181</v>
       </c>
-      <c r="CV4" s="27" t="s">
+      <c r="CW4" s="27" t="s">
         <v>182</v>
       </c>
-      <c r="CW4" s="27" t="s">
+      <c r="CX4" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="CX4" s="27" t="s">
+      <c r="CY4" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="CY4" s="27" t="s">
+      <c r="CZ4" s="27" t="s">
         <v>185</v>
       </c>
-      <c r="CZ4" s="27" t="s">
+      <c r="DA4" s="27" t="s">
         <v>186</v>
       </c>
-      <c r="DA4" s="27" t="s">
+      <c r="DB4" s="27" t="s">
         <v>187</v>
       </c>
-      <c r="DB4" s="27" t="s">
+      <c r="DC4" s="27" t="s">
         <v>188</v>
       </c>
-      <c r="DC4" s="27" t="s">
+      <c r="DD4" s="27" t="s">
         <v>189</v>
       </c>
-      <c r="DD4" s="27" t="s">
+      <c r="DE4" s="27" t="s">
         <v>190</v>
       </c>
-      <c r="DE4" s="27" t="s">
+      <c r="DF4" s="27" t="s">
         <v>191</v>
       </c>
-      <c r="DF4" s="27" t="s">
+      <c r="DG4" s="27" t="s">
         <v>192</v>
       </c>
-      <c r="DG4" s="27" t="s">
+      <c r="DH4" s="27" t="s">
         <v>193</v>
       </c>
-      <c r="DH4" s="27" t="s">
+      <c r="DI4" s="27" t="s">
         <v>194</v>
       </c>
-      <c r="DI4" s="27" t="s">
+      <c r="DJ4" s="27" t="s">
         <v>195</v>
       </c>
-      <c r="DJ4" s="27" t="s">
+      <c r="DK4" s="27" t="s">
         <v>309</v>
       </c>
-      <c r="DK4" s="28" t="s">
+      <c r="DL4" s="28" t="s">
         <v>310</v>
       </c>
-      <c r="DL4" s="27" t="s">
+      <c r="DM4" s="27" t="s">
         <v>311</v>
       </c>
-      <c r="DM4" s="27" t="s">
+      <c r="DN4" s="27" t="s">
         <v>312</v>
       </c>
-      <c r="DN4" s="27" t="s">
+      <c r="DO4" s="27" t="s">
         <v>313</v>
       </c>
-      <c r="DO4" s="27" t="s">
+      <c r="DP4" s="27" t="s">
         <v>314</v>
       </c>
-      <c r="DP4" s="27" t="s">
+      <c r="DQ4" s="27" t="s">
         <v>315</v>
       </c>
-      <c r="DQ4" s="27" t="s">
+      <c r="DR4" s="27" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="5" spans="1:121" ht="82" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:122" ht="82" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
         <v>196</v>
       </c>
@@ -3289,363 +3308,366 @@
         <v>205</v>
       </c>
       <c r="K5" s="32" t="s">
+        <v>342</v>
+      </c>
+      <c r="L5" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="L5" s="32" t="s">
+      <c r="M5" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="M5" s="32" t="s">
+      <c r="N5" s="32" t="s">
         <v>208</v>
       </c>
-      <c r="N5" s="32" t="s">
+      <c r="O5" s="32" t="s">
         <v>209</v>
       </c>
-      <c r="O5" s="33" t="s">
+      <c r="P5" s="33" t="s">
         <v>210</v>
       </c>
-      <c r="P5" s="33" t="s">
+      <c r="Q5" s="33" t="s">
         <v>211</v>
       </c>
-      <c r="Q5" s="31" t="s">
+      <c r="R5" s="31" t="s">
         <v>212</v>
       </c>
-      <c r="R5" s="33" t="s">
+      <c r="S5" s="33" t="s">
         <v>213</v>
       </c>
-      <c r="S5" s="32" t="s">
+      <c r="T5" s="32" t="s">
         <v>214</v>
       </c>
-      <c r="T5" s="32" t="s">
+      <c r="U5" s="32" t="s">
         <v>215</v>
       </c>
-      <c r="U5" s="33" t="s">
+      <c r="V5" s="33" t="s">
         <v>216</v>
       </c>
-      <c r="V5" s="33" t="s">
+      <c r="W5" s="33" t="s">
         <v>217</v>
       </c>
-      <c r="W5" s="31" t="s">
+      <c r="X5" s="31" t="s">
         <v>218</v>
       </c>
-      <c r="X5" s="33" t="s">
+      <c r="Y5" s="33" t="s">
         <v>219</v>
       </c>
-      <c r="Y5" s="32" t="s">
+      <c r="Z5" s="32" t="s">
         <v>220</v>
       </c>
-      <c r="Z5" s="32" t="s">
+      <c r="AA5" s="32" t="s">
         <v>221</v>
       </c>
-      <c r="AA5" s="32" t="s">
+      <c r="AB5" s="32" t="s">
         <v>222</v>
       </c>
-      <c r="AB5" s="32" t="s">
+      <c r="AC5" s="32" t="s">
         <v>223</v>
       </c>
-      <c r="AC5" s="32" t="s">
+      <c r="AD5" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="AD5" s="32" t="s">
+      <c r="AE5" s="32" t="s">
         <v>225</v>
       </c>
-      <c r="AE5" s="32" t="s">
+      <c r="AF5" s="32" t="s">
         <v>226</v>
       </c>
-      <c r="AF5" s="32" t="s">
+      <c r="AG5" s="32" t="s">
         <v>227</v>
       </c>
-      <c r="AG5" s="32" t="s">
+      <c r="AH5" s="32" t="s">
         <v>228</v>
       </c>
-      <c r="AH5" s="32" t="s">
+      <c r="AI5" s="32" t="s">
         <v>229</v>
       </c>
-      <c r="AI5" s="32" t="s">
+      <c r="AJ5" s="32" t="s">
         <v>230</v>
       </c>
-      <c r="AJ5" s="32" t="s">
+      <c r="AK5" s="32" t="s">
         <v>333</v>
       </c>
-      <c r="AK5" s="32" t="s">
+      <c r="AL5" s="32" t="s">
         <v>334</v>
       </c>
-      <c r="AL5" s="32" t="s">
+      <c r="AM5" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="AM5" s="32" t="s">
+      <c r="AN5" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="AN5" s="32" t="s">
+      <c r="AO5" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="AO5" s="32" t="s">
+      <c r="AP5" s="32" t="s">
         <v>234</v>
       </c>
-      <c r="AP5" s="32" t="s">
+      <c r="AQ5" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="AQ5" s="32" t="s">
+      <c r="AR5" s="32" t="s">
         <v>236</v>
       </c>
-      <c r="AR5" s="32" t="s">
+      <c r="AS5" s="32" t="s">
         <v>237</v>
       </c>
-      <c r="AS5" s="32" t="s">
+      <c r="AT5" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="AT5" s="32" t="s">
+      <c r="AU5" s="32" t="s">
         <v>239</v>
       </c>
-      <c r="AU5" s="32" t="s">
+      <c r="AV5" s="32" t="s">
         <v>240</v>
       </c>
-      <c r="AV5" s="32" t="s">
+      <c r="AW5" s="32" t="s">
         <v>241</v>
       </c>
-      <c r="AW5" s="32" t="s">
+      <c r="AX5" s="32" t="s">
         <v>242</v>
       </c>
-      <c r="AX5" s="32" t="s">
+      <c r="AY5" s="32" t="s">
         <v>243</v>
       </c>
-      <c r="AY5" s="32" t="s">
+      <c r="AZ5" s="32" t="s">
         <v>244</v>
       </c>
-      <c r="AZ5" s="32" t="s">
+      <c r="BA5" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="BA5" s="32" t="s">
+      <c r="BB5" s="32" t="s">
         <v>246</v>
       </c>
-      <c r="BB5" s="32" t="s">
+      <c r="BC5" s="32" t="s">
         <v>247</v>
       </c>
-      <c r="BC5" s="32" t="s">
+      <c r="BD5" s="32" t="s">
         <v>248</v>
       </c>
-      <c r="BD5" s="32" t="s">
+      <c r="BE5" s="32" t="s">
         <v>249</v>
       </c>
-      <c r="BE5" s="32" t="s">
+      <c r="BF5" s="32" t="s">
         <v>250</v>
       </c>
-      <c r="BF5" s="32" t="s">
+      <c r="BG5" s="32" t="s">
         <v>251</v>
       </c>
-      <c r="BG5" s="32" t="s">
+      <c r="BH5" s="32" t="s">
         <v>252</v>
       </c>
-      <c r="BH5" s="32" t="s">
+      <c r="BI5" s="32" t="s">
         <v>253</v>
       </c>
-      <c r="BI5" s="32" t="s">
+      <c r="BJ5" s="32" t="s">
         <v>254</v>
       </c>
-      <c r="BJ5" s="32" t="s">
+      <c r="BK5" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="BK5" s="32" t="s">
+      <c r="BL5" s="32" t="s">
         <v>256</v>
       </c>
-      <c r="BL5" s="32" t="s">
+      <c r="BM5" s="32" t="s">
         <v>257</v>
       </c>
-      <c r="BM5" s="32" t="s">
+      <c r="BN5" s="32" t="s">
         <v>258</v>
       </c>
-      <c r="BN5" s="31" t="s">
+      <c r="BO5" s="31" t="s">
         <v>259</v>
       </c>
-      <c r="BO5" s="31" t="s">
+      <c r="BP5" s="31" t="s">
         <v>260</v>
       </c>
-      <c r="BP5" s="32" t="s">
+      <c r="BQ5" s="32" t="s">
         <v>261</v>
       </c>
-      <c r="BQ5" s="32" t="s">
+      <c r="BR5" s="32" t="s">
         <v>262</v>
       </c>
-      <c r="BR5" s="32" t="s">
+      <c r="BS5" s="32" t="s">
         <v>263</v>
       </c>
-      <c r="BS5" s="32" t="s">
+      <c r="BT5" s="32" t="s">
         <v>264</v>
       </c>
-      <c r="BT5" s="31" t="s">
+      <c r="BU5" s="31" t="s">
         <v>265</v>
       </c>
-      <c r="BU5" s="31" t="s">
+      <c r="BV5" s="31" t="s">
         <v>266</v>
       </c>
-      <c r="BV5" s="32" t="s">
+      <c r="BW5" s="32" t="s">
         <v>267</v>
       </c>
-      <c r="BW5" s="32" t="s">
+      <c r="BX5" s="32" t="s">
         <v>268</v>
       </c>
-      <c r="BX5" s="32" t="s">
+      <c r="BY5" s="32" t="s">
         <v>269</v>
       </c>
-      <c r="BY5" s="32" t="s">
+      <c r="BZ5" s="32" t="s">
         <v>270</v>
       </c>
-      <c r="BZ5" s="32" t="s">
+      <c r="CA5" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="CA5" s="32" t="s">
+      <c r="CB5" s="32" t="s">
         <v>272</v>
       </c>
-      <c r="CB5" s="32" t="s">
+      <c r="CC5" s="32" t="s">
         <v>273</v>
       </c>
-      <c r="CC5" s="32" t="s">
+      <c r="CD5" s="32" t="s">
         <v>274</v>
       </c>
-      <c r="CD5" s="32" t="s">
+      <c r="CE5" s="32" t="s">
         <v>275</v>
       </c>
-      <c r="CE5" s="32" t="s">
+      <c r="CF5" s="32" t="s">
         <v>276</v>
       </c>
-      <c r="CF5" s="32" t="s">
+      <c r="CG5" s="32" t="s">
         <v>277</v>
       </c>
-      <c r="CG5" s="32" t="s">
+      <c r="CH5" s="32" t="s">
         <v>278</v>
       </c>
-      <c r="CH5" s="32" t="s">
+      <c r="CI5" s="32" t="s">
         <v>279</v>
       </c>
-      <c r="CI5" s="32" t="s">
+      <c r="CJ5" s="32" t="s">
         <v>280</v>
       </c>
-      <c r="CJ5" s="32" t="s">
+      <c r="CK5" s="32" t="s">
         <v>281</v>
       </c>
-      <c r="CK5" s="32" t="s">
+      <c r="CL5" s="32" t="s">
         <v>282</v>
       </c>
-      <c r="CL5" s="32" t="s">
+      <c r="CM5" s="32" t="s">
         <v>283</v>
       </c>
-      <c r="CM5" s="32" t="s">
+      <c r="CN5" s="32" t="s">
         <v>284</v>
       </c>
-      <c r="CN5" s="32" t="s">
+      <c r="CO5" s="32" t="s">
         <v>285</v>
       </c>
-      <c r="CO5" s="32" t="s">
+      <c r="CP5" s="32" t="s">
         <v>286</v>
       </c>
-      <c r="CP5" s="32" t="s">
+      <c r="CQ5" s="32" t="s">
         <v>287</v>
       </c>
-      <c r="CQ5" s="32" t="s">
+      <c r="CR5" s="32" t="s">
         <v>288</v>
       </c>
-      <c r="CR5" s="32" t="s">
+      <c r="CS5" s="32" t="s">
         <v>289</v>
       </c>
-      <c r="CS5" s="32" t="s">
+      <c r="CT5" s="32" t="s">
         <v>290</v>
       </c>
-      <c r="CT5" s="32" t="s">
+      <c r="CU5" s="32" t="s">
         <v>291</v>
       </c>
-      <c r="CU5" s="32" t="s">
+      <c r="CV5" s="32" t="s">
         <v>292</v>
       </c>
-      <c r="CV5" s="32" t="s">
+      <c r="CW5" s="32" t="s">
         <v>293</v>
       </c>
-      <c r="CW5" s="32" t="s">
+      <c r="CX5" s="32" t="s">
         <v>294</v>
       </c>
-      <c r="CX5" s="32" t="s">
+      <c r="CY5" s="32" t="s">
         <v>295</v>
       </c>
-      <c r="CY5" s="32" t="s">
+      <c r="CZ5" s="32" t="s">
         <v>296</v>
       </c>
-      <c r="CZ5" s="32" t="s">
+      <c r="DA5" s="32" t="s">
         <v>297</v>
       </c>
-      <c r="DA5" s="32" t="s">
+      <c r="DB5" s="32" t="s">
         <v>298</v>
       </c>
-      <c r="DB5" s="32" t="s">
+      <c r="DC5" s="32" t="s">
         <v>299</v>
       </c>
-      <c r="DC5" s="32" t="s">
+      <c r="DD5" s="32" t="s">
         <v>300</v>
       </c>
-      <c r="DD5" s="32" t="s">
+      <c r="DE5" s="32" t="s">
         <v>301</v>
       </c>
-      <c r="DE5" s="32" t="s">
+      <c r="DF5" s="32" t="s">
         <v>302</v>
       </c>
-      <c r="DF5" s="32" t="s">
+      <c r="DG5" s="32" t="s">
         <v>303</v>
       </c>
-      <c r="DG5" s="32" t="s">
+      <c r="DH5" s="32" t="s">
         <v>304</v>
       </c>
-      <c r="DH5" s="32" t="s">
+      <c r="DI5" s="32" t="s">
         <v>305</v>
       </c>
-      <c r="DI5" s="32" t="s">
+      <c r="DJ5" s="32" t="s">
         <v>306</v>
       </c>
-      <c r="DJ5" s="32" t="s">
+      <c r="DK5" s="32" t="s">
         <v>319</v>
       </c>
-      <c r="DK5" s="33" t="s">
+      <c r="DL5" s="33" t="s">
         <v>320</v>
       </c>
-      <c r="DL5" s="32" t="s">
+      <c r="DM5" s="32" t="s">
         <v>321</v>
       </c>
-      <c r="DM5" s="32" t="s">
+      <c r="DN5" s="32" t="s">
         <v>317</v>
       </c>
-      <c r="DN5" s="32" t="s">
+      <c r="DO5" s="32" t="s">
         <v>318</v>
       </c>
-      <c r="DO5" s="32" t="s">
+      <c r="DP5" s="32" t="s">
         <v>322</v>
       </c>
-      <c r="DP5" s="32" t="s">
+      <c r="DQ5" s="32" t="s">
         <v>323</v>
       </c>
-      <c r="DQ5" s="32" t="s">
+      <c r="DR5" s="32" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="6" spans="1:121" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:122" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1 L5" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M1 M5" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"cartographic,mixed_materials,moving_image,notated_music,software_multimedia,sound_recording,sound_recording_musical,sound_recording_nonmusical,still_image,text"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 L3:L4" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4 M3:M4" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1 K5" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1 L5" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"collection,image,work"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" operator="equal" allowBlank="1" showErrorMessage="1" sqref="AM1 AQ1" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" operator="equal" allowBlank="1" showErrorMessage="1" sqref="AN1 AR1" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"bibliography,accessrestrict,acqinfo,altformavail,bioghist,custodhist,dimensions,edition,extent,inscription,legalstatus,note,originalsloc,physdesc,prefercite,processinfo,relatedmaterial,summary,userestrict"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation operator="equal" allowBlank="1" showErrorMessage="1" sqref="AB1:AB5 AM2:AM5 AN1:AN5 AO2:AO5 AP1:AP5 AQ2:AQ5 AR1:AR5 AS2:AS5 AT1:AT5" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation operator="equal" allowBlank="1" showErrorMessage="1" sqref="AC1:AC5 AN2:AN5 AO1:AO5 AP2:AP5 AQ1:AQ5 AR2:AR5 AS1:AS5 AT2:AT5 AU1:AU5" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" operator="equal" allowBlank="1" showErrorMessage="1" sqref="AO1 AS1" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" operator="equal" allowBlank="1" showErrorMessage="1" sqref="AP1 AT1" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"TRUE,FALSE"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>